<commit_message>
cambios excel y yml
</commit_message>
<xml_diff>
--- a/Tablero_control_General_Instalación_180926.xlsx
+++ b/Tablero_control_General_Instalación_180926.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.garcia\Desktop\github\linea_tiempo_fase_instalacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1A3FC55-55AC-4542-B22F-DD9664588F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1CC137-D48C-47C6-823F-E6F831FA9E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Reporte semanal" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="680">
   <si>
     <t>CÓDIGO DIPOLA MUN</t>
   </si>
@@ -2465,13 +2465,6 @@
   <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\08770_Suan (Atlántico)\04_Instalación\05_Entrega
 NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
-    <t>Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
-NOMBRE ARCHIVO: 01_BTC_Ambalema_090726
-                                 02_BTC_Ambalema_100726
-                                 03_BTC_Ambalema_110726
-                                 04_BTC_Ambalema_120726</t>
   </si>
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\04_Capacitación
@@ -9752,7 +9745,7 @@
         <v>302</v>
       </c>
       <c r="Z26" s="19" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="AA26" s="19" t="s">
         <v>298</v>
@@ -10616,7 +10609,7 @@
         <v>504</v>
       </c>
       <c r="AB35" s="19" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="AC35" s="19" t="s">
         <v>506</v>
@@ -10712,7 +10705,7 @@
         <v>511</v>
       </c>
       <c r="AB36" s="19" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="AC36" s="19" t="s">
         <v>529</v>
@@ -10808,7 +10801,7 @@
         <v>514</v>
       </c>
       <c r="AB37" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="AC37" s="19" t="s">
         <v>590</v>
@@ -10904,7 +10897,7 @@
         <v>523</v>
       </c>
       <c r="AB38" s="19" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="AC38" s="19" t="s">
         <v>533</v>
@@ -11000,7 +10993,7 @@
         <v>538</v>
       </c>
       <c r="AB39" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="AC39" s="19" t="s">
         <v>563</v>
@@ -11087,7 +11080,7 @@
         <v>174</v>
       </c>
       <c r="Y40" s="19" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="Z40" s="19" t="s">
         <v>557</v>
@@ -11096,7 +11089,7 @@
         <v>539</v>
       </c>
       <c r="AB40" s="19" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="AC40" s="19" t="s">
         <v>565</v>
@@ -11192,7 +11185,7 @@
         <v>542</v>
       </c>
       <c r="AB41" s="19" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="AC41" s="19" t="s">
         <v>564</v>
@@ -11270,41 +11263,41 @@
         <v>608</v>
       </c>
       <c r="V42" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="W42" s="19" t="s">
         <v>621</v>
-      </c>
-      <c r="W42" s="19" t="s">
-        <v>622</v>
       </c>
       <c r="X42" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Y42" s="19" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="Z42" s="19" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="AA42" s="19" t="s">
         <v>615</v>
       </c>
       <c r="AB42" s="19" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="AC42" s="19" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="AD42" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AE42" s="19" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="AF42" s="78"/>
       <c r="AG42" s="63" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="43" spans="2:33" ht="72">
+    <row r="43" spans="2:33" ht="48">
       <c r="B43" s="23">
         <v>73030</v>
       </c>
@@ -11377,23 +11370,23 @@
       <c r="Y43" s="64" t="s">
         <v>174</v>
       </c>
-      <c r="Z43" s="19" t="s">
-        <v>617</v>
+      <c r="Z43" s="64" t="s">
+        <v>174</v>
       </c>
       <c r="AA43" s="19" t="s">
         <v>613</v>
       </c>
       <c r="AB43" s="19" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AC43" s="19" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="AD43" s="19" t="s">
+        <v>617</v>
+      </c>
+      <c r="AE43" s="19" t="s">
         <v>618</v>
-      </c>
-      <c r="AE43" s="19" t="s">
-        <v>619</v>
       </c>
       <c r="AF43" s="78"/>
       <c r="AG43" s="63" t="s">
@@ -11447,25 +11440,25 @@
         <v>46240</v>
       </c>
       <c r="Q44" s="80" t="s">
+        <v>633</v>
+      </c>
+      <c r="R44" s="80" t="s">
         <v>634</v>
       </c>
-      <c r="R44" s="80" t="s">
+      <c r="S44" s="74" t="s">
+        <v>632</v>
+      </c>
+      <c r="T44" s="81" t="s">
         <v>635</v>
       </c>
-      <c r="S44" s="74" t="s">
-        <v>633</v>
-      </c>
-      <c r="T44" s="81" t="s">
+      <c r="U44" s="80" t="s">
         <v>636</v>
       </c>
-      <c r="U44" s="80" t="s">
-        <v>637</v>
-      </c>
       <c r="V44" s="81" t="s">
+        <v>653</v>
+      </c>
+      <c r="W44" s="81" t="s">
         <v>654</v>
-      </c>
-      <c r="W44" s="81" t="s">
-        <v>655</v>
       </c>
       <c r="X44" s="79" t="s">
         <v>174</v>
@@ -11474,26 +11467,26 @@
         <v>174</v>
       </c>
       <c r="Z44" s="19" t="s">
+        <v>647</v>
+      </c>
+      <c r="AA44" s="19" t="s">
+        <v>642</v>
+      </c>
+      <c r="AB44" s="63" t="s">
         <v>648</v>
       </c>
-      <c r="AA44" s="19" t="s">
-        <v>643</v>
-      </c>
-      <c r="AB44" s="63" t="s">
+      <c r="AC44" s="19" t="s">
+        <v>656</v>
+      </c>
+      <c r="AD44" s="19" t="s">
         <v>649</v>
       </c>
-      <c r="AC44" s="19" t="s">
-        <v>657</v>
-      </c>
-      <c r="AD44" s="19" t="s">
+      <c r="AE44" s="63" t="s">
         <v>650</v>
-      </c>
-      <c r="AE44" s="63" t="s">
-        <v>651</v>
       </c>
       <c r="AF44" s="78"/>
       <c r="AG44" s="63" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="45" spans="2:33" ht="60">
@@ -11543,25 +11536,25 @@
         <v>46240</v>
       </c>
       <c r="Q45" s="32" t="s">
+        <v>638</v>
+      </c>
+      <c r="R45" s="32" t="s">
         <v>639</v>
       </c>
-      <c r="R45" s="32" t="s">
-        <v>640</v>
-      </c>
       <c r="S45" s="74" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="T45" s="19" t="s">
+        <v>651</v>
+      </c>
+      <c r="U45" s="32" t="s">
+        <v>637</v>
+      </c>
+      <c r="V45" s="19" t="s">
         <v>652</v>
       </c>
-      <c r="U45" s="32" t="s">
-        <v>638</v>
-      </c>
-      <c r="V45" s="19" t="s">
-        <v>653</v>
-      </c>
       <c r="W45" s="19" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="X45" s="64" t="s">
         <v>174</v>
@@ -11570,26 +11563,26 @@
         <v>174</v>
       </c>
       <c r="Z45" s="19" t="s">
+        <v>674</v>
+      </c>
+      <c r="AA45" s="19" t="s">
+        <v>644</v>
+      </c>
+      <c r="AB45" s="63" t="s">
+        <v>645</v>
+      </c>
+      <c r="AC45" s="19" t="s">
         <v>675</v>
       </c>
-      <c r="AA45" s="19" t="s">
-        <v>645</v>
-      </c>
-      <c r="AB45" s="63" t="s">
-        <v>646</v>
-      </c>
-      <c r="AC45" s="19" t="s">
+      <c r="AD45" s="19" t="s">
         <v>676</v>
       </c>
-      <c r="AD45" s="19" t="s">
-        <v>677</v>
-      </c>
       <c r="AE45" s="63" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="AF45" s="78"/>
       <c r="AG45" s="63" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="46" spans="2:33" ht="72">
@@ -11639,25 +11632,25 @@
         <v>46262</v>
       </c>
       <c r="Q46" s="32" t="s">
+        <v>678</v>
+      </c>
+      <c r="R46" s="32" t="s">
         <v>679</v>
       </c>
-      <c r="R46" s="32" t="s">
-        <v>680</v>
-      </c>
       <c r="S46" s="32" t="s">
+        <v>664</v>
+      </c>
+      <c r="T46" s="19" t="s">
         <v>665</v>
       </c>
-      <c r="T46" s="19" t="s">
+      <c r="U46" s="74" t="s">
         <v>666</v>
       </c>
-      <c r="U46" s="74" t="s">
+      <c r="V46" s="63" t="s">
         <v>667</v>
       </c>
-      <c r="V46" s="63" t="s">
+      <c r="W46" s="63" t="s">
         <v>668</v>
-      </c>
-      <c r="W46" s="63" t="s">
-        <v>669</v>
       </c>
       <c r="X46" s="64" t="s">
         <v>174</v>
@@ -11666,26 +11659,26 @@
         <v>174</v>
       </c>
       <c r="Z46" s="63" t="s">
+        <v>669</v>
+      </c>
+      <c r="AA46" s="63" t="s">
+        <v>662</v>
+      </c>
+      <c r="AB46" s="63" t="s">
+        <v>677</v>
+      </c>
+      <c r="AC46" s="63" t="s">
         <v>670</v>
       </c>
-      <c r="AA46" s="63" t="s">
-        <v>663</v>
-      </c>
-      <c r="AB46" s="63" t="s">
-        <v>678</v>
-      </c>
-      <c r="AC46" s="63" t="s">
+      <c r="AD46" s="63" t="s">
         <v>671</v>
       </c>
-      <c r="AD46" s="63" t="s">
+      <c r="AE46" s="63" t="s">
         <v>672</v>
-      </c>
-      <c r="AE46" s="63" t="s">
-        <v>673</v>
       </c>
       <c r="AF46" s="78"/>
       <c r="AG46" s="63" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="47" spans="2:33" ht="42.75" customHeight="1">
@@ -13978,6 +13971,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creador>
+    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010000E8DC80C026CA4DA909D73C325EE4F6" ma:contentTypeVersion="22" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="540ba7b4ebff7c81ec83231b347cbaa0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xmlns:ns3="a9ff745a-43b9-4806-bec3-e08ef3e383fc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45c75a4f992fb922f736f24948a438b4" ns2:_="" ns3:_="">
     <xsd:import namespace="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
@@ -14244,35 +14265,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
+    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creador>
-    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85AD5D61-E9C3-4156-A82C-31BB302CC72C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14289,29 +14307,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
-    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
index nuevo, excel update, yml cambios a index no al otro html
</commit_message>
<xml_diff>
--- a/Tablero_control_General_Instalación_180926.xlsx
+++ b/Tablero_control_General_Instalación_180926.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.garcia\Desktop\github\linea_tiempo_fase_instalacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BE1853-831E-4C74-9496-5D6B4BA15725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4856B5BD-D46A-4C48-9A96-46B3E8E0AA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="681">
   <si>
     <t>CÓDIGO DIPOLA MUN</t>
   </si>
@@ -2453,6 +2453,9 @@
                                  ACTA_VECINDAD_INICIO_210426_Predio1Repelon</t>
   </si>
   <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\03_SeguimientoCampo\03_CertificacionesCalidadMateriales\01_Anclajes\01_Contratista</t>
+  </si>
+  <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\05_Entrega
 NOMBRE ARCHIVO: </t>
   </si>
@@ -2462,6 +2465,13 @@
   <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\08770_Suan (Atlántico)\04_Instalación\05_Entrega
 NOMBRE ARCHIVO: </t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
+NOMBRE ARCHIVO: 01_BTC_Ambalema_090726
+                                 02_BTC_Ambalema_100726
+                                 03_BTC_Ambalema_110726
+                                 04_BTC_Ambalema_120726</t>
   </si>
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\04_Capacitación
@@ -8126,7 +8136,7 @@
     <col min="29" max="29" width="60.5703125" style="11" customWidth="1"/>
     <col min="30" max="30" width="64.140625" style="11" customWidth="1"/>
     <col min="31" max="31" width="57.42578125" style="11" customWidth="1"/>
-    <col min="32" max="32" width="29.28515625" style="11" customWidth="1"/>
+    <col min="32" max="32" width="0" style="11" hidden="1" customWidth="1"/>
     <col min="33" max="33" width="74.140625" style="11" customWidth="1"/>
     <col min="34" max="16384" width="11.42578125" style="11"/>
   </cols>
@@ -9742,7 +9752,7 @@
         <v>302</v>
       </c>
       <c r="Z26" s="19" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="AA26" s="19" t="s">
         <v>298</v>
@@ -10606,7 +10616,7 @@
         <v>504</v>
       </c>
       <c r="AB35" s="19" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="AC35" s="19" t="s">
         <v>506</v>
@@ -10702,7 +10712,7 @@
         <v>511</v>
       </c>
       <c r="AB36" s="19" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="AC36" s="19" t="s">
         <v>529</v>
@@ -10798,7 +10808,7 @@
         <v>514</v>
       </c>
       <c r="AB37" s="19" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="AC37" s="19" t="s">
         <v>590</v>
@@ -10894,7 +10904,7 @@
         <v>523</v>
       </c>
       <c r="AB38" s="19" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="AC38" s="19" t="s">
         <v>533</v>
@@ -10990,7 +11000,7 @@
         <v>538</v>
       </c>
       <c r="AB39" s="19" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="AC39" s="19" t="s">
         <v>563</v>
@@ -11077,7 +11087,7 @@
         <v>174</v>
       </c>
       <c r="Y40" s="19" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="Z40" s="19" t="s">
         <v>557</v>
@@ -11086,7 +11096,7 @@
         <v>539</v>
       </c>
       <c r="AB40" s="19" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="AC40" s="19" t="s">
         <v>565</v>
@@ -11182,7 +11192,7 @@
         <v>542</v>
       </c>
       <c r="AB41" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="AC41" s="19" t="s">
         <v>564</v>
@@ -11260,41 +11270,41 @@
         <v>608</v>
       </c>
       <c r="V42" s="19" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="W42" s="19" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="X42" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Y42" s="19" t="s">
+        <v>627</v>
+      </c>
+      <c r="Z42" s="19" t="s">
+        <v>626</v>
+      </c>
+      <c r="AA42" s="19" t="s">
+        <v>615</v>
+      </c>
+      <c r="AB42" s="19" t="s">
+        <v>659</v>
+      </c>
+      <c r="AC42" s="19" t="s">
         <v>625</v>
       </c>
-      <c r="Z42" s="19" t="s">
-        <v>624</v>
-      </c>
-      <c r="AA42" s="19" t="s">
-        <v>614</v>
-      </c>
-      <c r="AB42" s="19" t="s">
-        <v>657</v>
-      </c>
-      <c r="AC42" s="19" t="s">
+      <c r="AD42" s="19" t="s">
         <v>623</v>
       </c>
-      <c r="AD42" s="19" t="s">
-        <v>621</v>
-      </c>
       <c r="AE42" s="19" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="AF42" s="78"/>
       <c r="AG42" s="63" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
     </row>
-    <row r="43" spans="2:33" ht="48">
+    <row r="43" spans="2:33" ht="72">
       <c r="B43" s="23">
         <v>73030</v>
       </c>
@@ -11367,27 +11377,27 @@
       <c r="Y43" s="64" t="s">
         <v>174</v>
       </c>
-      <c r="Z43" s="64" t="s">
-        <v>174</v>
-      </c>
-      <c r="AA43" s="64" t="s">
-        <v>174</v>
+      <c r="Z43" s="19" t="s">
+        <v>617</v>
+      </c>
+      <c r="AA43" s="19" t="s">
+        <v>613</v>
       </c>
       <c r="AB43" s="19" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="AC43" s="19" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="AD43" s="19" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="AE43" s="19" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="AF43" s="78"/>
       <c r="AG43" s="63" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="44" spans="2:33" ht="72">
@@ -11437,25 +11447,25 @@
         <v>46240</v>
       </c>
       <c r="Q44" s="80" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="R44" s="80" t="s">
+        <v>635</v>
+      </c>
+      <c r="S44" s="74" t="s">
         <v>633</v>
       </c>
-      <c r="S44" s="74" t="s">
-        <v>631</v>
-      </c>
       <c r="T44" s="81" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="U44" s="80" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="V44" s="81" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="W44" s="81" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="X44" s="79" t="s">
         <v>174</v>
@@ -11464,26 +11474,26 @@
         <v>174</v>
       </c>
       <c r="Z44" s="19" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="AA44" s="19" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="AB44" s="63" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="AC44" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="AD44" s="19" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="AE44" s="63" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="AF44" s="78"/>
       <c r="AG44" s="63" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="45" spans="2:33" ht="60">
@@ -11533,25 +11543,25 @@
         <v>46240</v>
       </c>
       <c r="Q45" s="32" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="R45" s="32" t="s">
+        <v>640</v>
+      </c>
+      <c r="S45" s="74" t="s">
+        <v>662</v>
+      </c>
+      <c r="T45" s="19" t="s">
+        <v>652</v>
+      </c>
+      <c r="U45" s="32" t="s">
         <v>638</v>
       </c>
-      <c r="S45" s="74" t="s">
-        <v>660</v>
-      </c>
-      <c r="T45" s="19" t="s">
-        <v>650</v>
-      </c>
-      <c r="U45" s="32" t="s">
-        <v>636</v>
-      </c>
       <c r="V45" s="19" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="W45" s="19" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="X45" s="64" t="s">
         <v>174</v>
@@ -11560,26 +11570,26 @@
         <v>174</v>
       </c>
       <c r="Z45" s="19" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="AA45" s="19" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="AB45" s="63" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="AC45" s="19" t="s">
+        <v>676</v>
+      </c>
+      <c r="AD45" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="AE45" s="63" t="s">
         <v>674</v>
-      </c>
-      <c r="AD45" s="19" t="s">
-        <v>675</v>
-      </c>
-      <c r="AE45" s="63" t="s">
-        <v>672</v>
       </c>
       <c r="AF45" s="78"/>
       <c r="AG45" s="63" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="46" spans="2:33" ht="72">
@@ -11629,25 +11639,25 @@
         <v>46262</v>
       </c>
       <c r="Q46" s="32" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="R46" s="32" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="S46" s="32" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="T46" s="19" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="U46" s="74" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="V46" s="63" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="W46" s="63" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="X46" s="64" t="s">
         <v>174</v>
@@ -11656,26 +11666,26 @@
         <v>174</v>
       </c>
       <c r="Z46" s="63" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="AA46" s="63" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="AB46" s="63" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="AC46" s="63" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="AD46" s="63" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="AE46" s="63" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="AF46" s="78"/>
       <c r="AG46" s="63" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="47" spans="2:33" ht="42.75" customHeight="1">
@@ -13968,6 +13978,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creador>
+    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010000E8DC80C026CA4DA909D73C325EE4F6" ma:contentTypeVersion="22" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="540ba7b4ebff7c81ec83231b347cbaa0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xmlns:ns3="a9ff745a-43b9-4806-bec3-e08ef3e383fc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45c75a4f992fb922f736f24948a438b4" ns2:_="" ns3:_="">
     <xsd:import namespace="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
@@ -14234,7 +14263,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -14243,26 +14272,24 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creador>
-    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
+    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85AD5D61-E9C3-4156-A82C-31BB302CC72C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14281,27 +14308,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
-    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add html nuevo py con enlaces rutas, clic en pendientes
</commit_message>
<xml_diff>
--- a/Tablero_control_General_Instalación_180926.xlsx
+++ b/Tablero_control_General_Instalación_180926.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria.pardo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.garcia\Desktop\github\linea_tiempo_fase_instalacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADBB6A6-634A-4993-8DED-AEAD785F7E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AD08CC-F616-4476-9696-5BA3ADE42391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Reporte semanal" sheetId="2" r:id="rId1"/>
@@ -632,15 +632,6 @@
                                    05_BTC_MB_010925</t>
   </si>
   <si>
-    <t>Documentos\Documentos Tecnicos\Documentos por sitio\68575_Puerto Wilches - La Boya (Santander)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
-NOMBRE ARCHIVO: 01_BTC_PtoWilches_140725
-                                   02_BTC_PtoWilches_150725
-                                   03_BTC_PtoWilches_160725
-                                   04_BTC_PtoWilches_170725
-                                   05_BTC_PtoWilches_180725
-                                   06_BTC_PtoWilches_190725</t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\47555_Plato (Magdalena)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
 NOMBRE ARCHIVO: 01_BTC_PLATO_230925
                                    02_BTC_PLATO_240925
@@ -3080,6 +3071,15 @@
 NOMBRE ARCHIVO: 
 </t>
   </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\68575_Puerto Wilches - La Boya (Santander)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
+NOMBRE ARCHIVO: 01_BTC_PtoWilches_140725
+02_BTC_PtoWilches_150725
+03_BTC_PtoWilches_160725
+                                   04_BTC_PtoWilches_170725
+                                   05_BTC_PtoWilches_180725
+                                   06_BTC_PtoWilches_190725</t>
+  </si>
 </sst>
 </file>
 
@@ -3088,7 +3088,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3188,6 +3188,14 @@
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="CaIibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="18">
@@ -3392,10 +3400,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3635,8 +3644,12 @@
     <xf numFmtId="14" fontId="7" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="37">
@@ -5070,8 +5083,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="466421" y="0"/>
-          <a:ext cx="11296954" cy="1260929"/>
+          <a:off x="455838" y="0"/>
+          <a:ext cx="10775725" cy="1292679"/>
           <a:chOff x="748618" y="-95891"/>
           <a:chExt cx="1536898" cy="1592199"/>
         </a:xfrm>
@@ -5492,8 +5505,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="163287" y="302948"/>
-          <a:ext cx="66395296" cy="1116101"/>
+          <a:off x="163287" y="313531"/>
+          <a:ext cx="63339888" cy="1179601"/>
           <a:chOff x="597738" y="179718"/>
           <a:chExt cx="17343644" cy="1316590"/>
         </a:xfrm>
@@ -6267,27 +6280,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{875B28C0-B948-4D48-BD54-8EF7F295132D}">
   <dimension ref="B8:R51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.90625" customWidth="1"/>
-    <col min="2" max="2" width="7.08984375" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" customWidth="1"/>
-    <col min="4" max="4" width="7.453125" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" customWidth="1"/>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="11" width="10.08984375" customWidth="1"/>
-    <col min="12" max="12" width="10.90625" customWidth="1"/>
-    <col min="13" max="15" width="10.08984375" customWidth="1"/>
+    <col min="10" max="11" width="10.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="13" max="15" width="10.140625" customWidth="1"/>
     <col min="16" max="17" width="11" customWidth="1"/>
-    <col min="18" max="18" width="10.08984375" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="9.54296875" customWidth="1"/>
+    <col min="18" max="18" width="10.140625" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="2:18" ht="16.5" customHeight="1"/>
-    <row r="9" spans="2:18" ht="31.5">
+    <row r="9" spans="2:18" ht="45">
       <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
@@ -6304,7 +6317,7 @@
         <v>3</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>148</v>
@@ -6357,7 +6370,7 @@
         <v>4</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H10" s="57">
         <v>45852</v>
@@ -6412,7 +6425,7 @@
         <v>19</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H11" s="57">
         <v>45895</v>
@@ -6467,7 +6480,7 @@
         <v>17</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H12" s="57">
         <v>45894</v>
@@ -6522,7 +6535,7 @@
         <v>17</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H13" s="57">
         <v>45922</v>
@@ -6577,7 +6590,7 @@
         <v>17</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H14" s="57">
         <v>45923</v>
@@ -6632,7 +6645,7 @@
         <v>17</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H15" s="57">
         <v>45979</v>
@@ -6687,7 +6700,7 @@
         <v>45</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H16" s="57">
         <v>45985</v>
@@ -6742,7 +6755,7 @@
         <v>50</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H17" s="57">
         <v>45987</v>
@@ -6797,7 +6810,7 @@
         <v>45</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H18" s="57">
         <v>46001</v>
@@ -6852,7 +6865,7 @@
         <v>36</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H19" s="57">
         <v>46001</v>
@@ -6907,7 +6920,7 @@
         <v>36</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H20" s="57">
         <v>46002</v>
@@ -6962,7 +6975,7 @@
         <v>19</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H21" s="57">
         <v>46010</v>
@@ -7017,7 +7030,7 @@
         <v>19</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H22" s="57">
         <v>46038</v>
@@ -7072,7 +7085,7 @@
         <v>48</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H23" s="57">
         <v>46041</v>
@@ -7127,7 +7140,7 @@
         <v>48</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H24" s="57">
         <v>46043</v>
@@ -7182,7 +7195,7 @@
         <v>53</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H25" s="3">
         <v>46024</v>
@@ -7234,7 +7247,7 @@
         <v>68</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H26" s="3">
         <v>46024</v>
@@ -7269,7 +7282,7 @@
       </c>
       <c r="R26" s="8"/>
     </row>
-    <row r="27" spans="2:18" ht="26.4" customHeight="1">
+    <row r="27" spans="2:18" ht="26.45" customHeight="1">
       <c r="B27" s="2">
         <v>18</v>
       </c>
@@ -7277,16 +7290,16 @@
         <v>68575</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H27" s="3">
         <v>46070</v>
@@ -7321,7 +7334,7 @@
       </c>
       <c r="R27" s="8"/>
     </row>
-    <row r="28" spans="2:18" ht="26.4" customHeight="1">
+    <row r="28" spans="2:18" ht="26.45" customHeight="1">
       <c r="B28" s="2">
         <v>19</v>
       </c>
@@ -7338,7 +7351,7 @@
         <v>19</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H28" s="3">
         <v>46121</v>
@@ -7372,7 +7385,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="2:18" ht="26.4" customHeight="1">
+    <row r="29" spans="2:18" ht="26.45" customHeight="1">
       <c r="B29" s="2">
         <v>20</v>
       </c>
@@ -7389,7 +7402,7 @@
         <v>19</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H29" s="3">
         <v>46121</v>
@@ -7440,7 +7453,7 @@
         <v>21</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H30" s="3">
         <v>46126</v>
@@ -7474,7 +7487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="2:18" ht="23.4" customHeight="1">
+    <row r="31" spans="2:18" ht="23.45" customHeight="1">
       <c r="B31" s="2">
         <v>22</v>
       </c>
@@ -7491,7 +7504,7 @@
         <v>19</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H31" s="3">
         <v>46129</v>
@@ -7525,7 +7538,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="2:18" ht="26.4" customHeight="1">
+    <row r="32" spans="2:18" ht="26.45" customHeight="1">
       <c r="B32" s="2">
         <v>23</v>
       </c>
@@ -7542,7 +7555,7 @@
         <v>21</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H32" s="3">
         <v>46132</v>
@@ -7576,7 +7589,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="2:17" ht="26.15" customHeight="1">
+    <row r="33" spans="2:17" ht="26.1" customHeight="1">
       <c r="B33" s="2">
         <v>24</v>
       </c>
@@ -7593,7 +7606,7 @@
         <v>36</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H33" s="3">
         <v>46155</v>
@@ -7627,7 +7640,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="2:17" ht="26.15" customHeight="1">
+    <row r="34" spans="2:17" ht="26.1" customHeight="1">
       <c r="B34" s="2">
         <v>25</v>
       </c>
@@ -7644,7 +7657,7 @@
         <v>19</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H34" s="3">
         <v>46175</v>
@@ -7678,7 +7691,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="2:17" ht="26.15" customHeight="1">
+    <row r="35" spans="2:17" ht="26.1" customHeight="1">
       <c r="B35" s="2">
         <v>26</v>
       </c>
@@ -7695,7 +7708,7 @@
         <v>19</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H35" s="3">
         <v>46177</v>
@@ -7729,7 +7742,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="2:17" ht="26.15" customHeight="1">
+    <row r="36" spans="2:17" ht="26.1" customHeight="1">
       <c r="B36" s="2">
         <v>27</v>
       </c>
@@ -7746,7 +7759,7 @@
         <v>19</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H36" s="3">
         <v>46185</v>
@@ -7780,7 +7793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="2:17" ht="26.15" customHeight="1">
+    <row r="37" spans="2:17" ht="26.1" customHeight="1">
       <c r="B37" s="2">
         <v>28</v>
       </c>
@@ -7797,7 +7810,7 @@
         <v>19</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H37" s="3">
         <v>46184</v>
@@ -7831,7 +7844,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="2:17" ht="26.15" customHeight="1">
+    <row r="38" spans="2:17" ht="26.1" customHeight="1">
       <c r="B38" s="2">
         <v>29</v>
       </c>
@@ -7848,7 +7861,7 @@
         <v>19</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H38" s="3">
         <v>46197</v>
@@ -7882,7 +7895,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="2:17" ht="26.15" customHeight="1">
+    <row r="39" spans="2:17" ht="26.1" customHeight="1">
       <c r="B39" s="2">
         <v>30</v>
       </c>
@@ -7899,7 +7912,7 @@
         <v>17</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H39" s="3">
         <v>46197</v>
@@ -7933,7 +7946,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="2:17" ht="26.15" customHeight="1">
+    <row r="40" spans="2:17" ht="26.1" customHeight="1">
       <c r="B40" s="2">
         <v>31</v>
       </c>
@@ -7950,7 +7963,7 @@
         <v>50</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H40" s="3">
         <v>46197</v>
@@ -7984,7 +7997,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="2:17" ht="26.15" customHeight="1">
+    <row r="41" spans="2:17" ht="26.1" customHeight="1">
       <c r="B41" s="2">
         <v>32</v>
       </c>
@@ -8001,7 +8014,7 @@
         <v>21</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H41" s="3">
         <v>46210</v>
@@ -8035,7 +8048,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="2:17" ht="26.15" customHeight="1">
+    <row r="42" spans="2:17" ht="26.1" customHeight="1">
       <c r="B42" s="2">
         <v>33</v>
       </c>
@@ -8052,7 +8065,7 @@
         <v>45</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H42" s="3">
         <v>46210</v>
@@ -8086,7 +8099,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="2:17" ht="26.15" customHeight="1">
+    <row r="43" spans="2:17" ht="26.1" customHeight="1">
       <c r="B43" s="2">
         <v>34</v>
       </c>
@@ -8137,7 +8150,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:17" ht="26.15" customHeight="1">
+    <row r="44" spans="2:17" ht="26.1" customHeight="1">
       <c r="B44" s="2">
         <v>35</v>
       </c>
@@ -8188,7 +8201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="2:17" ht="26.15" customHeight="1">
+    <row r="45" spans="2:17" ht="26.1" customHeight="1">
       <c r="B45" s="2">
         <v>36</v>
       </c>
@@ -8237,7 +8250,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:17" ht="26.15" customHeight="1">
+    <row r="46" spans="2:17" ht="26.1" customHeight="1">
       <c r="B46" s="2">
         <v>37</v>
       </c>
@@ -8286,7 +8299,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="2:17" ht="26.15" customHeight="1">
+    <row r="47" spans="2:17" ht="26.1" customHeight="1">
       <c r="B47" s="2">
         <v>38</v>
       </c>
@@ -8335,7 +8348,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="2:17" ht="26.15" customHeight="1">
+    <row r="48" spans="2:17" ht="26.1" customHeight="1">
       <c r="B48" s="2">
         <v>39</v>
       </c>
@@ -8384,7 +8397,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="2:17" ht="26.15" customHeight="1">
+    <row r="49" spans="2:17" ht="26.1" customHeight="1">
       <c r="B49" s="2">
         <v>40</v>
       </c>
@@ -8416,7 +8429,7 @@
       <c r="P49" s="65"/>
       <c r="Q49" s="56"/>
     </row>
-    <row r="50" spans="2:17" ht="26.15" customHeight="1">
+    <row r="50" spans="2:17" ht="26.1" customHeight="1">
       <c r="B50" s="2"/>
       <c r="C50" s="2">
         <v>5659</v>
@@ -8442,7 +8455,7 @@
       <c r="P50" s="65"/>
       <c r="Q50" s="56"/>
     </row>
-    <row r="51" spans="2:17" ht="24.65" customHeight="1">
+    <row r="51" spans="2:17" ht="24.6" customHeight="1">
       <c r="B51" s="76"/>
       <c r="C51" s="2">
         <v>13650</v>
@@ -8486,36 +8499,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C015DEDA-282C-4A92-9944-4B7B289C369E}">
   <dimension ref="B9:AH100"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.08984375" style="11" customWidth="1"/>
-    <col min="2" max="2" width="18.90625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="18.90625" style="11" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="18.90625" style="11" customWidth="1"/>
-    <col min="5" max="5" width="15.90625" style="11" customWidth="1"/>
-    <col min="6" max="6" width="23.08984375" style="11" customWidth="1"/>
-    <col min="7" max="8" width="18.90625" style="11" customWidth="1"/>
-    <col min="9" max="9" width="23.90625" style="11" customWidth="1"/>
-    <col min="10" max="12" width="22.90625" style="11" customWidth="1"/>
-    <col min="13" max="13" width="25.90625" style="11" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" style="11" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" style="11" customWidth="1"/>
+    <col min="7" max="8" width="18.85546875" style="11" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" style="11" customWidth="1"/>
+    <col min="10" max="12" width="22.85546875" style="11" customWidth="1"/>
+    <col min="13" max="13" width="25.85546875" style="11" customWidth="1"/>
     <col min="14" max="15" width="29" style="11" customWidth="1"/>
-    <col min="16" max="16" width="27.08984375" style="11" customWidth="1"/>
-    <col min="17" max="17" width="74.7265625" style="11" customWidth="1"/>
-    <col min="18" max="18" width="67.90625" style="11" customWidth="1"/>
-    <col min="19" max="20" width="63.90625" style="11" customWidth="1"/>
-    <col min="21" max="21" width="63.08984375" style="11" customWidth="1"/>
+    <col min="16" max="16" width="27.140625" style="11" customWidth="1"/>
+    <col min="17" max="17" width="74.7109375" style="11" customWidth="1"/>
+    <col min="18" max="18" width="67.85546875" style="11" customWidth="1"/>
+    <col min="19" max="20" width="63.85546875" style="11" customWidth="1"/>
+    <col min="21" max="21" width="63.140625" style="11" customWidth="1"/>
     <col min="22" max="22" width="73" style="11" customWidth="1"/>
-    <col min="23" max="23" width="72.54296875" style="11" customWidth="1"/>
-    <col min="24" max="24" width="79.453125" style="11" customWidth="1"/>
+    <col min="23" max="23" width="72.5703125" style="11" customWidth="1"/>
+    <col min="24" max="24" width="79.42578125" style="11" customWidth="1"/>
     <col min="25" max="25" width="71" style="11" customWidth="1"/>
-    <col min="26" max="28" width="71.90625" style="11" customWidth="1"/>
-    <col min="29" max="29" width="74.08984375" style="11" customWidth="1"/>
-    <col min="30" max="30" width="60.54296875" style="11" customWidth="1"/>
-    <col min="31" max="31" width="64.08984375" style="11" customWidth="1"/>
-    <col min="32" max="32" width="57.453125" style="11" customWidth="1"/>
+    <col min="26" max="28" width="71.85546875" style="11" customWidth="1"/>
+    <col min="29" max="29" width="74.140625" style="11" customWidth="1"/>
+    <col min="30" max="30" width="60.5703125" style="11" customWidth="1"/>
+    <col min="31" max="31" width="64.140625" style="11" customWidth="1"/>
+    <col min="32" max="32" width="57.42578125" style="11" customWidth="1"/>
     <col min="33" max="33" width="0" style="11" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="74.08984375" style="11" customWidth="1"/>
-    <col min="35" max="16384" width="11.453125" style="11"/>
+    <col min="34" max="34" width="74.140625" style="11" customWidth="1"/>
+    <col min="35" max="16384" width="11.42578125" style="11"/>
   </cols>
   <sheetData>
     <row r="9" spans="2:34" s="10" customFormat="1">
@@ -8535,7 +8548,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>145</v>
@@ -8574,16 +8587,16 @@
         <v>13</v>
       </c>
       <c r="Q10" s="69" t="s">
+        <v>352</v>
+      </c>
+      <c r="R10" s="69" t="s">
         <v>353</v>
       </c>
-      <c r="R10" s="69" t="s">
-        <v>354</v>
-      </c>
       <c r="S10" s="69" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="T10" s="69" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="U10" s="15" t="s">
         <v>137</v>
@@ -8625,10 +8638,10 @@
         <v>153</v>
       </c>
       <c r="AH10" s="45" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
-    <row r="11" spans="2:34" ht="97.65" customHeight="1">
+    <row r="11" spans="2:34" ht="149.25" customHeight="1">
       <c r="B11" s="31">
         <v>68575</v>
       </c>
@@ -8679,7 +8692,7 @@
       <c r="S11" s="70"/>
       <c r="T11" s="70"/>
       <c r="U11" s="19" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="V11" s="19" t="s">
         <v>156</v>
@@ -8696,14 +8709,14 @@
       <c r="Z11" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="AA11" s="19" t="s">
-        <v>184</v>
+      <c r="AA11" s="81" t="s">
+        <v>734</v>
       </c>
       <c r="AB11" s="19" t="s">
         <v>140</v>
       </c>
       <c r="AC11" s="19" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AD11" s="19" t="s">
         <v>165</v>
@@ -8718,10 +8731,10 @@
         <v>138</v>
       </c>
       <c r="AH11" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
-    <row r="12" spans="2:34" ht="92">
+    <row r="12" spans="2:34" ht="96">
       <c r="B12" s="16">
         <v>13442</v>
       </c>
@@ -8768,19 +8781,19 @@
         <v>45905</v>
       </c>
       <c r="Q12" s="19" t="s">
+        <v>629</v>
+      </c>
+      <c r="R12" s="19" t="s">
         <v>630</v>
       </c>
-      <c r="R12" s="19" t="s">
-        <v>631</v>
-      </c>
       <c r="S12" s="19" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="T12" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U12" s="19" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="V12" s="19" t="s">
         <v>158</v>
@@ -8813,14 +8826,14 @@
         <v>164</v>
       </c>
       <c r="AF12" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AG12" s="46"/>
       <c r="AH12" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
-    <row r="13" spans="2:34" ht="143" customHeight="1">
+    <row r="13" spans="2:34" ht="143.1" customHeight="1">
       <c r="B13" s="16">
         <v>47161</v>
       </c>
@@ -8867,19 +8880,19 @@
         <v>45908</v>
       </c>
       <c r="Q13" s="19" t="s">
+        <v>633</v>
+      </c>
+      <c r="R13" s="19" t="s">
         <v>634</v>
       </c>
-      <c r="R13" s="19" t="s">
-        <v>635</v>
-      </c>
       <c r="S13" s="19" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="T13" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U13" s="19" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="V13" s="19" t="s">
         <v>168</v>
@@ -8888,7 +8901,7 @@
         <v>169</v>
       </c>
       <c r="X13" s="19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="Y13" s="64" t="s">
         <v>174</v>
@@ -8897,7 +8910,7 @@
         <v>170</v>
       </c>
       <c r="AA13" s="19" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="AB13" s="19" t="s">
         <v>167</v>
@@ -8916,10 +8929,10 @@
       </c>
       <c r="AG13" s="46"/>
       <c r="AH13" s="19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
-    <row r="14" spans="2:34" ht="80.5">
+    <row r="14" spans="2:34" ht="84">
       <c r="B14" s="16">
         <v>47555</v>
       </c>
@@ -8966,19 +8979,19 @@
         <v>45933</v>
       </c>
       <c r="Q14" s="19" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="R14" s="19" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="S14" s="19" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="T14" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U14" s="19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="V14" s="19" t="s">
         <v>176</v>
@@ -8987,7 +9000,7 @@
         <v>177</v>
       </c>
       <c r="X14" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Y14" s="64" t="s">
         <v>174</v>
@@ -8996,7 +9009,7 @@
         <v>174</v>
       </c>
       <c r="AA14" s="19" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AB14" s="19" t="s">
         <v>175</v>
@@ -9015,10 +9028,10 @@
       </c>
       <c r="AG14" s="46"/>
       <c r="AH14" s="19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
-    <row r="15" spans="2:34" ht="69">
+    <row r="15" spans="2:34" ht="72">
       <c r="B15" s="16">
         <v>47692</v>
       </c>
@@ -9065,59 +9078,59 @@
         <v>45933</v>
       </c>
       <c r="Q15" s="19" t="s">
+        <v>621</v>
+      </c>
+      <c r="R15" s="19" t="s">
         <v>622</v>
       </c>
-      <c r="R15" s="19" t="s">
-        <v>623</v>
-      </c>
       <c r="S15" s="19" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="T15" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U15" s="19" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="V15" s="19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="W15" s="19" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="X15" s="19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Y15" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z15" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="AA15" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="AA15" s="19" t="s">
+      <c r="AB15" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="AC15" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="AB15" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="AC15" s="19" t="s">
+      <c r="AD15" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="AD15" s="19" t="s">
+      <c r="AE15" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="AE15" s="19" t="s">
+      <c r="AF15" s="19" t="s">
         <v>193</v>
-      </c>
-      <c r="AF15" s="19" t="s">
-        <v>194</v>
       </c>
       <c r="AG15" s="46"/>
       <c r="AH15" s="19" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
-    <row r="16" spans="2:34" ht="80.5">
+    <row r="16" spans="2:34" ht="96">
       <c r="B16" s="16">
         <v>47745</v>
       </c>
@@ -9164,59 +9177,59 @@
         <v>45985</v>
       </c>
       <c r="Q16" s="19" t="s">
+        <v>623</v>
+      </c>
+      <c r="R16" s="19" t="s">
         <v>624</v>
       </c>
-      <c r="R16" s="19" t="s">
-        <v>625</v>
-      </c>
       <c r="S16" s="19" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="T16" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U16" s="19" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="V16" s="19" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="W16" s="64" t="s">
         <v>174</v>
       </c>
       <c r="X16" s="19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Y16" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z16" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="AA16" s="19" t="s">
         <v>282</v>
       </c>
-      <c r="AA16" s="19" t="s">
-        <v>283</v>
-      </c>
       <c r="AB16" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="AC16" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="AC16" s="19" t="s">
+      <c r="AD16" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="AD16" s="19" t="s">
+      <c r="AE16" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="AE16" s="19" t="s">
+      <c r="AF16" s="19" t="s">
         <v>199</v>
-      </c>
-      <c r="AF16" s="19" t="s">
-        <v>200</v>
       </c>
       <c r="AG16" s="46"/>
       <c r="AH16" s="19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
-    <row r="17" spans="2:34" ht="69">
+    <row r="17" spans="2:34" ht="72">
       <c r="B17" s="16">
         <v>73275</v>
       </c>
@@ -9263,28 +9276,28 @@
         <v>45994</v>
       </c>
       <c r="Q17" s="19" t="s">
+        <v>625</v>
+      </c>
+      <c r="R17" s="19" t="s">
         <v>626</v>
       </c>
-      <c r="R17" s="19" t="s">
-        <v>627</v>
-      </c>
       <c r="S17" s="19" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="T17" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U17" s="19" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="V17" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="W17" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="W17" s="19" t="s">
-        <v>203</v>
-      </c>
       <c r="X17" s="19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="Y17" s="64" t="s">
         <v>174</v>
@@ -9293,29 +9306,29 @@
         <v>174</v>
       </c>
       <c r="AA17" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="AB17" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="AC17" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="AD17" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="AB17" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="AC17" s="19" t="s">
+      <c r="AE17" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="AD17" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="AE17" s="19" t="s">
+      <c r="AF17" s="19" t="s">
         <v>207</v>
-      </c>
-      <c r="AF17" s="19" t="s">
-        <v>208</v>
       </c>
       <c r="AG17" s="46"/>
       <c r="AH17" s="19" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
-    <row r="18" spans="2:34" ht="69">
+    <row r="18" spans="2:34" ht="72">
       <c r="B18" s="16">
         <v>5591</v>
       </c>
@@ -9362,59 +9375,59 @@
         <v>45996</v>
       </c>
       <c r="Q18" s="19" t="s">
+        <v>627</v>
+      </c>
+      <c r="R18" s="19" t="s">
         <v>628</v>
       </c>
-      <c r="R18" s="19" t="s">
-        <v>629</v>
-      </c>
       <c r="S18" s="19" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="T18" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U18" s="19" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="V18" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="W18" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="W18" s="19" t="s">
-        <v>211</v>
-      </c>
       <c r="X18" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="Y18" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z18" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="AA18" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="AA18" s="19" t="s">
+      <c r="AB18" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="AC18" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="AB18" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="AC18" s="19" t="s">
+      <c r="AD18" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="AD18" s="19" t="s">
+      <c r="AE18" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="AE18" s="19" t="s">
+      <c r="AF18" s="19" t="s">
         <v>216</v>
-      </c>
-      <c r="AF18" s="19" t="s">
-        <v>217</v>
       </c>
       <c r="AG18" s="46"/>
       <c r="AH18" s="19" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
-    <row r="19" spans="2:34" ht="69">
+    <row r="19" spans="2:34" ht="72">
       <c r="B19" s="16">
         <v>73217</v>
       </c>
@@ -9461,59 +9474,59 @@
         <v>46008</v>
       </c>
       <c r="Q19" s="19" t="s">
+        <v>635</v>
+      </c>
+      <c r="R19" s="19" t="s">
         <v>636</v>
       </c>
-      <c r="R19" s="19" t="s">
-        <v>637</v>
-      </c>
       <c r="S19" s="19" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="T19" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U19" s="19" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="V19" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="W19" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="W19" s="19" t="s">
-        <v>220</v>
-      </c>
       <c r="X19" s="19" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Y19" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z19" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="AA19" s="19" t="s">
         <v>228</v>
       </c>
-      <c r="AA19" s="19" t="s">
+      <c r="AB19" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="AC19" s="19" t="s">
+        <v>230</v>
+      </c>
+      <c r="AD19" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="AB19" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="AC19" s="19" t="s">
+      <c r="AE19" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="AD19" s="19" t="s">
-        <v>230</v>
-      </c>
-      <c r="AE19" s="19" t="s">
+      <c r="AF19" s="19" t="s">
         <v>232</v>
-      </c>
-      <c r="AF19" s="19" t="s">
-        <v>233</v>
       </c>
       <c r="AG19" s="46"/>
       <c r="AH19" s="19" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
-    <row r="20" spans="2:34" ht="92">
+    <row r="20" spans="2:34" ht="96">
       <c r="B20" s="16">
         <v>20295</v>
       </c>
@@ -9560,59 +9573,59 @@
         <v>46011</v>
       </c>
       <c r="Q20" s="19" t="s">
+        <v>637</v>
+      </c>
+      <c r="R20" s="19" t="s">
         <v>638</v>
       </c>
-      <c r="R20" s="19" t="s">
-        <v>639</v>
-      </c>
       <c r="S20" s="19" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="T20" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U20" s="19" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="V20" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W20" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="X20" s="19" t="s">
         <v>236</v>
-      </c>
-      <c r="X20" s="19" t="s">
-        <v>237</v>
       </c>
       <c r="Y20" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z20" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="AA20" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="AA20" s="19" t="s">
+      <c r="AB20" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="AC20" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="AB20" s="19" t="s">
-        <v>235</v>
-      </c>
-      <c r="AC20" s="19" t="s">
+      <c r="AD20" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="AD20" s="19" t="s">
+      <c r="AE20" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="AF20" s="19" t="s">
         <v>241</v>
-      </c>
-      <c r="AE20" s="19" t="s">
-        <v>315</v>
-      </c>
-      <c r="AF20" s="19" t="s">
-        <v>242</v>
       </c>
       <c r="AG20" s="46"/>
       <c r="AH20" s="19" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
-    <row r="21" spans="2:34" ht="80.5">
+    <row r="21" spans="2:34" ht="84">
       <c r="B21" s="16">
         <v>20787</v>
       </c>
@@ -9659,59 +9672,59 @@
         <v>46008</v>
       </c>
       <c r="Q21" s="19" t="s">
+        <v>639</v>
+      </c>
+      <c r="R21" s="19" t="s">
         <v>640</v>
       </c>
-      <c r="R21" s="19" t="s">
-        <v>641</v>
-      </c>
       <c r="S21" s="19" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="T21" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U21" s="19" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="V21" s="64" t="s">
         <v>174</v>
       </c>
       <c r="W21" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="X21" s="19" t="s">
         <v>244</v>
-      </c>
-      <c r="X21" s="19" t="s">
-        <v>245</v>
       </c>
       <c r="Y21" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z21" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="AA21" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="AA21" s="19" t="s">
+      <c r="AB21" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="AC21" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="AD21" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="AB21" s="19" t="s">
-        <v>243</v>
-      </c>
-      <c r="AC21" s="19" t="s">
+      <c r="AE21" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="AF21" s="19" t="s">
         <v>249</v>
-      </c>
-      <c r="AD21" s="19" t="s">
-        <v>248</v>
-      </c>
-      <c r="AE21" s="19" t="s">
-        <v>316</v>
-      </c>
-      <c r="AF21" s="19" t="s">
-        <v>250</v>
       </c>
       <c r="AG21" s="46"/>
       <c r="AH21" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
-    <row r="22" spans="2:34" ht="57.5">
+    <row r="22" spans="2:34" ht="60">
       <c r="B22" s="16">
         <v>13248</v>
       </c>
@@ -9758,28 +9771,28 @@
         <v>46014</v>
       </c>
       <c r="Q22" s="19" t="s">
+        <v>641</v>
+      </c>
+      <c r="R22" s="19" t="s">
         <v>642</v>
       </c>
-      <c r="R22" s="19" t="s">
-        <v>643</v>
-      </c>
       <c r="S22" s="19" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="T22" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U22" s="19" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="V22" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="W22" s="19" t="s">
         <v>252</v>
       </c>
-      <c r="W22" s="19" t="s">
+      <c r="X22" s="19" t="s">
         <v>253</v>
-      </c>
-      <c r="X22" s="19" t="s">
-        <v>254</v>
       </c>
       <c r="Y22" s="64" t="s">
         <v>174</v>
@@ -9788,29 +9801,29 @@
         <v>174</v>
       </c>
       <c r="AA22" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="AB22" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="AC22" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="AD22" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="AB22" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="AC22" s="19" t="s">
+      <c r="AE22" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="AF22" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="AD22" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="AE22" s="19" t="s">
-        <v>317</v>
-      </c>
-      <c r="AF22" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="AG22" s="46"/>
       <c r="AH22" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
-    <row r="23" spans="2:34" ht="115">
+    <row r="23" spans="2:34" ht="120">
       <c r="B23" s="16">
         <v>13140</v>
       </c>
@@ -9857,57 +9870,57 @@
         <v>46045</v>
       </c>
       <c r="Q23" s="19" t="s">
+        <v>643</v>
+      </c>
+      <c r="R23" s="19" t="s">
         <v>644</v>
       </c>
-      <c r="R23" s="19" t="s">
-        <v>645</v>
-      </c>
       <c r="S23" s="73" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="T23" s="71"/>
       <c r="U23" s="19" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="V23" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="W23" s="19" t="s">
+        <v>296</v>
+      </c>
+      <c r="X23" s="19" t="s">
         <v>260</v>
-      </c>
-      <c r="W23" s="19" t="s">
-        <v>297</v>
-      </c>
-      <c r="X23" s="19" t="s">
-        <v>261</v>
       </c>
       <c r="Y23" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z23" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="AA23" s="19" t="s">
         <v>262</v>
       </c>
-      <c r="AA23" s="19" t="s">
+      <c r="AB23" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="AC23" s="19" t="s">
+        <v>358</v>
+      </c>
+      <c r="AD23" s="19" t="s">
         <v>263</v>
       </c>
-      <c r="AB23" s="19" t="s">
-        <v>259</v>
-      </c>
-      <c r="AC23" s="19" t="s">
-        <v>359</v>
-      </c>
-      <c r="AD23" s="19" t="s">
+      <c r="AE23" s="19" t="s">
+        <v>317</v>
+      </c>
+      <c r="AF23" s="19" t="s">
         <v>264</v>
-      </c>
-      <c r="AE23" s="19" t="s">
-        <v>318</v>
-      </c>
-      <c r="AF23" s="19" t="s">
-        <v>265</v>
       </c>
       <c r="AG23" s="46"/>
       <c r="AH23" s="19" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
-    <row r="24" spans="2:34" ht="80.5">
+    <row r="24" spans="2:34" ht="84">
       <c r="B24" s="16">
         <v>70124</v>
       </c>
@@ -9954,59 +9967,59 @@
         <v>46048</v>
       </c>
       <c r="Q24" s="19" t="s">
+        <v>645</v>
+      </c>
+      <c r="R24" s="19" t="s">
         <v>646</v>
       </c>
-      <c r="R24" s="19" t="s">
-        <v>647</v>
-      </c>
       <c r="S24" s="19" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="T24" s="19" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="U24" s="19" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="V24" s="19" t="s">
+        <v>266</v>
+      </c>
+      <c r="W24" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="W24" s="19" t="s">
+      <c r="X24" s="19" t="s">
         <v>268</v>
-      </c>
-      <c r="X24" s="19" t="s">
-        <v>269</v>
       </c>
       <c r="Y24" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z24" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA24" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="AA24" s="19" t="s">
+      <c r="AB24" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="AC24" s="19" t="s">
+        <v>359</v>
+      </c>
+      <c r="AD24" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="AB24" s="19" t="s">
-        <v>266</v>
-      </c>
-      <c r="AC24" s="19" t="s">
-        <v>360</v>
-      </c>
-      <c r="AD24" s="19" t="s">
+      <c r="AE24" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="AF24" s="19" t="s">
         <v>272</v>
-      </c>
-      <c r="AE24" s="19" t="s">
-        <v>319</v>
-      </c>
-      <c r="AF24" s="19" t="s">
-        <v>273</v>
       </c>
       <c r="AG24" s="46"/>
       <c r="AH24" s="19" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
-    <row r="25" spans="2:34" ht="80.5">
+    <row r="25" spans="2:34" ht="84">
       <c r="B25" s="16">
         <v>70678</v>
       </c>
@@ -10053,59 +10066,59 @@
         <v>46049</v>
       </c>
       <c r="Q25" s="19" t="s">
+        <v>647</v>
+      </c>
+      <c r="R25" s="19" t="s">
         <v>648</v>
       </c>
-      <c r="R25" s="19" t="s">
-        <v>649</v>
-      </c>
       <c r="S25" s="19" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="T25" s="19" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="U25" s="19" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="V25" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="W25" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="W25" s="19" t="s">
+      <c r="X25" s="19" t="s">
         <v>276</v>
-      </c>
-      <c r="X25" s="19" t="s">
-        <v>277</v>
       </c>
       <c r="Y25" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z25" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA25" s="19" t="s">
         <v>278</v>
       </c>
-      <c r="AA25" s="19" t="s">
+      <c r="AB25" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="AC25" s="19" t="s">
+        <v>360</v>
+      </c>
+      <c r="AD25" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="AE25" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="AF25" s="19" t="s">
         <v>279</v>
-      </c>
-      <c r="AB25" s="19" t="s">
-        <v>274</v>
-      </c>
-      <c r="AC25" s="19" t="s">
-        <v>361</v>
-      </c>
-      <c r="AD25" s="19" t="s">
-        <v>304</v>
-      </c>
-      <c r="AE25" s="19" t="s">
-        <v>320</v>
-      </c>
-      <c r="AF25" s="19" t="s">
-        <v>280</v>
       </c>
       <c r="AG25" s="46"/>
       <c r="AH25" s="19" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
-    <row r="26" spans="2:34" ht="92">
+    <row r="26" spans="2:34" ht="96">
       <c r="B26" s="16">
         <v>95001</v>
       </c>
@@ -10152,59 +10165,59 @@
         <v>46066</v>
       </c>
       <c r="Q26" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="R26" s="19" t="s">
         <v>650</v>
       </c>
-      <c r="R26" s="19" t="s">
-        <v>651</v>
-      </c>
       <c r="S26" s="19" t="s">
+        <v>599</v>
+      </c>
+      <c r="T26" s="19" t="s">
         <v>600</v>
       </c>
-      <c r="T26" s="19" t="s">
-        <v>601</v>
-      </c>
       <c r="U26" s="19" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="V26" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="W26" s="19" t="s">
         <v>299</v>
       </c>
-      <c r="W26" s="19" t="s">
+      <c r="X26" s="19" t="s">
         <v>300</v>
-      </c>
-      <c r="X26" s="19" t="s">
-        <v>301</v>
       </c>
       <c r="Y26" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z26" s="19" t="s">
+        <v>301</v>
+      </c>
+      <c r="AA26" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="AB26" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="AC26" s="19" t="s">
+        <v>327</v>
+      </c>
+      <c r="AD26" s="19" t="s">
         <v>302</v>
       </c>
-      <c r="AA26" s="19" t="s">
-        <v>548</v>
-      </c>
-      <c r="AB26" s="19" t="s">
-        <v>298</v>
-      </c>
-      <c r="AC26" s="19" t="s">
-        <v>328</v>
-      </c>
-      <c r="AD26" s="19" t="s">
-        <v>303</v>
-      </c>
       <c r="AE26" s="19" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AF26" s="19" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AG26" s="66"/>
       <c r="AH26" s="19" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
-    <row r="27" spans="2:34" ht="80.5">
+    <row r="27" spans="2:34" ht="96">
       <c r="B27" s="16">
         <v>17495</v>
       </c>
@@ -10251,28 +10264,28 @@
         <v>46069</v>
       </c>
       <c r="Q27" s="19" t="s">
+        <v>651</v>
+      </c>
+      <c r="R27" s="19" t="s">
         <v>652</v>
       </c>
-      <c r="R27" s="19" t="s">
-        <v>653</v>
-      </c>
       <c r="S27" s="19" t="s">
+        <v>601</v>
+      </c>
+      <c r="T27" s="19" t="s">
         <v>602</v>
       </c>
-      <c r="T27" s="19" t="s">
-        <v>603</v>
-      </c>
       <c r="U27" s="19" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="V27" s="19" t="s">
+        <v>322</v>
+      </c>
+      <c r="W27" s="19" t="s">
+        <v>329</v>
+      </c>
+      <c r="X27" s="19" t="s">
         <v>323</v>
-      </c>
-      <c r="W27" s="19" t="s">
-        <v>330</v>
-      </c>
-      <c r="X27" s="19" t="s">
-        <v>324</v>
       </c>
       <c r="Y27" s="64" t="s">
         <v>174</v>
@@ -10281,29 +10294,29 @@
         <v>174</v>
       </c>
       <c r="AA27" s="19" t="s">
+        <v>324</v>
+      </c>
+      <c r="AB27" s="19" t="s">
+        <v>321</v>
+      </c>
+      <c r="AC27" s="19" t="s">
+        <v>330</v>
+      </c>
+      <c r="AD27" s="19" t="s">
+        <v>354</v>
+      </c>
+      <c r="AE27" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="AB27" s="19" t="s">
-        <v>322</v>
-      </c>
-      <c r="AC27" s="19" t="s">
-        <v>331</v>
-      </c>
-      <c r="AD27" s="19" t="s">
-        <v>355</v>
-      </c>
-      <c r="AE27" s="19" t="s">
+      <c r="AF27" s="19" t="s">
         <v>326</v>
-      </c>
-      <c r="AF27" s="19" t="s">
-        <v>327</v>
       </c>
       <c r="AG27" s="66"/>
       <c r="AH27" s="19" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
-    <row r="28" spans="2:34" ht="161">
+    <row r="28" spans="2:34" ht="168">
       <c r="B28" s="67">
         <v>68575</v>
       </c>
@@ -10317,7 +10330,7 @@
         <v>60</v>
       </c>
       <c r="F28" s="68" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G28" s="68" t="s">
         <v>4</v>
@@ -10354,44 +10367,44 @@
       <c r="S28" s="71"/>
       <c r="T28" s="71"/>
       <c r="U28" s="19" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="V28" s="64" t="s">
         <v>174</v>
       </c>
       <c r="W28" s="19" t="s">
+        <v>309</v>
+      </c>
+      <c r="X28" s="19" t="s">
         <v>310</v>
-      </c>
-      <c r="X28" s="19" t="s">
-        <v>311</v>
       </c>
       <c r="Y28" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z28" s="19" t="s">
+        <v>311</v>
+      </c>
+      <c r="AA28" s="19" t="s">
         <v>312</v>
       </c>
-      <c r="AA28" s="19" t="s">
+      <c r="AB28" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="AC28" s="19" t="s">
+        <v>361</v>
+      </c>
+      <c r="AD28" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="AE28" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="AF28" s="19" t="s">
         <v>313</v>
-      </c>
-      <c r="AB28" s="19" t="s">
-        <v>309</v>
-      </c>
-      <c r="AC28" s="19" t="s">
-        <v>362</v>
-      </c>
-      <c r="AD28" s="19" t="s">
-        <v>333</v>
-      </c>
-      <c r="AE28" s="19" t="s">
-        <v>332</v>
-      </c>
-      <c r="AF28" s="19" t="s">
-        <v>314</v>
       </c>
       <c r="AG28" s="66"/>
       <c r="AH28" s="19" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="29" spans="2:34" ht="72" customHeight="1">
@@ -10441,56 +10454,56 @@
         <v>46129</v>
       </c>
       <c r="Q29" s="32" t="s">
+        <v>653</v>
+      </c>
+      <c r="R29" s="32" t="s">
         <v>654</v>
       </c>
-      <c r="R29" s="32" t="s">
-        <v>655</v>
-      </c>
       <c r="S29" s="32" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="T29" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U29" s="19" t="s">
+        <v>366</v>
+      </c>
+      <c r="V29" s="19" t="s">
         <v>367</v>
       </c>
-      <c r="V29" s="19" t="s">
-        <v>368</v>
-      </c>
       <c r="W29" s="19" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="X29" s="19" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="Y29" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z29" s="19" t="s">
+        <v>371</v>
+      </c>
+      <c r="AA29" s="19" t="s">
         <v>372</v>
       </c>
-      <c r="AA29" s="19" t="s">
+      <c r="AB29" s="19" t="s">
         <v>373</v>
       </c>
-      <c r="AB29" s="19" t="s">
+      <c r="AC29" s="19" t="s">
+        <v>414</v>
+      </c>
+      <c r="AD29" s="19" t="s">
         <v>374</v>
       </c>
-      <c r="AC29" s="19" t="s">
-        <v>415</v>
-      </c>
-      <c r="AD29" s="19" t="s">
+      <c r="AE29" s="19" t="s">
         <v>375</v>
       </c>
-      <c r="AE29" s="19" t="s">
+      <c r="AF29" s="19" t="s">
         <v>376</v>
-      </c>
-      <c r="AF29" s="19" t="s">
-        <v>377</v>
       </c>
       <c r="AG29" s="46"/>
       <c r="AH29" s="19" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="30" spans="2:34" ht="76.5" customHeight="1">
@@ -10540,59 +10553,59 @@
         <v>46129</v>
       </c>
       <c r="Q30" s="32" t="s">
+        <v>655</v>
+      </c>
+      <c r="R30" s="32" t="s">
         <v>656</v>
       </c>
-      <c r="R30" s="32" t="s">
-        <v>657</v>
-      </c>
       <c r="S30" s="32" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="T30" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U30" s="19" t="s">
+        <v>368</v>
+      </c>
+      <c r="V30" s="19" t="s">
         <v>369</v>
       </c>
-      <c r="V30" s="19" t="s">
-        <v>370</v>
-      </c>
       <c r="W30" s="19" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="X30" s="19" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="Y30" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z30" s="19" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="AA30" s="19" t="s">
+        <v>409</v>
+      </c>
+      <c r="AB30" s="19" t="s">
+        <v>378</v>
+      </c>
+      <c r="AC30" s="19" t="s">
+        <v>415</v>
+      </c>
+      <c r="AD30" s="19" t="s">
         <v>410</v>
       </c>
-      <c r="AB30" s="19" t="s">
+      <c r="AE30" s="19" t="s">
         <v>379</v>
       </c>
-      <c r="AC30" s="19" t="s">
-        <v>416</v>
-      </c>
-      <c r="AD30" s="19" t="s">
-        <v>411</v>
-      </c>
-      <c r="AE30" s="19" t="s">
+      <c r="AF30" s="19" t="s">
         <v>380</v>
-      </c>
-      <c r="AF30" s="19" t="s">
-        <v>381</v>
       </c>
       <c r="AG30" s="74"/>
       <c r="AH30" s="19" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
-    <row r="31" spans="2:34" ht="80.150000000000006" customHeight="1">
+    <row r="31" spans="2:34" ht="80.099999999999994" customHeight="1">
       <c r="B31" s="16">
         <v>8137</v>
       </c>
@@ -10639,28 +10652,28 @@
         <v>46134</v>
       </c>
       <c r="Q31" s="32" t="s">
+        <v>657</v>
+      </c>
+      <c r="R31" s="32" t="s">
         <v>658</v>
       </c>
-      <c r="R31" s="32" t="s">
-        <v>659</v>
-      </c>
       <c r="S31" s="32" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="T31" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U31" s="19" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="V31" s="19" t="s">
+        <v>381</v>
+      </c>
+      <c r="W31" s="19" t="s">
+        <v>391</v>
+      </c>
+      <c r="X31" s="19" t="s">
         <v>382</v>
-      </c>
-      <c r="W31" s="19" t="s">
-        <v>392</v>
-      </c>
-      <c r="X31" s="19" t="s">
-        <v>383</v>
       </c>
       <c r="Y31" s="64" t="s">
         <v>174</v>
@@ -10669,29 +10682,29 @@
         <v>174</v>
       </c>
       <c r="AA31" s="19" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AB31" s="19" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AC31" s="19" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="AD31" s="19" t="s">
+        <v>407</v>
+      </c>
+      <c r="AE31" s="19" t="s">
         <v>408</v>
       </c>
-      <c r="AE31" s="19" t="s">
-        <v>409</v>
-      </c>
       <c r="AF31" s="19" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="AG31" s="46"/>
       <c r="AH31" s="19" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
-    <row r="32" spans="2:34" ht="131.4" customHeight="1">
+    <row r="32" spans="2:34" ht="131.44999999999999" customHeight="1">
       <c r="B32" s="16">
         <v>13188</v>
       </c>
@@ -10738,59 +10751,59 @@
         <v>46135</v>
       </c>
       <c r="Q32" s="32" t="s">
+        <v>659</v>
+      </c>
+      <c r="R32" s="32" t="s">
         <v>660</v>
       </c>
-      <c r="R32" s="32" t="s">
-        <v>661</v>
-      </c>
       <c r="S32" s="32" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="T32" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U32" s="19" t="s">
+        <v>387</v>
+      </c>
+      <c r="V32" s="19" t="s">
         <v>388</v>
       </c>
-      <c r="V32" s="19" t="s">
-        <v>389</v>
-      </c>
       <c r="W32" s="19" t="s">
+        <v>392</v>
+      </c>
+      <c r="X32" s="19" t="s">
         <v>393</v>
-      </c>
-      <c r="X32" s="19" t="s">
-        <v>394</v>
       </c>
       <c r="Y32" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z32" s="19" t="s">
+        <v>394</v>
+      </c>
+      <c r="AA32" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="AA32" s="19" t="s">
+      <c r="AB32" s="19" t="s">
+        <v>386</v>
+      </c>
+      <c r="AC32" s="19" t="s">
+        <v>416</v>
+      </c>
+      <c r="AD32" s="19" t="s">
         <v>396</v>
       </c>
-      <c r="AB32" s="19" t="s">
-        <v>387</v>
-      </c>
-      <c r="AC32" s="19" t="s">
-        <v>417</v>
-      </c>
-      <c r="AD32" s="19" t="s">
+      <c r="AE32" s="19" t="s">
         <v>397</v>
       </c>
-      <c r="AE32" s="19" t="s">
+      <c r="AF32" s="19" t="s">
         <v>398</v>
-      </c>
-      <c r="AF32" s="19" t="s">
-        <v>399</v>
       </c>
       <c r="AG32" s="46"/>
       <c r="AH32" s="19" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
-    <row r="33" spans="2:34" ht="92">
+    <row r="33" spans="2:34" ht="96">
       <c r="B33" s="23">
         <v>8606</v>
       </c>
@@ -10837,59 +10850,59 @@
         <v>46140</v>
       </c>
       <c r="Q33" s="32" t="s">
+        <v>661</v>
+      </c>
+      <c r="R33" s="32" t="s">
         <v>662</v>
       </c>
-      <c r="R33" s="32" t="s">
-        <v>663</v>
-      </c>
       <c r="S33" s="32" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="T33" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U33" s="19" t="s">
+        <v>400</v>
+      </c>
+      <c r="V33" s="19" t="s">
         <v>401</v>
       </c>
-      <c r="V33" s="19" t="s">
-        <v>402</v>
-      </c>
       <c r="W33" s="19" t="s">
+        <v>411</v>
+      </c>
+      <c r="X33" s="19" t="s">
         <v>412</v>
-      </c>
-      <c r="X33" s="19" t="s">
-        <v>413</v>
       </c>
       <c r="Y33" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z33" s="19" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="AA33" s="19" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AB33" s="19" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AC33" s="19" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="AD33" s="19" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AE33" s="19" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AF33" s="19" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AG33" s="74"/>
       <c r="AH33" s="19" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
-    <row r="34" spans="2:34" ht="89.15" customHeight="1">
+    <row r="34" spans="2:34" ht="89.1" customHeight="1">
       <c r="B34" s="31">
         <v>20383</v>
       </c>
@@ -10936,28 +10949,28 @@
         <v>46162</v>
       </c>
       <c r="Q34" s="32" t="s">
+        <v>663</v>
+      </c>
+      <c r="R34" s="32" t="s">
         <v>664</v>
       </c>
-      <c r="R34" s="32" t="s">
-        <v>665</v>
-      </c>
       <c r="S34" s="32" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="T34" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U34" s="19" t="s">
+        <v>418</v>
+      </c>
+      <c r="V34" s="19" t="s">
         <v>419</v>
       </c>
-      <c r="V34" s="19" t="s">
+      <c r="W34" s="19" t="s">
         <v>420</v>
       </c>
-      <c r="W34" s="19" t="s">
+      <c r="X34" s="19" t="s">
         <v>421</v>
-      </c>
-      <c r="X34" s="19" t="s">
-        <v>422</v>
       </c>
       <c r="Y34" s="64" t="s">
         <v>174</v>
@@ -10966,29 +10979,29 @@
         <v>174</v>
       </c>
       <c r="AA34" s="19" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="AB34" s="19" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AC34" s="19" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="AD34" s="19" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="AE34" s="19" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="AF34" s="19" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="AG34" s="46"/>
       <c r="AH34" s="19" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
-    <row r="35" spans="2:34" ht="62.4" customHeight="1">
+    <row r="35" spans="2:34" ht="62.45" customHeight="1">
       <c r="B35" s="23">
         <v>13667</v>
       </c>
@@ -11035,28 +11048,28 @@
         <v>46183</v>
       </c>
       <c r="Q35" s="32" t="s">
+        <v>665</v>
+      </c>
+      <c r="R35" s="32" t="s">
         <v>666</v>
       </c>
-      <c r="R35" s="32" t="s">
-        <v>667</v>
-      </c>
       <c r="S35" s="32" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="T35" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U35" s="19" t="s">
+        <v>429</v>
+      </c>
+      <c r="V35" s="19" t="s">
         <v>430</v>
       </c>
-      <c r="V35" s="19" t="s">
-        <v>431</v>
-      </c>
       <c r="W35" s="19" t="s">
+        <v>435</v>
+      </c>
+      <c r="X35" s="19" t="s">
         <v>436</v>
-      </c>
-      <c r="X35" s="19" t="s">
-        <v>437</v>
       </c>
       <c r="Y35" s="64" t="s">
         <v>174</v>
@@ -11065,29 +11078,29 @@
         <v>174</v>
       </c>
       <c r="AA35" s="19" t="s">
+        <v>438</v>
+      </c>
+      <c r="AB35" s="19" t="s">
+        <v>437</v>
+      </c>
+      <c r="AC35" s="19" t="s">
+        <v>536</v>
+      </c>
+      <c r="AD35" s="19" t="s">
         <v>439</v>
       </c>
-      <c r="AB35" s="19" t="s">
-        <v>438</v>
-      </c>
-      <c r="AC35" s="19" t="s">
-        <v>537</v>
-      </c>
-      <c r="AD35" s="19" t="s">
+      <c r="AE35" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="AE35" s="19" t="s">
+      <c r="AF35" s="19" t="s">
         <v>441</v>
-      </c>
-      <c r="AF35" s="19" t="s">
-        <v>442</v>
       </c>
       <c r="AG35" s="46"/>
       <c r="AH35" s="19" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
-    <row r="36" spans="2:34" ht="69">
+    <row r="36" spans="2:34" ht="72">
       <c r="B36" s="16">
         <v>13780</v>
       </c>
@@ -11134,28 +11147,28 @@
         <v>46184</v>
       </c>
       <c r="Q36" s="32" t="s">
+        <v>667</v>
+      </c>
+      <c r="R36" s="32" t="s">
         <v>668</v>
       </c>
-      <c r="R36" s="32" t="s">
-        <v>669</v>
-      </c>
       <c r="S36" s="32" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="T36" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U36" s="19" t="s">
+        <v>431</v>
+      </c>
+      <c r="V36" s="19" t="s">
         <v>432</v>
       </c>
-      <c r="V36" s="19" t="s">
-        <v>433</v>
-      </c>
       <c r="W36" s="19" t="s">
+        <v>452</v>
+      </c>
+      <c r="X36" s="19" t="s">
         <v>453</v>
-      </c>
-      <c r="X36" s="19" t="s">
-        <v>454</v>
       </c>
       <c r="Y36" s="64" t="s">
         <v>174</v>
@@ -11164,29 +11177,29 @@
         <v>174</v>
       </c>
       <c r="AA36" s="19" t="s">
+        <v>454</v>
+      </c>
+      <c r="AB36" s="19" t="s">
+        <v>443</v>
+      </c>
+      <c r="AC36" s="19" t="s">
+        <v>537</v>
+      </c>
+      <c r="AD36" s="19" t="s">
         <v>455</v>
       </c>
-      <c r="AB36" s="19" t="s">
-        <v>444</v>
-      </c>
-      <c r="AC36" s="19" t="s">
-        <v>538</v>
-      </c>
-      <c r="AD36" s="19" t="s">
+      <c r="AE36" s="19" t="s">
         <v>456</v>
       </c>
-      <c r="AE36" s="19" t="s">
+      <c r="AF36" s="19" t="s">
         <v>457</v>
-      </c>
-      <c r="AF36" s="19" t="s">
-        <v>458</v>
       </c>
       <c r="AG36" s="46"/>
       <c r="AH36" s="19" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
-    <row r="37" spans="2:34" ht="69">
+    <row r="37" spans="2:34" ht="72">
       <c r="B37" s="16">
         <v>13160</v>
       </c>
@@ -11233,28 +11246,28 @@
         <v>46191</v>
       </c>
       <c r="Q37" s="32" t="s">
+        <v>669</v>
+      </c>
+      <c r="R37" s="32" t="s">
         <v>670</v>
       </c>
-      <c r="R37" s="32" t="s">
-        <v>671</v>
-      </c>
       <c r="S37" s="32" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="T37" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U37" s="19" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="V37" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="W37" s="19" t="s">
         <v>461</v>
       </c>
-      <c r="W37" s="19" t="s">
+      <c r="X37" s="19" t="s">
         <v>462</v>
-      </c>
-      <c r="X37" s="19" t="s">
-        <v>463</v>
       </c>
       <c r="Y37" s="64" t="s">
         <v>174</v>
@@ -11263,29 +11276,29 @@
         <v>174</v>
       </c>
       <c r="AA37" s="19" t="s">
+        <v>504</v>
+      </c>
+      <c r="AB37" s="19" t="s">
+        <v>444</v>
+      </c>
+      <c r="AC37" s="19" t="s">
+        <v>538</v>
+      </c>
+      <c r="AD37" s="19" t="s">
         <v>505</v>
       </c>
-      <c r="AB37" s="19" t="s">
-        <v>445</v>
-      </c>
-      <c r="AC37" s="19" t="s">
-        <v>539</v>
-      </c>
-      <c r="AD37" s="19" t="s">
-        <v>506</v>
-      </c>
       <c r="AE37" s="19" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="AF37" s="19" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="AG37" s="46"/>
       <c r="AH37" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
-    <row r="38" spans="2:34" ht="84.9" customHeight="1">
+    <row r="38" spans="2:34" ht="84.95" customHeight="1">
       <c r="B38" s="16">
         <v>13600</v>
       </c>
@@ -11332,28 +11345,28 @@
         <v>46192</v>
       </c>
       <c r="Q38" s="32" t="s">
+        <v>671</v>
+      </c>
+      <c r="R38" s="32" t="s">
         <v>672</v>
       </c>
-      <c r="R38" s="32" t="s">
-        <v>673</v>
-      </c>
       <c r="S38" s="32" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="T38" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U38" s="19" t="s">
+        <v>445</v>
+      </c>
+      <c r="V38" s="19" t="s">
         <v>446</v>
       </c>
-      <c r="V38" s="19" t="s">
+      <c r="W38" s="19" t="s">
         <v>447</v>
       </c>
-      <c r="W38" s="19" t="s">
+      <c r="X38" s="19" t="s">
         <v>448</v>
-      </c>
-      <c r="X38" s="19" t="s">
-        <v>449</v>
       </c>
       <c r="Y38" s="64" t="s">
         <v>174</v>
@@ -11362,29 +11375,29 @@
         <v>174</v>
       </c>
       <c r="AA38" s="19" t="s">
+        <v>458</v>
+      </c>
+      <c r="AB38" s="19" t="s">
+        <v>449</v>
+      </c>
+      <c r="AC38" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="AD38" s="19" t="s">
         <v>459</v>
       </c>
-      <c r="AB38" s="19" t="s">
+      <c r="AE38" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="AC38" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="AD38" s="19" t="s">
-        <v>460</v>
-      </c>
-      <c r="AE38" s="19" t="s">
-        <v>451</v>
-      </c>
       <c r="AF38" s="19" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="AG38" s="46"/>
       <c r="AH38" s="19" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
-    <row r="39" spans="2:34" ht="78.900000000000006" customHeight="1">
+    <row r="39" spans="2:34" ht="78.95" customHeight="1">
       <c r="B39" s="16">
         <v>13300</v>
       </c>
@@ -11431,28 +11444,28 @@
         <v>46205</v>
       </c>
       <c r="Q39" s="32" t="s">
+        <v>673</v>
+      </c>
+      <c r="R39" s="32" t="s">
         <v>674</v>
       </c>
-      <c r="R39" s="32" t="s">
-        <v>675</v>
-      </c>
       <c r="S39" s="32" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="T39" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U39" s="19" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="V39" s="19" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="W39" s="19" t="s">
+        <v>469</v>
+      </c>
+      <c r="X39" s="19" t="s">
         <v>470</v>
-      </c>
-      <c r="X39" s="19" t="s">
-        <v>471</v>
       </c>
       <c r="Y39" s="64" t="s">
         <v>174</v>
@@ -11461,29 +11474,29 @@
         <v>174</v>
       </c>
       <c r="AA39" s="19" t="s">
+        <v>483</v>
+      </c>
+      <c r="AB39" s="19" t="s">
+        <v>464</v>
+      </c>
+      <c r="AC39" s="19" t="s">
+        <v>548</v>
+      </c>
+      <c r="AD39" s="19" t="s">
+        <v>486</v>
+      </c>
+      <c r="AE39" s="19" t="s">
         <v>484</v>
       </c>
-      <c r="AB39" s="19" t="s">
-        <v>465</v>
-      </c>
-      <c r="AC39" s="19" t="s">
-        <v>549</v>
-      </c>
-      <c r="AD39" s="19" t="s">
-        <v>487</v>
-      </c>
-      <c r="AE39" s="19" t="s">
-        <v>485</v>
-      </c>
       <c r="AF39" s="19" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="AG39" s="46"/>
       <c r="AH39" s="19" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
-    <row r="40" spans="2:34" ht="80.5">
+    <row r="40" spans="2:34" ht="84">
       <c r="B40" s="16">
         <v>47720</v>
       </c>
@@ -11530,59 +11543,59 @@
         <v>46205</v>
       </c>
       <c r="Q40" s="32" t="s">
+        <v>675</v>
+      </c>
+      <c r="R40" s="32" t="s">
         <v>676</v>
       </c>
-      <c r="R40" s="32" t="s">
-        <v>677</v>
-      </c>
       <c r="S40" s="32" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="T40" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U40" s="19" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="V40" s="19" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="W40" s="19" t="s">
+        <v>473</v>
+      </c>
+      <c r="X40" s="19" t="s">
         <v>474</v>
-      </c>
-      <c r="X40" s="19" t="s">
-        <v>475</v>
       </c>
       <c r="Y40" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z40" s="19" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="AA40" s="19" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="AB40" s="19" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AC40" s="19" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AD40" s="19" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AE40" s="19" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="AF40" s="19" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AG40" s="46"/>
       <c r="AH40" s="19" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
-    <row r="41" spans="2:34" ht="69.650000000000006" customHeight="1">
+    <row r="41" spans="2:34" ht="69.599999999999994" customHeight="1">
       <c r="B41" s="16">
         <v>5579</v>
       </c>
@@ -11629,59 +11642,59 @@
         <v>46205</v>
       </c>
       <c r="Q41" s="32" t="s">
+        <v>677</v>
+      </c>
+      <c r="R41" s="32" t="s">
         <v>678</v>
       </c>
-      <c r="R41" s="32" t="s">
-        <v>679</v>
-      </c>
       <c r="S41" s="32" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="T41" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U41" s="19" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="V41" s="19" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="W41" s="19" t="s">
+        <v>471</v>
+      </c>
+      <c r="X41" s="19" t="s">
         <v>472</v>
-      </c>
-      <c r="X41" s="19" t="s">
-        <v>473</v>
       </c>
       <c r="Y41" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z41" s="19" t="s">
+        <v>481</v>
+      </c>
+      <c r="AA41" s="19" t="s">
+        <v>485</v>
+      </c>
+      <c r="AB41" s="19" t="s">
+        <v>468</v>
+      </c>
+      <c r="AC41" s="19" t="s">
+        <v>563</v>
+      </c>
+      <c r="AD41" s="19" t="s">
+        <v>487</v>
+      </c>
+      <c r="AE41" s="19" t="s">
         <v>482</v>
       </c>
-      <c r="AA41" s="19" t="s">
-        <v>486</v>
-      </c>
-      <c r="AB41" s="19" t="s">
-        <v>469</v>
-      </c>
-      <c r="AC41" s="19" t="s">
-        <v>564</v>
-      </c>
-      <c r="AD41" s="19" t="s">
-        <v>488</v>
-      </c>
-      <c r="AE41" s="19" t="s">
-        <v>483</v>
-      </c>
       <c r="AF41" s="19" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="AG41" s="46"/>
       <c r="AH41" s="19" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
-    <row r="42" spans="2:34" ht="69">
+    <row r="42" spans="2:34" ht="72">
       <c r="B42" s="16">
         <v>8770</v>
       </c>
@@ -11728,59 +11741,59 @@
         <v>46218</v>
       </c>
       <c r="Q42" s="32" t="s">
+        <v>679</v>
+      </c>
+      <c r="R42" s="32" t="s">
         <v>680</v>
       </c>
-      <c r="R42" s="32" t="s">
-        <v>681</v>
-      </c>
       <c r="S42" s="32" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="T42" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U42" s="19" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="V42" s="19" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="W42" s="19" t="s">
+        <v>528</v>
+      </c>
+      <c r="X42" s="19" t="s">
         <v>529</v>
-      </c>
-      <c r="X42" s="19" t="s">
-        <v>530</v>
       </c>
       <c r="Y42" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z42" s="19" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="AA42" s="19" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="AB42" s="19" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="AC42" s="19" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AD42" s="19" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AE42" s="19" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AF42" s="19" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="AG42" s="77"/>
       <c r="AH42" s="19" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
-    <row r="43" spans="2:34" ht="69">
+    <row r="43" spans="2:34" ht="72">
       <c r="B43" s="23">
         <v>73030</v>
       </c>
@@ -11827,59 +11840,59 @@
         <v>46218</v>
       </c>
       <c r="Q43" s="32" t="s">
+        <v>681</v>
+      </c>
+      <c r="R43" s="32" t="s">
         <v>682</v>
       </c>
-      <c r="R43" s="32" t="s">
-        <v>683</v>
-      </c>
       <c r="S43" s="32" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="T43" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U43" s="19" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="V43" s="32" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="W43" s="19" t="s">
+        <v>514</v>
+      </c>
+      <c r="X43" s="19" t="s">
         <v>515</v>
-      </c>
-      <c r="X43" s="19" t="s">
-        <v>516</v>
       </c>
       <c r="Y43" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z43" s="19" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="AA43" s="19" t="s">
+        <v>524</v>
+      </c>
+      <c r="AB43" s="19" t="s">
+        <v>522</v>
+      </c>
+      <c r="AC43" s="19" t="s">
+        <v>565</v>
+      </c>
+      <c r="AD43" s="19" t="s">
+        <v>535</v>
+      </c>
+      <c r="AE43" s="19" t="s">
         <v>525</v>
       </c>
-      <c r="AB43" s="19" t="s">
-        <v>523</v>
-      </c>
-      <c r="AC43" s="19" t="s">
-        <v>566</v>
-      </c>
-      <c r="AD43" s="19" t="s">
-        <v>536</v>
-      </c>
-      <c r="AE43" s="19" t="s">
+      <c r="AF43" s="19" t="s">
         <v>526</v>
-      </c>
-      <c r="AF43" s="19" t="s">
-        <v>527</v>
       </c>
       <c r="AG43" s="77"/>
       <c r="AH43" s="19" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
-    <row r="44" spans="2:34" ht="57.5">
+    <row r="44" spans="2:34" ht="72">
       <c r="B44" s="16">
         <v>73483</v>
       </c>
@@ -11926,28 +11939,28 @@
         <v>46240</v>
       </c>
       <c r="Q44" s="32" t="s">
+        <v>540</v>
+      </c>
+      <c r="R44" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="R44" s="32" t="s">
-        <v>542</v>
-      </c>
       <c r="S44" s="73" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="T44" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U44" s="19" t="s">
+        <v>542</v>
+      </c>
+      <c r="V44" s="32" t="s">
         <v>543</v>
       </c>
-      <c r="V44" s="32" t="s">
-        <v>544</v>
-      </c>
       <c r="W44" s="19" t="s">
+        <v>559</v>
+      </c>
+      <c r="X44" s="19" t="s">
         <v>560</v>
-      </c>
-      <c r="X44" s="19" t="s">
-        <v>561</v>
       </c>
       <c r="Y44" s="64" t="s">
         <v>174</v>
@@ -11956,29 +11969,29 @@
         <v>174</v>
       </c>
       <c r="AA44" s="19" t="s">
+        <v>553</v>
+      </c>
+      <c r="AB44" s="19" t="s">
+        <v>550</v>
+      </c>
+      <c r="AC44" s="63" t="s">
         <v>554</v>
       </c>
-      <c r="AB44" s="19" t="s">
-        <v>551</v>
-      </c>
-      <c r="AC44" s="63" t="s">
+      <c r="AD44" s="19" t="s">
+        <v>562</v>
+      </c>
+      <c r="AE44" s="19" t="s">
         <v>555</v>
       </c>
-      <c r="AD44" s="19" t="s">
-        <v>563</v>
-      </c>
-      <c r="AE44" s="19" t="s">
+      <c r="AF44" s="63" t="s">
         <v>556</v>
-      </c>
-      <c r="AF44" s="63" t="s">
-        <v>557</v>
       </c>
       <c r="AG44" s="77"/>
       <c r="AH44" s="19" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
-    <row r="45" spans="2:34" ht="57.5">
+    <row r="45" spans="2:34" ht="60">
       <c r="B45" s="16">
         <v>73563</v>
       </c>
@@ -12025,28 +12038,28 @@
         <v>46240</v>
       </c>
       <c r="Q45" s="32" t="s">
+        <v>545</v>
+      </c>
+      <c r="R45" s="32" t="s">
         <v>546</v>
       </c>
-      <c r="R45" s="32" t="s">
-        <v>547</v>
-      </c>
       <c r="S45" s="73" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="T45" s="64" t="s">
         <v>174</v>
       </c>
       <c r="U45" s="19" t="s">
+        <v>557</v>
+      </c>
+      <c r="V45" s="32" t="s">
+        <v>544</v>
+      </c>
+      <c r="W45" s="19" t="s">
         <v>558</v>
       </c>
-      <c r="V45" s="32" t="s">
-        <v>545</v>
-      </c>
-      <c r="W45" s="19" t="s">
-        <v>559</v>
-      </c>
       <c r="X45" s="19" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="Y45" s="64" t="s">
         <v>174</v>
@@ -12055,29 +12068,29 @@
         <v>174</v>
       </c>
       <c r="AA45" s="19" t="s">
+        <v>577</v>
+      </c>
+      <c r="AB45" s="19" t="s">
+        <v>551</v>
+      </c>
+      <c r="AC45" s="63" t="s">
+        <v>552</v>
+      </c>
+      <c r="AD45" s="19" t="s">
         <v>578</v>
       </c>
-      <c r="AB45" s="19" t="s">
-        <v>552</v>
-      </c>
-      <c r="AC45" s="63" t="s">
-        <v>553</v>
-      </c>
-      <c r="AD45" s="19" t="s">
+      <c r="AE45" s="19" t="s">
         <v>579</v>
       </c>
-      <c r="AE45" s="19" t="s">
-        <v>580</v>
-      </c>
       <c r="AF45" s="63" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="AG45" s="77"/>
       <c r="AH45" s="19" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
-    <row r="46" spans="2:34" ht="69">
+    <row r="46" spans="2:34" ht="72">
       <c r="B46" s="16">
         <v>23417</v>
       </c>
@@ -12124,26 +12137,26 @@
         <v>46262</v>
       </c>
       <c r="Q46" s="32" t="s">
+        <v>581</v>
+      </c>
+      <c r="R46" s="32" t="s">
         <v>582</v>
       </c>
-      <c r="R46" s="32" t="s">
-        <v>583</v>
-      </c>
       <c r="S46" s="32" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="T46" s="73"/>
       <c r="U46" s="19" t="s">
+        <v>568</v>
+      </c>
+      <c r="V46" s="32" t="s">
         <v>569</v>
       </c>
-      <c r="V46" s="32" t="s">
+      <c r="W46" s="19" t="s">
         <v>570</v>
       </c>
-      <c r="W46" s="19" t="s">
+      <c r="X46" s="19" t="s">
         <v>571</v>
-      </c>
-      <c r="X46" s="19" t="s">
-        <v>572</v>
       </c>
       <c r="Y46" s="64" t="s">
         <v>174</v>
@@ -12152,29 +12165,29 @@
         <v>174</v>
       </c>
       <c r="AA46" s="19" t="s">
+        <v>572</v>
+      </c>
+      <c r="AB46" s="19" t="s">
+        <v>567</v>
+      </c>
+      <c r="AC46" s="63" t="s">
+        <v>580</v>
+      </c>
+      <c r="AD46" s="19" t="s">
         <v>573</v>
       </c>
-      <c r="AB46" s="19" t="s">
-        <v>568</v>
-      </c>
-      <c r="AC46" s="63" t="s">
-        <v>581</v>
-      </c>
-      <c r="AD46" s="19" t="s">
+      <c r="AE46" s="19" t="s">
         <v>574</v>
       </c>
-      <c r="AE46" s="19" t="s">
+      <c r="AF46" s="63" t="s">
         <v>575</v>
-      </c>
-      <c r="AF46" s="63" t="s">
-        <v>576</v>
       </c>
       <c r="AG46" s="77"/>
       <c r="AH46" s="19" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
-    <row r="47" spans="2:34" ht="92">
+    <row r="47" spans="2:34" ht="96">
       <c r="B47" s="16">
         <v>18150</v>
       </c>
@@ -12221,54 +12234,54 @@
         <v>46275</v>
       </c>
       <c r="Q47" s="32" t="s">
+        <v>685</v>
+      </c>
+      <c r="R47" s="32" t="s">
         <v>686</v>
       </c>
-      <c r="R47" s="32" t="s">
+      <c r="S47" s="32" t="s">
         <v>687</v>
-      </c>
-      <c r="S47" s="32" t="s">
-        <v>688</v>
       </c>
       <c r="T47" s="80"/>
       <c r="U47" s="19" t="s">
+        <v>697</v>
+      </c>
+      <c r="V47" s="32" t="s">
         <v>698</v>
       </c>
-      <c r="V47" s="32" t="s">
+      <c r="W47" s="19" t="s">
         <v>699</v>
       </c>
-      <c r="W47" s="19" t="s">
+      <c r="X47" s="19" t="s">
         <v>700</v>
-      </c>
-      <c r="X47" s="19" t="s">
-        <v>701</v>
       </c>
       <c r="Y47" s="64" t="s">
         <v>174</v>
       </c>
       <c r="Z47" s="19" t="s">
+        <v>701</v>
+      </c>
+      <c r="AA47" s="19" t="s">
         <v>702</v>
       </c>
-      <c r="AA47" s="19" t="s">
+      <c r="AB47" s="19" t="s">
+        <v>694</v>
+      </c>
+      <c r="AC47" s="63" t="s">
+        <v>695</v>
+      </c>
+      <c r="AD47" s="63" t="s">
+        <v>696</v>
+      </c>
+      <c r="AE47" s="19" t="s">
         <v>703</v>
       </c>
-      <c r="AB47" s="19" t="s">
-        <v>695</v>
-      </c>
-      <c r="AC47" s="63" t="s">
-        <v>696</v>
-      </c>
-      <c r="AD47" s="63" t="s">
-        <v>697</v>
-      </c>
-      <c r="AE47" s="19" t="s">
+      <c r="AF47" s="63" t="s">
         <v>704</v>
-      </c>
-      <c r="AF47" s="63" t="s">
-        <v>705</v>
       </c>
       <c r="AG47" s="77"/>
       <c r="AH47" s="19" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="48" spans="2:34" ht="42.75" customHeight="1">
@@ -12318,26 +12331,26 @@
         <v>46286</v>
       </c>
       <c r="Q48" s="32" t="s">
+        <v>688</v>
+      </c>
+      <c r="R48" s="32" t="s">
         <v>689</v>
       </c>
-      <c r="R48" s="32" t="s">
+      <c r="S48" s="32" t="s">
         <v>690</v>
-      </c>
-      <c r="S48" s="32" t="s">
-        <v>691</v>
       </c>
       <c r="T48" s="80"/>
       <c r="U48" s="19" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="V48" s="32" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="W48" s="19" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="X48" s="19" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="Y48" s="64" t="s">
         <v>174</v>
@@ -12346,26 +12359,26 @@
         <v>174</v>
       </c>
       <c r="AA48" s="63" t="s">
+        <v>705</v>
+      </c>
+      <c r="AB48" s="19" t="s">
         <v>706</v>
       </c>
-      <c r="AB48" s="19" t="s">
+      <c r="AC48" s="63" t="s">
         <v>707</v>
       </c>
-      <c r="AC48" s="63" t="s">
+      <c r="AD48" s="63" t="s">
         <v>708</v>
       </c>
-      <c r="AD48" s="63" t="s">
-        <v>709</v>
-      </c>
       <c r="AE48" s="19" t="s">
+        <v>711</v>
+      </c>
+      <c r="AF48" s="63" t="s">
         <v>712</v>
-      </c>
-      <c r="AF48" s="63" t="s">
-        <v>713</v>
       </c>
       <c r="AG48" s="77"/>
       <c r="AH48" s="19" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="49" spans="2:34" ht="42.75" customHeight="1">
@@ -12415,26 +12428,26 @@
         <v>46286</v>
       </c>
       <c r="Q49" s="32" t="s">
+        <v>692</v>
+      </c>
+      <c r="R49" s="32" t="s">
         <v>693</v>
       </c>
-      <c r="R49" s="32" t="s">
-        <v>694</v>
-      </c>
       <c r="S49" s="32" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="T49" s="80"/>
       <c r="U49" s="19" t="s">
+        <v>717</v>
+      </c>
+      <c r="V49" s="32" t="s">
         <v>718</v>
       </c>
-      <c r="V49" s="32" t="s">
+      <c r="W49" s="19" t="s">
         <v>719</v>
       </c>
-      <c r="W49" s="19" t="s">
+      <c r="X49" s="19" t="s">
         <v>720</v>
-      </c>
-      <c r="X49" s="19" t="s">
-        <v>721</v>
       </c>
       <c r="Y49" s="64" t="s">
         <v>174</v>
@@ -12443,26 +12456,26 @@
         <v>174</v>
       </c>
       <c r="AA49" s="63" t="s">
+        <v>713</v>
+      </c>
+      <c r="AB49" s="19" t="s">
         <v>714</v>
       </c>
-      <c r="AB49" s="19" t="s">
+      <c r="AC49" s="63" t="s">
         <v>715</v>
       </c>
-      <c r="AC49" s="63" t="s">
+      <c r="AD49" s="63" t="s">
         <v>716</v>
       </c>
-      <c r="AD49" s="63" t="s">
-        <v>717</v>
-      </c>
       <c r="AE49" s="19" t="s">
+        <v>721</v>
+      </c>
+      <c r="AF49" s="63" t="s">
         <v>722</v>
-      </c>
-      <c r="AF49" s="63" t="s">
-        <v>723</v>
       </c>
       <c r="AG49" s="77"/>
       <c r="AH49" s="19" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="50" spans="2:34" ht="49.5" customHeight="1">
@@ -12533,22 +12546,22 @@
       <c r="O51" s="20"/>
       <c r="P51" s="20"/>
       <c r="Q51" s="32" t="s">
+        <v>683</v>
+      </c>
+      <c r="R51" s="32" t="s">
         <v>684</v>
-      </c>
-      <c r="R51" s="32" t="s">
-        <v>685</v>
       </c>
       <c r="S51" s="18"/>
       <c r="T51" s="18"/>
       <c r="U51" s="32"/>
       <c r="V51" s="32" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="W51" s="19" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="X51" s="19" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="Y51" s="19"/>
       <c r="Z51" s="46"/>
@@ -12557,7 +12570,7 @@
       <c r="AC51" s="46"/>
       <c r="AD51" s="46"/>
       <c r="AE51" s="46" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AF51" s="46"/>
       <c r="AG51" s="46"/>
@@ -14670,16 +14683,47 @@
     </row>
   </sheetData>
   <phoneticPr fontId="12" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="AA11" r:id="rId1" display="https://mailuis.sharepoint.com/:f:/s/INTERVENTORIA/IgBscwwdYL2eT4Rok2j9HkE3AZKPFhZI1j2dAJfLL5f47KQ?e=XF4bNQ" xr:uid="{9B6FDFA9-F412-43C4-9A6F-FBD37FC11736}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creador>
+    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010000E8DC80C026CA4DA909D73C325EE4F6" ma:contentTypeVersion="22" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="540ba7b4ebff7c81ec83231b347cbaa0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xmlns:ns3="a9ff745a-43b9-4806-bec3-e08ef3e383fc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45c75a4f992fb922f736f24948a438b4" ns2:_="" ns3:_="">
     <xsd:import namespace="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
@@ -14946,35 +14990,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
+    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creador>
-    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85AD5D61-E9C3-4156-A82C-31BB302CC72C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14991,29 +15032,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
-    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
NOMBRE ARCHIVO COL S
</commit_message>
<xml_diff>
--- a/Tablero_control_General_Instalación_180926.xlsx
+++ b/Tablero_control_General_Instalación_180926.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria.pardo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.garcia\Desktop\github\linea_tiempo_fase_instalacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD35F06-EB3B-4285-864A-56825F7A41F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0451166-88D9-482A-AECB-9896B1E3EFBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Reporte semanal" sheetId="2" r:id="rId1"/>
@@ -2341,11 +2341,6 @@
 NOMBRE ARCHIVO: ACTA DE INICIO CORMAGDALENA LA GLORIA</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\13667_San Martín de Loba (Bolívar)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
-NOMBRE DE ARCHIVO: ACTA DE INICIO CORMAGDALENA SAN MARTIN DE LOBA
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\13780_Talaigua Nuevo (Bolívar)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
 NOMBRE ARCHIVO: ACTA DE INICIO CORMAGDALENA TALAIGUA NUEVO
 </t>
@@ -2357,15 +2352,6 @@
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\13600_Río Viejo (Bolívar)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
 NOMBRE ARCHIVO: ACTA DE INICIO CORMAGDALENA RIO VIEJO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\13300_Hatillo de Loba (Bolívar)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
-NOMBRE DE ARCHIVO: ACTA DE INICIO CORMAGDALENA HATILLO DE LOBA
-</t>
-  </si>
-  <si>
-    <t>Documentos\Documentos Tecnicos\Documentos por sitio\47720_Santa Bárbara de Pinto (Magdalena)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
-NOMBRE DE ARCHIVO: ACTA DE INICIO CORMAGDALENA SANTA BÁRBARA DE PINTO</t>
   </si>
   <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5579_Puerto Berrío (Antioquia)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
@@ -3080,6 +3066,20 @@
   </si>
   <si>
     <t>PUERTO WILCHES 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\13667_San Martín de Loba (Bolívar)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
+NOMBRE ARCHIVO: ACTA DE INICIO CORMAGDALENA SAN MARTIN DE LOBA
+</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\47720_Santa Bárbara de Pinto (Magdalena)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
+NOMBRE ARCHIVO: ACTA DE INICIO CORMAGDALENA SANTA BÁRBARA DE PINTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\13300_Hatillo de Loba (Bolívar)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
+NOMBRE ARCHIVO: ACTA DE INICIO CORMAGDALENA HATILLO DE LOBA
+</t>
   </si>
 </sst>
 </file>
@@ -5023,8 +5023,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="463776" y="0"/>
-          <a:ext cx="11315474" cy="1245054"/>
+          <a:off x="455838" y="0"/>
+          <a:ext cx="10775725" cy="1292679"/>
           <a:chOff x="748618" y="-95891"/>
           <a:chExt cx="1536898" cy="1592199"/>
         </a:xfrm>
@@ -5445,8 +5445,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="160112" y="300831"/>
-          <a:ext cx="66959388" cy="1084351"/>
+          <a:off x="163287" y="313531"/>
+          <a:ext cx="63876463" cy="1179601"/>
           <a:chOff x="597738" y="179718"/>
           <a:chExt cx="17343644" cy="1316590"/>
         </a:xfrm>
@@ -6219,27 +6219,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{875B28C0-B948-4D48-BD54-8EF7F295132D}">
   <dimension ref="B8:R51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.90625" customWidth="1"/>
-    <col min="2" max="2" width="7.08984375" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" customWidth="1"/>
-    <col min="4" max="4" width="7.453125" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.08984375" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" customWidth="1"/>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="11" width="10.08984375" customWidth="1"/>
-    <col min="12" max="12" width="10.90625" customWidth="1"/>
-    <col min="13" max="15" width="10.08984375" customWidth="1"/>
+    <col min="10" max="11" width="10.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="13" max="15" width="10.140625" customWidth="1"/>
     <col min="16" max="17" width="11" customWidth="1"/>
-    <col min="18" max="18" width="10.08984375" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="9.54296875" customWidth="1"/>
+    <col min="18" max="18" width="10.140625" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="2:18" ht="16.5" customHeight="1"/>
-    <row r="9" spans="2:18" ht="31.5">
+    <row r="9" spans="2:18" ht="45">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
@@ -6303,7 +6303,7 @@
         <v>64</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>4</v>
@@ -7221,7 +7221,7 @@
       </c>
       <c r="R26" s="8"/>
     </row>
-    <row r="27" spans="2:18" ht="26.4" customHeight="1">
+    <row r="27" spans="2:18" ht="26.45" customHeight="1">
       <c r="B27" s="2">
         <v>18</v>
       </c>
@@ -7232,7 +7232,7 @@
         <v>292</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>4</v>
@@ -7273,7 +7273,7 @@
       </c>
       <c r="R27" s="8"/>
     </row>
-    <row r="28" spans="2:18" ht="26.4" customHeight="1">
+    <row r="28" spans="2:18" ht="26.45" customHeight="1">
       <c r="B28" s="2">
         <v>19</v>
       </c>
@@ -7324,7 +7324,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="2:18" ht="26.4" customHeight="1">
+    <row r="29" spans="2:18" ht="26.45" customHeight="1">
       <c r="B29" s="2">
         <v>20</v>
       </c>
@@ -7426,7 +7426,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="2:18" ht="23.4" customHeight="1">
+    <row r="31" spans="2:18" ht="23.45" customHeight="1">
       <c r="B31" s="2">
         <v>22</v>
       </c>
@@ -7477,7 +7477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="2:18" ht="26.4" customHeight="1">
+    <row r="32" spans="2:18" ht="26.45" customHeight="1">
       <c r="B32" s="2">
         <v>23</v>
       </c>
@@ -7528,7 +7528,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="2:17" ht="26.15" customHeight="1">
+    <row r="33" spans="2:17" ht="26.1" customHeight="1">
       <c r="B33" s="2">
         <v>24</v>
       </c>
@@ -7579,7 +7579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="2:17" ht="26.15" customHeight="1">
+    <row r="34" spans="2:17" ht="26.1" customHeight="1">
       <c r="B34" s="2">
         <v>25</v>
       </c>
@@ -7630,7 +7630,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="2:17" ht="26.15" customHeight="1">
+    <row r="35" spans="2:17" ht="26.1" customHeight="1">
       <c r="B35" s="2">
         <v>26</v>
       </c>
@@ -7681,7 +7681,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="2:17" ht="26.15" customHeight="1">
+    <row r="36" spans="2:17" ht="26.1" customHeight="1">
       <c r="B36" s="2">
         <v>27</v>
       </c>
@@ -7732,7 +7732,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="2:17" ht="26.15" customHeight="1">
+    <row r="37" spans="2:17" ht="26.1" customHeight="1">
       <c r="B37" s="2">
         <v>28</v>
       </c>
@@ -7783,7 +7783,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="2:17" ht="26.15" customHeight="1">
+    <row r="38" spans="2:17" ht="26.1" customHeight="1">
       <c r="B38" s="2">
         <v>29</v>
       </c>
@@ -7834,7 +7834,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="2:17" ht="26.15" customHeight="1">
+    <row r="39" spans="2:17" ht="26.1" customHeight="1">
       <c r="B39" s="2">
         <v>30</v>
       </c>
@@ -7885,7 +7885,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="2:17" ht="26.15" customHeight="1">
+    <row r="40" spans="2:17" ht="26.1" customHeight="1">
       <c r="B40" s="2">
         <v>31</v>
       </c>
@@ -7936,7 +7936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="2:17" ht="26.15" customHeight="1">
+    <row r="41" spans="2:17" ht="26.1" customHeight="1">
       <c r="B41" s="2">
         <v>32</v>
       </c>
@@ -7987,7 +7987,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="2:17" ht="26.15" customHeight="1">
+    <row r="42" spans="2:17" ht="26.1" customHeight="1">
       <c r="B42" s="2">
         <v>33</v>
       </c>
@@ -8038,7 +8038,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="2:17" ht="26.15" customHeight="1">
+    <row r="43" spans="2:17" ht="26.1" customHeight="1">
       <c r="B43" s="2">
         <v>34</v>
       </c>
@@ -8089,7 +8089,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:17" ht="26.15" customHeight="1">
+    <row r="44" spans="2:17" ht="26.1" customHeight="1">
       <c r="B44" s="2">
         <v>35</v>
       </c>
@@ -8140,7 +8140,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="2:17" ht="26.15" customHeight="1">
+    <row r="45" spans="2:17" ht="26.1" customHeight="1">
       <c r="B45" s="2">
         <v>36</v>
       </c>
@@ -8189,7 +8189,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:17" ht="26.15" customHeight="1">
+    <row r="46" spans="2:17" ht="26.1" customHeight="1">
       <c r="B46" s="2">
         <v>37</v>
       </c>
@@ -8238,7 +8238,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="2:17" ht="26.15" customHeight="1">
+    <row r="47" spans="2:17" ht="26.1" customHeight="1">
       <c r="B47" s="2">
         <v>38</v>
       </c>
@@ -8287,7 +8287,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="2:17" ht="26.15" customHeight="1">
+    <row r="48" spans="2:17" ht="26.1" customHeight="1">
       <c r="B48" s="2">
         <v>39</v>
       </c>
@@ -8336,7 +8336,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="2:17" ht="26.15" customHeight="1">
+    <row r="49" spans="2:17" ht="26.1" customHeight="1">
       <c r="B49" s="2">
         <v>40</v>
       </c>
@@ -8368,7 +8368,7 @@
       <c r="P49" s="65"/>
       <c r="Q49" s="56"/>
     </row>
-    <row r="50" spans="2:17" ht="26.15" customHeight="1">
+    <row r="50" spans="2:17" ht="26.1" customHeight="1">
       <c r="B50" s="2"/>
       <c r="C50" s="2">
         <v>5659</v>
@@ -8394,7 +8394,7 @@
       <c r="P50" s="65"/>
       <c r="Q50" s="56"/>
     </row>
-    <row r="51" spans="2:17" ht="24.65" customHeight="1">
+    <row r="51" spans="2:17" ht="24.6" customHeight="1">
       <c r="B51" s="74"/>
       <c r="C51" s="2">
         <v>13650</v>
@@ -8438,35 +8438,35 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C015DEDA-282C-4A92-9944-4B7B289C369E}">
   <dimension ref="B9:AI100"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.08984375" style="11" customWidth="1"/>
-    <col min="2" max="2" width="18.90625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="18.90625" style="11" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="18.90625" style="11" customWidth="1"/>
-    <col min="5" max="5" width="15.90625" style="11" customWidth="1"/>
-    <col min="6" max="6" width="23.08984375" style="11" customWidth="1"/>
-    <col min="7" max="8" width="18.90625" style="11" customWidth="1"/>
-    <col min="9" max="9" width="23.90625" style="11" customWidth="1"/>
-    <col min="10" max="12" width="22.90625" style="11" customWidth="1"/>
-    <col min="13" max="13" width="25.90625" style="11" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" style="11" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" style="11" customWidth="1"/>
+    <col min="7" max="8" width="18.85546875" style="11" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" style="11" customWidth="1"/>
+    <col min="10" max="12" width="22.85546875" style="11" customWidth="1"/>
+    <col min="13" max="13" width="25.85546875" style="11" customWidth="1"/>
     <col min="14" max="15" width="29" style="11" customWidth="1"/>
-    <col min="16" max="16" width="27.08984375" style="11" customWidth="1"/>
+    <col min="16" max="16" width="27.140625" style="11" customWidth="1"/>
     <col min="17" max="17" width="80" style="11" customWidth="1"/>
-    <col min="18" max="18" width="67.90625" style="11" customWidth="1"/>
-    <col min="19" max="20" width="63.90625" style="11" customWidth="1"/>
-    <col min="21" max="21" width="63.08984375" style="11" customWidth="1"/>
+    <col min="18" max="18" width="67.85546875" style="11" customWidth="1"/>
+    <col min="19" max="20" width="63.85546875" style="11" customWidth="1"/>
+    <col min="21" max="21" width="63.140625" style="11" customWidth="1"/>
     <col min="22" max="22" width="73" style="11" customWidth="1"/>
-    <col min="23" max="23" width="75.08984375" style="11" customWidth="1"/>
-    <col min="24" max="24" width="79.453125" style="11" customWidth="1"/>
+    <col min="23" max="23" width="75.140625" style="11" customWidth="1"/>
+    <col min="24" max="24" width="79.42578125" style="11" customWidth="1"/>
     <col min="25" max="25" width="71" style="11" customWidth="1"/>
-    <col min="26" max="28" width="71.90625" style="11" customWidth="1"/>
-    <col min="29" max="29" width="74.08984375" style="11" customWidth="1"/>
-    <col min="30" max="30" width="62.36328125" style="11" customWidth="1"/>
-    <col min="31" max="31" width="64.08984375" style="11" customWidth="1"/>
-    <col min="32" max="32" width="83.90625" style="11" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="74.08984375" style="11" customWidth="1"/>
-    <col min="34" max="16384" width="11.453125" style="11"/>
+    <col min="26" max="28" width="71.85546875" style="11" customWidth="1"/>
+    <col min="29" max="29" width="74.140625" style="11" customWidth="1"/>
+    <col min="30" max="30" width="62.42578125" style="11" customWidth="1"/>
+    <col min="31" max="31" width="64.140625" style="11" customWidth="1"/>
+    <col min="32" max="32" width="83.85546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="74.140625" style="11" customWidth="1"/>
+    <col min="34" max="16384" width="11.42578125" style="11"/>
   </cols>
   <sheetData>
     <row r="9" spans="2:34" s="10" customFormat="1">
@@ -8576,7 +8576,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="11" spans="2:34" ht="145">
+    <row r="11" spans="2:34" ht="165">
       <c r="B11" s="31">
         <v>68575</v>
       </c>
@@ -8590,7 +8590,7 @@
         <v>64</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="G11" s="17" t="s">
         <v>4</v>
@@ -8627,47 +8627,47 @@
       <c r="S11" s="69"/>
       <c r="T11" s="69"/>
       <c r="U11" s="78" t="s">
+        <v>709</v>
+      </c>
+      <c r="V11" s="78" t="s">
+        <v>710</v>
+      </c>
+      <c r="W11" s="78" t="s">
+        <v>711</v>
+      </c>
+      <c r="X11" s="78" t="s">
         <v>712</v>
-      </c>
-      <c r="V11" s="78" t="s">
-        <v>713</v>
-      </c>
-      <c r="W11" s="78" t="s">
-        <v>714</v>
-      </c>
-      <c r="X11" s="78" t="s">
-        <v>715</v>
       </c>
       <c r="Y11" s="78" t="s">
         <v>129</v>
       </c>
       <c r="Z11" s="78" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="AA11" s="78" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="AB11" s="19" t="s">
         <v>136</v>
       </c>
       <c r="AC11" s="78" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="AD11" s="78" t="s">
+        <v>715</v>
+      </c>
+      <c r="AE11" s="78" t="s">
+        <v>707</v>
+      </c>
+      <c r="AF11" s="78" t="s">
         <v>718</v>
       </c>
-      <c r="AE11" s="78" t="s">
-        <v>710</v>
-      </c>
-      <c r="AF11" s="78" t="s">
-        <v>721</v>
-      </c>
       <c r="AG11" s="78" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="AH11" s="10"/>
     </row>
-    <row r="12" spans="2:34" ht="130.5">
+    <row r="12" spans="2:34" ht="135">
       <c r="B12" s="16">
         <v>13442</v>
       </c>
@@ -8714,10 +8714,10 @@
         <v>45905</v>
       </c>
       <c r="Q12" s="78" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="R12" s="78" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="S12" s="78" t="s">
         <v>561</v>
@@ -8744,7 +8744,7 @@
         <v>151</v>
       </c>
       <c r="AA12" s="78" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="AB12" s="19" t="s">
         <v>152</v>
@@ -8753,7 +8753,7 @@
         <v>153</v>
       </c>
       <c r="AD12" s="78" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="AE12" s="78" t="s">
         <v>155</v>
@@ -8765,7 +8765,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="13" spans="2:34" ht="159.5">
+    <row r="13" spans="2:34" ht="165">
       <c r="B13" s="16">
         <v>47161</v>
       </c>
@@ -8812,10 +8812,10 @@
         <v>45908</v>
       </c>
       <c r="Q13" s="78" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="R13" s="78" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="S13" s="78" t="s">
         <v>560</v>
@@ -8863,7 +8863,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="14" spans="2:34" ht="101.5">
+    <row r="14" spans="2:34" ht="105">
       <c r="B14" s="16">
         <v>47555</v>
       </c>
@@ -8910,10 +8910,10 @@
         <v>45933</v>
       </c>
       <c r="Q14" s="78" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="R14" s="78" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="S14" s="78" t="s">
         <v>558</v>
@@ -8952,7 +8952,7 @@
         <v>167</v>
       </c>
       <c r="AE14" s="78" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="AF14" s="78" t="s">
         <v>170</v>
@@ -8961,7 +8961,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="15" spans="2:34" ht="87">
+    <row r="15" spans="2:34" ht="105">
       <c r="B15" s="16">
         <v>47692</v>
       </c>
@@ -9008,10 +9008,10 @@
         <v>45933</v>
       </c>
       <c r="Q15" s="78" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="R15" s="78" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="S15" s="78" t="s">
         <v>559</v>
@@ -9059,7 +9059,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="16" spans="2:34" ht="116">
+    <row r="16" spans="2:34" ht="120">
       <c r="B16" s="16">
         <v>47745</v>
       </c>
@@ -9106,10 +9106,10 @@
         <v>45985</v>
       </c>
       <c r="Q16" s="78" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="R16" s="78" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="S16" s="78" t="s">
         <v>562</v>
@@ -9157,7 +9157,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="17" spans="2:35" ht="87">
+    <row r="17" spans="2:35" ht="90">
       <c r="B17" s="16">
         <v>73275</v>
       </c>
@@ -9204,10 +9204,10 @@
         <v>45994</v>
       </c>
       <c r="Q17" s="78" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="R17" s="78" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="S17" s="78" t="s">
         <v>563</v>
@@ -9255,7 +9255,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="18" spans="2:35" ht="87">
+    <row r="18" spans="2:35" ht="90">
       <c r="B18" s="16">
         <v>5591</v>
       </c>
@@ -9302,10 +9302,10 @@
         <v>45996</v>
       </c>
       <c r="Q18" s="78" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="R18" s="78" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="S18" s="78" t="s">
         <v>564</v>
@@ -9353,7 +9353,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" spans="2:35" ht="87">
+    <row r="19" spans="2:35" ht="90">
       <c r="B19" s="16">
         <v>73217</v>
       </c>
@@ -9400,10 +9400,10 @@
         <v>46008</v>
       </c>
       <c r="Q19" s="78" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="R19" s="78" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="S19" s="78" t="s">
         <v>565</v>
@@ -9451,7 +9451,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="20" spans="2:35" ht="116">
+    <row r="20" spans="2:35" ht="120">
       <c r="B20" s="16">
         <v>20295</v>
       </c>
@@ -9498,10 +9498,10 @@
         <v>46011</v>
       </c>
       <c r="Q20" s="78" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="R20" s="78" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="S20" s="78" t="s">
         <v>566</v>
@@ -9549,7 +9549,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="21" spans="2:35" ht="101.5">
+    <row r="21" spans="2:35" ht="120">
       <c r="B21" s="16">
         <v>20787</v>
       </c>
@@ -9596,10 +9596,10 @@
         <v>46008</v>
       </c>
       <c r="Q21" s="78" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="R21" s="78" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="S21" s="78" t="s">
         <v>567</v>
@@ -9647,7 +9647,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="22" spans="2:35" ht="72.5">
+    <row r="22" spans="2:35" ht="75">
       <c r="B22" s="16">
         <v>13248</v>
       </c>
@@ -9694,10 +9694,10 @@
         <v>46014</v>
       </c>
       <c r="Q22" s="78" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="R22" s="78" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="S22" s="78" t="s">
         <v>568</v>
@@ -9745,7 +9745,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="23" spans="2:35" ht="145">
+    <row r="23" spans="2:35" ht="150">
       <c r="B23" s="16">
         <v>13140</v>
       </c>
@@ -9792,13 +9792,13 @@
         <v>46045</v>
       </c>
       <c r="Q23" s="78" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="R23" s="78" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="S23" s="72" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="T23" s="70"/>
       <c r="U23" s="78" t="s">
@@ -9841,7 +9841,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="24" spans="2:35" ht="101.5">
+    <row r="24" spans="2:35" ht="105">
       <c r="B24" s="16">
         <v>70124</v>
       </c>
@@ -9888,10 +9888,10 @@
         <v>46048</v>
       </c>
       <c r="Q24" s="78" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="R24" s="78" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="S24" s="78" t="s">
         <v>569</v>
@@ -9939,7 +9939,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="25" spans="2:35" ht="101.5">
+    <row r="25" spans="2:35" ht="120">
       <c r="B25" s="16">
         <v>70678</v>
       </c>
@@ -9986,10 +9986,10 @@
         <v>46049</v>
       </c>
       <c r="Q25" s="78" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="R25" s="78" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="S25" s="78" t="s">
         <v>570</v>
@@ -10037,7 +10037,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="26" spans="2:35" ht="116">
+    <row r="26" spans="2:35" ht="135">
       <c r="B26" s="16">
         <v>95001</v>
       </c>
@@ -10084,10 +10084,10 @@
         <v>46066</v>
       </c>
       <c r="Q26" s="78" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="R26" s="78" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="S26" s="78" t="s">
         <v>573</v>
@@ -10135,7 +10135,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="27" spans="2:35" ht="116">
+    <row r="27" spans="2:35" ht="135">
       <c r="B27" s="16">
         <v>17495</v>
       </c>
@@ -10182,10 +10182,10 @@
         <v>46069</v>
       </c>
       <c r="Q27" s="78" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="R27" s="78" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="S27" s="78" t="s">
         <v>575</v>
@@ -10233,7 +10233,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="28" spans="2:35" ht="203">
+    <row r="28" spans="2:35" ht="225">
       <c r="B28" s="66">
         <v>68575</v>
       </c>
@@ -10247,7 +10247,7 @@
         <v>60</v>
       </c>
       <c r="F28" s="67" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="G28" s="67" t="s">
         <v>4</v>
@@ -10284,22 +10284,22 @@
       <c r="S28" s="70"/>
       <c r="T28" s="70"/>
       <c r="U28" s="78" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="V28" s="64" t="s">
         <v>163</v>
       </c>
       <c r="W28" s="78" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="X28" s="78" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="Y28" s="64" t="s">
         <v>163</v>
       </c>
       <c r="Z28" s="78" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="AA28" s="78" t="s">
         <v>294</v>
@@ -10311,13 +10311,13 @@
         <v>338</v>
       </c>
       <c r="AD28" s="78" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="AE28" s="78" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="AF28" s="78" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="AG28" s="78" t="s">
         <v>341</v>
@@ -10372,10 +10372,10 @@
         <v>46129</v>
       </c>
       <c r="Q29" s="81" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="R29" s="81" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="S29" s="81" t="s">
         <v>577</v>
@@ -10393,7 +10393,7 @@
         <v>364</v>
       </c>
       <c r="X29" s="78" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="Y29" s="64" t="s">
         <v>163</v>
@@ -10423,7 +10423,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="30" spans="2:35" ht="101.5">
+    <row r="30" spans="2:35" ht="105">
       <c r="B30" s="16">
         <v>13473</v>
       </c>
@@ -10470,10 +10470,10 @@
         <v>46129</v>
       </c>
       <c r="Q30" s="81" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="R30" s="81" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="S30" s="81" t="s">
         <v>578</v>
@@ -10521,7 +10521,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="31" spans="2:35" ht="80.150000000000006" customHeight="1">
+    <row r="31" spans="2:35" ht="80.099999999999994" customHeight="1">
       <c r="B31" s="16">
         <v>8137</v>
       </c>
@@ -10568,10 +10568,10 @@
         <v>46134</v>
       </c>
       <c r="Q31" s="81" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="R31" s="81" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="S31" s="81" t="s">
         <v>579</v>
@@ -10619,7 +10619,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="32" spans="2:35" ht="131.4" customHeight="1">
+    <row r="32" spans="2:35" ht="131.44999999999999" customHeight="1">
       <c r="B32" s="16">
         <v>13188</v>
       </c>
@@ -10666,10 +10666,10 @@
         <v>46135</v>
       </c>
       <c r="Q32" s="81" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="R32" s="81" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="S32" s="81" t="s">
         <v>580</v>
@@ -10717,7 +10717,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="33" spans="2:33" ht="116">
+    <row r="33" spans="2:33" ht="120">
       <c r="B33" s="23">
         <v>8606</v>
       </c>
@@ -10764,10 +10764,10 @@
         <v>46140</v>
       </c>
       <c r="Q33" s="81" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="R33" s="81" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="S33" s="81" t="s">
         <v>581</v>
@@ -10815,7 +10815,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="34" spans="2:33" ht="89.15" customHeight="1">
+    <row r="34" spans="2:33" ht="89.1" customHeight="1">
       <c r="B34" s="31">
         <v>20383</v>
       </c>
@@ -10862,10 +10862,10 @@
         <v>46162</v>
       </c>
       <c r="Q34" s="81" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="R34" s="81" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="S34" s="81" t="s">
         <v>582</v>
@@ -10880,7 +10880,7 @@
         <v>394</v>
       </c>
       <c r="W34" s="78" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="X34" s="78" t="s">
         <v>395</v>
@@ -10913,7 +10913,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="35" spans="2:33" ht="62.4" customHeight="1">
+    <row r="35" spans="2:33" ht="62.45" customHeight="1">
       <c r="B35" s="23">
         <v>13667</v>
       </c>
@@ -10960,13 +10960,13 @@
         <v>46183</v>
       </c>
       <c r="Q35" s="81" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="R35" s="81" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="S35" s="81" t="s">
-        <v>583</v>
+        <v>730</v>
       </c>
       <c r="T35" s="64" t="s">
         <v>163</v>
@@ -11011,7 +11011,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="36" spans="2:33" ht="87">
+    <row r="36" spans="2:33" ht="90">
       <c r="B36" s="16">
         <v>13780</v>
       </c>
@@ -11058,13 +11058,13 @@
         <v>46184</v>
       </c>
       <c r="Q36" s="81" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="R36" s="81" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="S36" s="81" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="T36" s="64" t="s">
         <v>163</v>
@@ -11109,7 +11109,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="37" spans="2:33" ht="101.5">
+    <row r="37" spans="2:33" ht="105">
       <c r="B37" s="16">
         <v>13160</v>
       </c>
@@ -11156,13 +11156,13 @@
         <v>46191</v>
       </c>
       <c r="Q37" s="81" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="R37" s="81" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="S37" s="81" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="T37" s="64" t="s">
         <v>163</v>
@@ -11207,7 +11207,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="38" spans="2:33" ht="84.9" customHeight="1">
+    <row r="38" spans="2:33" ht="84.95" customHeight="1">
       <c r="B38" s="16">
         <v>13600</v>
       </c>
@@ -11254,13 +11254,13 @@
         <v>46192</v>
       </c>
       <c r="Q38" s="81" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="R38" s="81" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="S38" s="81" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="T38" s="64" t="s">
         <v>163</v>
@@ -11305,7 +11305,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="39" spans="2:33" ht="78.900000000000006" customHeight="1">
+    <row r="39" spans="2:33" ht="78.95" customHeight="1">
       <c r="B39" s="16">
         <v>13300</v>
       </c>
@@ -11352,13 +11352,13 @@
         <v>46205</v>
       </c>
       <c r="Q39" s="81" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="R39" s="81" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="S39" s="81" t="s">
-        <v>587</v>
+        <v>732</v>
       </c>
       <c r="T39" s="64" t="s">
         <v>163</v>
@@ -11403,7 +11403,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="40" spans="2:33" ht="101.5">
+    <row r="40" spans="2:33" ht="120">
       <c r="B40" s="16">
         <v>47720</v>
       </c>
@@ -11450,13 +11450,13 @@
         <v>46205</v>
       </c>
       <c r="Q40" s="81" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="R40" s="81" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="S40" s="81" t="s">
-        <v>588</v>
+        <v>731</v>
       </c>
       <c r="T40" s="64" t="s">
         <v>163</v>
@@ -11501,7 +11501,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="41" spans="2:33" ht="69.650000000000006" customHeight="1">
+    <row r="41" spans="2:33" ht="69.599999999999994" customHeight="1">
       <c r="B41" s="16">
         <v>5579</v>
       </c>
@@ -11548,13 +11548,13 @@
         <v>46205</v>
       </c>
       <c r="Q41" s="81" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="R41" s="81" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="S41" s="81" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="T41" s="64" t="s">
         <v>163</v>
@@ -11599,7 +11599,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="42" spans="2:33" ht="87">
+    <row r="42" spans="2:33" ht="90">
       <c r="B42" s="16">
         <v>8770</v>
       </c>
@@ -11646,13 +11646,13 @@
         <v>46218</v>
       </c>
       <c r="Q42" s="81" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="R42" s="81" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="S42" s="81" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="T42" s="64" t="s">
         <v>163</v>
@@ -11694,10 +11694,10 @@
         <v>501</v>
       </c>
       <c r="AG42" s="78" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
     </row>
-    <row r="43" spans="2:33" ht="87">
+    <row r="43" spans="2:33" ht="90">
       <c r="B43" s="23">
         <v>73030</v>
       </c>
@@ -11744,13 +11744,13 @@
         <v>46218</v>
       </c>
       <c r="Q43" s="81" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="R43" s="81" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="S43" s="81" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="T43" s="64" t="s">
         <v>163</v>
@@ -11792,10 +11792,10 @@
         <v>500</v>
       </c>
       <c r="AG43" s="78" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
-    <row r="44" spans="2:33" ht="87">
+    <row r="44" spans="2:33" ht="90">
       <c r="B44" s="16">
         <v>73483</v>
       </c>
@@ -11848,7 +11848,7 @@
         <v>515</v>
       </c>
       <c r="S44" s="72" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="T44" s="64" t="s">
         <v>163</v>
@@ -11890,10 +11890,10 @@
         <v>530</v>
       </c>
       <c r="AG44" s="78" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
     </row>
-    <row r="45" spans="2:33" ht="72.5">
+    <row r="45" spans="2:33" ht="75">
       <c r="B45" s="16">
         <v>73563</v>
       </c>
@@ -11946,7 +11946,7 @@
         <v>520</v>
       </c>
       <c r="S45" s="72" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="T45" s="64" t="s">
         <v>163</v>
@@ -11988,10 +11988,10 @@
         <v>550</v>
       </c>
       <c r="AG45" s="78" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
     </row>
-    <row r="46" spans="2:33" ht="87">
+    <row r="46" spans="2:33" ht="90">
       <c r="B46" s="16">
         <v>23417</v>
       </c>
@@ -12044,7 +12044,7 @@
         <v>556</v>
       </c>
       <c r="S46" s="81" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="T46" s="72"/>
       <c r="U46" s="78" t="s">
@@ -12084,10 +12084,10 @@
         <v>549</v>
       </c>
       <c r="AG46" s="78" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
     </row>
-    <row r="47" spans="2:33" ht="116">
+    <row r="47" spans="2:33" ht="135">
       <c r="B47" s="16">
         <v>18150</v>
       </c>
@@ -12134,56 +12134,56 @@
         <v>46275</v>
       </c>
       <c r="Q47" s="81" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="R47" s="81" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="S47" s="81" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="T47" s="77"/>
       <c r="U47" s="78" t="s">
+        <v>665</v>
+      </c>
+      <c r="V47" s="81" t="s">
+        <v>666</v>
+      </c>
+      <c r="W47" s="78" t="s">
+        <v>667</v>
+      </c>
+      <c r="X47" s="78" t="s">
         <v>668</v>
-      </c>
-      <c r="V47" s="81" t="s">
-        <v>669</v>
-      </c>
-      <c r="W47" s="78" t="s">
-        <v>670</v>
-      </c>
-      <c r="X47" s="78" t="s">
-        <v>671</v>
       </c>
       <c r="Y47" s="64" t="s">
         <v>163</v>
       </c>
       <c r="Z47" s="78" t="s">
+        <v>669</v>
+      </c>
+      <c r="AA47" s="78" t="s">
+        <v>670</v>
+      </c>
+      <c r="AB47" s="19" t="s">
+        <v>663</v>
+      </c>
+      <c r="AC47" s="63" t="s">
+        <v>664</v>
+      </c>
+      <c r="AD47" s="78" t="s">
+        <v>702</v>
+      </c>
+      <c r="AE47" s="78" t="s">
+        <v>671</v>
+      </c>
+      <c r="AF47" s="80" t="s">
         <v>672</v>
       </c>
-      <c r="AA47" s="78" t="s">
-        <v>673</v>
-      </c>
-      <c r="AB47" s="19" t="s">
-        <v>666</v>
-      </c>
-      <c r="AC47" s="63" t="s">
-        <v>667</v>
-      </c>
-      <c r="AD47" s="78" t="s">
-        <v>705</v>
-      </c>
-      <c r="AE47" s="78" t="s">
-        <v>674</v>
-      </c>
-      <c r="AF47" s="80" t="s">
-        <v>675</v>
-      </c>
       <c r="AG47" s="78" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
     </row>
-    <row r="48" spans="2:33" ht="72.5">
+    <row r="48" spans="2:33" ht="75">
       <c r="B48" s="16">
         <v>86568</v>
       </c>
@@ -12230,26 +12230,26 @@
         <v>46286</v>
       </c>
       <c r="Q48" s="81" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="R48" s="81" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="S48" s="81" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="T48" s="77"/>
       <c r="U48" s="78" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="V48" s="81" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="W48" s="78" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="X48" s="78" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="Y48" s="64" t="s">
         <v>163</v>
@@ -12258,25 +12258,25 @@
         <v>163</v>
       </c>
       <c r="AA48" s="80" t="s">
+        <v>673</v>
+      </c>
+      <c r="AB48" s="19" t="s">
+        <v>674</v>
+      </c>
+      <c r="AC48" s="63" t="s">
+        <v>675</v>
+      </c>
+      <c r="AD48" s="80" t="s">
         <v>676</v>
       </c>
-      <c r="AB48" s="19" t="s">
-        <v>677</v>
-      </c>
-      <c r="AC48" s="63" t="s">
-        <v>678</v>
-      </c>
-      <c r="AD48" s="80" t="s">
+      <c r="AE48" s="78" t="s">
         <v>679</v>
       </c>
-      <c r="AE48" s="78" t="s">
-        <v>682</v>
-      </c>
       <c r="AF48" s="80" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="AG48" s="78" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
     </row>
     <row r="49" spans="2:33" ht="42.75" customHeight="1">
@@ -12326,26 +12326,26 @@
         <v>46286</v>
       </c>
       <c r="Q49" s="81" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="R49" s="81" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="S49" s="81" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="T49" s="77"/>
       <c r="U49" s="78" t="s">
+        <v>685</v>
+      </c>
+      <c r="V49" s="81" t="s">
+        <v>686</v>
+      </c>
+      <c r="W49" s="78" t="s">
+        <v>687</v>
+      </c>
+      <c r="X49" s="78" t="s">
         <v>688</v>
-      </c>
-      <c r="V49" s="81" t="s">
-        <v>689</v>
-      </c>
-      <c r="W49" s="78" t="s">
-        <v>690</v>
-      </c>
-      <c r="X49" s="78" t="s">
-        <v>691</v>
       </c>
       <c r="Y49" s="64" t="s">
         <v>163</v>
@@ -12354,25 +12354,25 @@
         <v>163</v>
       </c>
       <c r="AA49" s="80" t="s">
+        <v>681</v>
+      </c>
+      <c r="AB49" s="19" t="s">
+        <v>682</v>
+      </c>
+      <c r="AC49" s="63" t="s">
+        <v>683</v>
+      </c>
+      <c r="AD49" s="80" t="s">
         <v>684</v>
       </c>
-      <c r="AB49" s="19" t="s">
-        <v>685</v>
-      </c>
-      <c r="AC49" s="63" t="s">
-        <v>686</v>
-      </c>
-      <c r="AD49" s="80" t="s">
-        <v>687</v>
-      </c>
       <c r="AE49" s="78" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="AF49" s="80" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="AG49" s="78" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
     </row>
     <row r="50" spans="2:33" ht="49.5" customHeight="1">
@@ -12442,10 +12442,10 @@
       <c r="O51" s="20"/>
       <c r="P51" s="20"/>
       <c r="Q51" s="32" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="R51" s="32" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="S51" s="18"/>
       <c r="T51" s="18"/>
@@ -15060,6 +15060,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creador>
+    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010000E8DC80C026CA4DA909D73C325EE4F6" ma:contentTypeVersion="22" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="540ba7b4ebff7c81ec83231b347cbaa0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xmlns:ns3="a9ff745a-43b9-4806-bec3-e08ef3e383fc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="45c75a4f992fb922f736f24948a438b4" ns2:_="" ns3:_="">
     <xsd:import namespace="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
@@ -15326,35 +15354,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
+    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a9ff745a-43b9-4806-bec3-e08ef3e383fc" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Creador xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creador>
-    <Fechaderecepci_x00f3_n xmlns="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85AD5D61-E9C3-4156-A82C-31BB302CC72C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -15371,29 +15396,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FA9B33A-7157-4A1E-9827-44FA9C375306}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A29D9C3D-7EA4-44AF-A5F6-2789F88411EE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a9ff745a-43b9-4806-bec3-e08ef3e383fc"/>
-    <ds:schemaRef ds:uri="2f8bdde9-d83d-45ad-9698-6e538cb1e8b3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
excel update 16 octubre
</commit_message>
<xml_diff>
--- a/Tablero_control_General_Instalación_180926.xlsx
+++ b/Tablero_control_General_Instalación_180926.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria.pardo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA3456CB-C318-489B-BB07-5ACDEEF12E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19E01D54-FDD7-452B-8F29-F41EAD270872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{AF266DC3-C9DA-44A8-AC5C-80B1432A13E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Reporte semanal" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1069" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="780">
   <si>
     <t>CÓDIGO DIPOLA MUN</t>
   </si>
@@ -1602,9 +1602,6 @@
 NOMBRE ARCHIVO: Acta Capacitacion Río Viejo</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\13780_Talaigua Nuevo (Bolívar)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
 NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_TalaiguaNuevo</t>
   </si>
@@ -1805,12 +1802,6 @@
 NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_Santa_Barbara_de_Pinto</t>
   </si>
   <si>
-    <t>Documentos\Documentos Tecnicos\Documentos por sitio\13650_San Fernando (Bolívar)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
-NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_SanFernando
-Documentos\Documentos Tecnicos\Documentos por sitio\13650_San Fernando (Bolívar)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionSeguimientoInicioInstalacion
-NOMBRE ARCHIVO: ACTA_REUNIÓN_SanFernando_Seguimiento_Instalación</t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\73030_Ambalema (Tolima)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
 NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_Ambalema</t>
   </si>
@@ -1821,10 +1812,6 @@
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\47720_Santa Bárbara de Pinto (Magdalena)\04_Instalación\04_Capacitación
 NOMBRE ARCHIVO: Acta Capacitacion Santa Barbara de Pinto</t>
-  </si>
-  <si>
-    <t>Documentos\Documentos Tecnicos\Documentos por sitio\13650_San Fernando (Bolívar)\04_Instalación\01_SocializaciónInicio\01_Municipio\03_ReunionInicioActividades
-NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_SanFernando</t>
   </si>
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\13473_Morales_LaPalma (Bolívar)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
@@ -2710,10 +2697,6 @@
 NOMBRE ARCHIVO: ACTA ENTREGA FINAL FNTC-560-2024 - MUNICIPIO CARTAGENA DEL CHAIRA</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_BrisasHongKong (Putumayo)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_BrisasHongKong (Putumayo)\04_Instalación\03_SeguimientoCampo\03_CertificacionesCalidadMateriales\01_Anclajes\01_Contratista</t>
   </si>
   <si>
@@ -2721,10 +2704,6 @@
 NOMBRE ARCHIVO:</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_BrisasHongKong (Putumayo)\04_Instalación\03_SeguimientoCampo\02_SeguimientoArmado
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_BrisasHongKong (Putumayo)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
 NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_PuertoAsis_BHK-VGA</t>
   </si>
@@ -2741,19 +2720,11 @@
 NOMBRE ARCHIVO: ACTA ENTREGA FINAL FNTC-560-2024 - MUNICIPIO PUERTO BHK</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\03_SeguimientoCampo\03_CertificacionesCalidadMateriales\01_Anclajes\01_Contratista</t>
   </si>
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\03_SeguimientoCampo\03_CertificacionesCalidadMateriales\01_Anclajes\02_Interventoria
 NOMBRE ARCHIVO:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\03_SeguimientoCampo\02_SeguimientoArmado
-NOMBRE ARCHIVO: </t>
   </si>
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\01_SocializaciónInicio\00_Cronograma
@@ -2982,18 +2953,6 @@
     <t>AQUITANIA 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\01_SocializaciónInicio\02_Comunidad
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\03_SeguimientoCampo\03_CertificacionesCalidadMateriales\01_Anclajes\01_Contratista</t>
   </si>
   <si>
@@ -3005,10 +2964,6 @@
 NOMBRE ARCHIVO: </t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\04_Capacitación
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\05_Entrega
 NOMBRE ARCHIVO: </t>
   </si>
@@ -3029,22 +2984,10 @@
 NOMBRE ARCHIVO:poliza 1083136 - recibo 14278091</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\02_Comunidad
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
 NOMBRE ARCHIVO: </t>
   </si>
   <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\00_Cronograma
 NOMBRE ARCHIVO: PPT - ZARAGOZA</t>
   </si>
@@ -3065,14 +3008,6 @@
   </si>
   <si>
     <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\05_Entrega
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
-NOMBRE ARCHIVO: </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\01_SocializaciónInicio\02_Comunidad
 NOMBRE ARCHIVO: </t>
   </si>
   <si>
@@ -3116,10 +3051,6 @@
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\00_DocumentaciónInicio
 NOMBRE ARCHIVO: 2026S-VBOG-051618 - Dibulla
                   CERTIFICACIÓN VIABILIDAD INSTALACIÓN EMBARCADERO RÍO JERÉZ</t>
-  </si>
-  <si>
-    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
-NOMBRE ARCHIVO: 2026S-VANT-069080 - Zaragoza</t>
   </si>
   <si>
     <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
@@ -3228,6 +3159,128 @@
                                      InformeResistenciaEsclerometroPuertoWilches1
                                     GraficaCorrelacionIndiceReboteEsclerometro
                                     Calibración esclerometro</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
+NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_PuertoLeguizamo</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\01_SocializaciónInicio\02_Comunidad
+NOMBRE ARCHIVO: Acta Socializacion Comunidad PuertoLeguizamo</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\04_Capacitación
+NOMBRE ARCHIVO: Acta Capacitacion Puerto Leguizamo</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\05_Entrega
+NOMBRE ARCHIVO: ACTA ENTREGA FINAL FNTC-560-2024 - MUNICIPIO PUERTO LEGUIZAMO</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\02_AutorizacionesPermisos\01_EspacioPúblico
+NOMBRE ARCHIVO: PERMISO EXP MUNICIPIO DIBULLA
+AUTORIZACIÓN PREDIO COLINDANTE DIBULLA</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
+NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_Dibulla
+ACTA_REUNION_TECNICA_Replanteo_Dibulla</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5659_San Juan de Urabá (Antioquia)\04_Instalación\01_SocializaciónInicio\00_Cronograma
+NOMBRE ARCHIVO: PPT - SAN JUAN DE URABÁ
+CronogramaReinicio_SanJuandeUrabá</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5659_San Juan de Urabá (Antioquia)\04_Instalación\01_SocializaciónInicio\02_Comunidad
+NOMBRE ARCHIVO: Acta Socializacion Comunidad SanJuandeUrabá</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5659_San Juan de Urabá (Antioquia)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
+NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_SanJuandeUraba</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5659_San Juan de Urabá (Antioquia)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
+NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_SanJuandeUrabá
+Comunicación_condiciones_acceso_SanJuandeUraba</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_BrisasHongKong (Putumayo)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
+NOMBRE ARCHIVO: 01_BTC_BrisasHK_130926
+02_BTC_BrisasHK_150926
+03_BTC_BrisasHK_160926</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_BrisasHongKong (Putumayo)\04_Instalación\03_SeguimientoCampo\02_SeguimientoArmado
+NOMBRE ARCHIVO: INST_BrisasHK_180926</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
+NOMBRE ARCHIVO: 01_BTC_PuertoVega_130926
+02_BTC_PuertoVega_140926
+03_BTC_PuertoVega_160926</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\86573_Puerto Leguízamo (Putumayo)\04_Instalación\03_SeguimientoCampo\01_BitacoraObra
+NOMBRE ARCHIVO: 01_BTC_PtoLeguizamo_140926
+02_BTC_PtoLeguizamo_150926
+03_BTC_PtoLeguizamo_160926</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
+NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_Zaragoza</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\02_Comunidad
+NOMBRE ARCHIVO: Acta Socializacion Comunidad Zaragoza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\86568_Puerto Asís_PuertoVega (Putumayo)\04_Instalación\03_SeguimientoCampo\02_SeguimientoArmado
+NOMBRE ARCHIVO: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\00_DocumentaciónInicio\02_ActaInicio
+NOMBRE ARCHIVO: </t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\5895_Zaragoza (Antioquia)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
+NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_Zaragoza</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\01_SocializaciónInicio\02_Comunidad
+NOMBRE ARCHIVO: Acta Socializacion Comunidad Dibulla</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\44090_Dibulla (La Guajira)\04_Instalación\05_Entrega
+NOMBRE ARCHIVO: ACTA ENTREGA FINAL FNTC-560-2024 - MUNICIPIO DIBULLA</t>
+  </si>
+  <si>
+    <t>NO APLICA</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\13650_San Fernando (Bolívar)\04_Instalación\01_SocializaciónInicio\00_Cronograma
+NOMBRE ARCHIVO: PPT - SAN FERNANDO</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\13650_San Fernando (Bolívar)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
+NOMBRE ARCHIVO: ACTA_REUNIÓN_SOCIALIZACIÓN_SanFernando</t>
+  </si>
+  <si>
+    <t>Documentos\Documentos Tecnicos\Documentos por sitio\13650_San Fernando (Bolívar)\04_Instalación\01_SocializaciónInicio\01_Municipio\02_ReunionInicioActividades
+NOMBRE ARCHIVO: ACTA_REUNION_TECNICA_SanFernando
+ACTA_REUNIÓN_SanFernando_Seguimiento_Instalación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\94001_Inírida_Inírida (Guainía)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
+NOMBRE ARCHIVO: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\94001_Inírida_R_ElVenado(Guainía)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
+NOMBRE ARCHIVO: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentos\Documentos Tecnicos\Documentos por sitio\94001_Inírida_R_ElRemanso(Guainía)\04_Instalación\01_SocializaciónInicio\01_Municipio\01_ReunionPreparaciónInstalación
+NOMBRE ARCHIVO: </t>
   </si>
 </sst>
 </file>
@@ -3530,7 +3583,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3725,32 +3778,35 @@
     <xf numFmtId="14" fontId="7" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5566,8 +5622,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="160112" y="300831"/>
-          <a:ext cx="68626263" cy="1084351"/>
+          <a:off x="163287" y="304460"/>
+          <a:ext cx="68843070" cy="1125172"/>
           <a:chOff x="597738" y="179718"/>
           <a:chExt cx="17343644" cy="1316590"/>
         </a:xfrm>
@@ -6377,7 +6433,7 @@
         <v>3</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>126</v>
@@ -6424,13 +6480,13 @@
         <v>64</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H10" s="39">
         <v>45852</v>
@@ -6485,7 +6541,7 @@
         <v>18</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H11" s="39">
         <v>45895</v>
@@ -6540,7 +6596,7 @@
         <v>16</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H12" s="39">
         <v>45894</v>
@@ -6595,7 +6651,7 @@
         <v>16</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H13" s="39">
         <v>45922</v>
@@ -6650,7 +6706,7 @@
         <v>16</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H14" s="39">
         <v>45923</v>
@@ -6705,7 +6761,7 @@
         <v>16</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H15" s="39">
         <v>45979</v>
@@ -6760,7 +6816,7 @@
         <v>44</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H16" s="39">
         <v>45985</v>
@@ -6815,7 +6871,7 @@
         <v>49</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H17" s="39">
         <v>45987</v>
@@ -6870,7 +6926,7 @@
         <v>44</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H18" s="39">
         <v>46001</v>
@@ -6925,7 +6981,7 @@
         <v>35</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H19" s="39">
         <v>46001</v>
@@ -6980,7 +7036,7 @@
         <v>35</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="H20" s="39">
         <v>46002</v>
@@ -7035,7 +7091,7 @@
         <v>18</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H21" s="39">
         <v>46010</v>
@@ -7090,7 +7146,7 @@
         <v>18</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="H22" s="39">
         <v>46038</v>
@@ -7145,7 +7201,7 @@
         <v>47</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H23" s="39">
         <v>46041</v>
@@ -7200,7 +7256,7 @@
         <v>47</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H24" s="39">
         <v>46043</v>
@@ -7255,7 +7311,7 @@
         <v>52</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H25" s="3">
         <v>46024</v>
@@ -7307,7 +7363,7 @@
         <v>67</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H26" s="3">
         <v>46024</v>
@@ -7353,13 +7409,13 @@
         <v>275</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>696</v>
+        <v>689</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H27" s="3">
         <v>46070</v>
@@ -7411,7 +7467,7 @@
         <v>18</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H28" s="3">
         <v>46121</v>
@@ -7462,7 +7518,7 @@
         <v>18</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H29" s="3">
         <v>46121</v>
@@ -7513,7 +7569,7 @@
         <v>20</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H30" s="3">
         <v>46126</v>
@@ -7564,7 +7620,7 @@
         <v>18</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H31" s="3">
         <v>46129</v>
@@ -7615,7 +7671,7 @@
         <v>20</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H32" s="3">
         <v>46132</v>
@@ -7659,14 +7715,14 @@
       <c r="D33" s="2">
         <v>30</v>
       </c>
-      <c r="E33" s="68" t="s">
+      <c r="E33" s="66" t="s">
         <v>101</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>35</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H33" s="3">
         <v>46155</v>
@@ -7710,14 +7766,14 @@
       <c r="D34" s="2">
         <v>49</v>
       </c>
-      <c r="E34" s="68" t="s">
+      <c r="E34" s="66" t="s">
         <v>28</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H34" s="3">
         <v>46175</v>
@@ -7761,14 +7817,14 @@
       <c r="D35" s="2">
         <v>45</v>
       </c>
-      <c r="E35" s="68" t="s">
+      <c r="E35" s="66" t="s">
         <v>17</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H35" s="3">
         <v>46177</v>
@@ -7812,14 +7868,14 @@
       <c r="D36" s="2">
         <v>74</v>
       </c>
-      <c r="E36" s="68" t="s">
+      <c r="E36" s="66" t="s">
         <v>33</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H36" s="3">
         <v>46185</v>
@@ -7863,14 +7919,14 @@
       <c r="D37" s="2">
         <v>34</v>
       </c>
-      <c r="E37" s="68" t="s">
+      <c r="E37" s="66" t="s">
         <v>72</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="H37" s="3">
         <v>46184</v>
@@ -7914,14 +7970,14 @@
       <c r="D38" s="2">
         <v>62</v>
       </c>
-      <c r="E38" s="68" t="s">
+      <c r="E38" s="66" t="s">
         <v>23</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H38" s="3">
         <v>46197</v>
@@ -7965,14 +8021,14 @@
       <c r="D39" s="2">
         <v>39</v>
       </c>
-      <c r="E39" s="68" t="s">
+      <c r="E39" s="66" t="s">
         <v>56</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="H39" s="3">
         <v>46197</v>
@@ -8023,7 +8079,7 @@
         <v>49</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H40" s="3">
         <v>46197</v>
@@ -8074,7 +8130,7 @@
         <v>20</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H41" s="3">
         <v>46210</v>
@@ -8125,7 +8181,7 @@
         <v>44</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="H42" s="3">
         <v>46210</v>
@@ -8578,7 +8634,9 @@
       <c r="I51" s="3">
         <v>46303</v>
       </c>
-      <c r="J51" s="3"/>
+      <c r="J51" s="3">
+        <v>46310</v>
+      </c>
       <c r="K51" s="3">
         <v>46301</v>
       </c>
@@ -8588,16 +8646,24 @@
       <c r="M51" s="3">
         <v>46304</v>
       </c>
-      <c r="N51" s="3"/>
-      <c r="O51" s="3"/>
-      <c r="P51" s="47"/>
+      <c r="N51" s="3">
+        <v>46310</v>
+      </c>
+      <c r="O51" s="3">
+        <v>46310</v>
+      </c>
+      <c r="P51" s="47">
+        <v>46310</v>
+      </c>
       <c r="Q51" s="38">
         <f t="shared" ref="Q51" ca="1" si="4">IF(P51&gt;0,P51-I51+1,IF(I51&gt;0,TODAY()-I51+1,""))</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" spans="2:17" ht="26.15" customHeight="1">
-      <c r="B52" s="2"/>
+      <c r="B52" s="2">
+        <v>43</v>
+      </c>
       <c r="C52" s="2">
         <v>5659</v>
       </c>
@@ -8685,7 +8751,7 @@
     <col min="19" max="19" width="67.36328125" style="11" customWidth="1"/>
     <col min="20" max="20" width="63.90625" style="11" customWidth="1"/>
     <col min="21" max="21" width="66.81640625" style="11" customWidth="1"/>
-    <col min="22" max="22" width="82.453125" style="11" customWidth="1"/>
+    <col min="22" max="22" width="85.1796875" style="11" customWidth="1"/>
     <col min="23" max="23" width="82.54296875" style="11" customWidth="1"/>
     <col min="24" max="24" width="79.453125" style="11" customWidth="1"/>
     <col min="25" max="25" width="71" style="11" customWidth="1"/>
@@ -8763,7 +8829,7 @@
         <v>293</v>
       </c>
       <c r="T10" s="50" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="U10" s="15" t="s">
         <v>117</v>
@@ -8819,7 +8885,7 @@
         <v>64</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
       <c r="G11" s="17" t="s">
         <v>4</v>
@@ -8851,56 +8917,56 @@
       <c r="P11" s="40">
         <v>45863</v>
       </c>
-      <c r="Q11" s="73" t="s">
-        <v>756</v>
-      </c>
-      <c r="R11" s="73" t="s">
-        <v>756</v>
-      </c>
-      <c r="S11" s="73" t="s">
-        <v>756</v>
+      <c r="Q11" s="68" t="s">
+        <v>739</v>
+      </c>
+      <c r="R11" s="68" t="s">
+        <v>739</v>
+      </c>
+      <c r="S11" s="68" t="s">
+        <v>739</v>
       </c>
       <c r="T11" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U11" s="57" t="s">
-        <v>683</v>
+        <v>676</v>
       </c>
       <c r="V11" s="57" t="s">
-        <v>684</v>
+        <v>677</v>
       </c>
       <c r="W11" s="57" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="X11" s="57" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
       <c r="Y11" s="57" t="s">
-        <v>767</v>
+        <v>750</v>
       </c>
       <c r="Z11" s="57" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
       <c r="AA11" s="57" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
       <c r="AB11" s="19" t="s">
         <v>119</v>
       </c>
       <c r="AC11" s="57" t="s">
-        <v>768</v>
+        <v>751</v>
       </c>
       <c r="AD11" s="57" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
       <c r="AE11" s="57" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="AF11" s="57" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="AG11" s="57" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="AH11" s="10"/>
     </row>
@@ -8951,13 +9017,13 @@
         <v>45905</v>
       </c>
       <c r="Q12" s="57" t="s">
-        <v>678</v>
+        <v>671</v>
       </c>
       <c r="R12" s="57" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="S12" s="57" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="T12" s="46" t="s">
         <v>146</v>
@@ -8981,7 +9047,7 @@
         <v>134</v>
       </c>
       <c r="AA12" s="57" t="s">
-        <v>693</v>
+        <v>686</v>
       </c>
       <c r="AB12" s="19" t="s">
         <v>135</v>
@@ -8990,7 +9056,7 @@
         <v>136</v>
       </c>
       <c r="AD12" s="57" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
       <c r="AE12" s="57" t="s">
         <v>138</v>
@@ -9049,13 +9115,13 @@
         <v>45908</v>
       </c>
       <c r="Q13" s="57" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="R13" s="57" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="S13" s="57" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="T13" s="46" t="s">
         <v>146</v>
@@ -9147,13 +9213,13 @@
         <v>45933</v>
       </c>
       <c r="Q14" s="57" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="R14" s="57" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="S14" s="57" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="T14" s="46" t="s">
         <v>146</v>
@@ -9189,7 +9255,7 @@
         <v>150</v>
       </c>
       <c r="AE14" s="57" t="s">
-        <v>680</v>
+        <v>673</v>
       </c>
       <c r="AF14" s="57" t="s">
         <v>153</v>
@@ -9245,13 +9311,13 @@
         <v>45933</v>
       </c>
       <c r="Q15" s="57" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="R15" s="57" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="S15" s="57" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="T15" s="46" t="s">
         <v>146</v>
@@ -9343,13 +9409,13 @@
         <v>45985</v>
       </c>
       <c r="Q16" s="57" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="R16" s="57" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="S16" s="57" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="T16" s="46" t="s">
         <v>146</v>
@@ -9441,13 +9507,13 @@
         <v>45994</v>
       </c>
       <c r="Q17" s="57" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="R17" s="57" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="S17" s="57" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="T17" s="46" t="s">
         <v>146</v>
@@ -9539,13 +9605,13 @@
         <v>45996</v>
       </c>
       <c r="Q18" s="57" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="R18" s="57" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="S18" s="57" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="T18" s="46" t="s">
         <v>146</v>
@@ -9637,13 +9703,13 @@
         <v>46008</v>
       </c>
       <c r="Q19" s="57" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="R19" s="57" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="S19" s="57" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="T19" s="46" t="s">
         <v>146</v>
@@ -9735,13 +9801,13 @@
         <v>46011</v>
       </c>
       <c r="Q20" s="57" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="R20" s="57" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="S20" s="57" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="T20" s="46" t="s">
         <v>146</v>
@@ -9833,13 +9899,13 @@
         <v>46008</v>
       </c>
       <c r="Q21" s="57" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="R21" s="57" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="S21" s="57" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="T21" s="46" t="s">
         <v>146</v>
@@ -9931,13 +9997,13 @@
         <v>46014</v>
       </c>
       <c r="Q22" s="57" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="R22" s="57" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="S22" s="57" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="T22" s="46" t="s">
         <v>146</v>
@@ -10029,13 +10095,13 @@
         <v>46045</v>
       </c>
       <c r="Q23" s="57" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="R23" s="57" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="S23" s="52" t="s">
-        <v>676</v>
+        <v>669</v>
       </c>
       <c r="T23" s="46" t="s">
         <v>146</v>
@@ -10127,16 +10193,16 @@
         <v>46048</v>
       </c>
       <c r="Q24" s="57" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="R24" s="57" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="S24" s="57" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="T24" s="57" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="U24" s="57" t="s">
         <v>306</v>
@@ -10225,16 +10291,16 @@
         <v>46049</v>
       </c>
       <c r="Q25" s="57" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="R25" s="57" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="S25" s="57" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="T25" s="57" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="U25" s="57" t="s">
         <v>307</v>
@@ -10323,16 +10389,16 @@
         <v>46066</v>
       </c>
       <c r="Q26" s="57" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="R26" s="57" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="S26" s="57" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="T26" s="57" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="U26" s="57" t="s">
         <v>308</v>
@@ -10353,7 +10419,7 @@
         <v>270</v>
       </c>
       <c r="AA26" s="57" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="AB26" s="19" t="s">
         <v>266</v>
@@ -10421,16 +10487,16 @@
         <v>46069</v>
       </c>
       <c r="Q27" s="57" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="R27" s="57" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="S27" s="57" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="T27" s="57" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="U27" s="57" t="s">
         <v>309</v>
@@ -10438,8 +10504,8 @@
       <c r="V27" s="57" t="s">
         <v>285</v>
       </c>
-      <c r="W27" s="74" t="s">
-        <v>755</v>
+      <c r="W27" s="69" t="s">
+        <v>738</v>
       </c>
       <c r="X27" s="57" t="s">
         <v>286</v>
@@ -10486,7 +10552,7 @@
         <v>60</v>
       </c>
       <c r="F28" s="49" t="s">
-        <v>696</v>
+        <v>689</v>
       </c>
       <c r="G28" s="49" t="s">
         <v>4</v>
@@ -10518,56 +10584,56 @@
       <c r="P28" s="47">
         <v>46078</v>
       </c>
-      <c r="Q28" s="73" t="s">
-        <v>756</v>
-      </c>
-      <c r="R28" s="73" t="s">
-        <v>756</v>
-      </c>
-      <c r="S28" s="73" t="s">
-        <v>756</v>
+      <c r="Q28" s="68" t="s">
+        <v>739</v>
+      </c>
+      <c r="R28" s="68" t="s">
+        <v>739</v>
+      </c>
+      <c r="S28" s="68" t="s">
+        <v>739</v>
       </c>
       <c r="T28" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U28" s="57" t="s">
-        <v>757</v>
+        <v>740</v>
       </c>
       <c r="V28" s="46" t="s">
         <v>146</v>
       </c>
       <c r="W28" s="57" t="s">
-        <v>758</v>
+        <v>741</v>
       </c>
       <c r="X28" s="57" t="s">
-        <v>759</v>
+        <v>742</v>
       </c>
       <c r="Y28" s="46" t="s">
         <v>146</v>
       </c>
       <c r="Z28" s="57" t="s">
-        <v>760</v>
+        <v>743</v>
       </c>
       <c r="AA28" s="57" t="s">
-        <v>761</v>
+        <v>744</v>
       </c>
       <c r="AB28" s="19" t="s">
         <v>276</v>
       </c>
       <c r="AC28" s="57" t="s">
-        <v>762</v>
+        <v>745</v>
       </c>
       <c r="AD28" s="57" t="s">
-        <v>763</v>
+        <v>746</v>
       </c>
       <c r="AE28" s="57" t="s">
-        <v>766</v>
+        <v>749</v>
       </c>
       <c r="AF28" s="57" t="s">
-        <v>764</v>
+        <v>747</v>
       </c>
       <c r="AG28" s="57" t="s">
-        <v>765</v>
+        <v>748</v>
       </c>
       <c r="AH28" s="10"/>
       <c r="AI28" s="10"/>
@@ -10619,13 +10685,13 @@
         <v>46129</v>
       </c>
       <c r="Q29" s="60" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="R29" s="60" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="S29" s="60" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="T29" s="46" t="s">
         <v>146</v>
@@ -10640,7 +10706,7 @@
         <v>343</v>
       </c>
       <c r="X29" s="57" t="s">
-        <v>694</v>
+        <v>687</v>
       </c>
       <c r="Y29" s="46" t="s">
         <v>146</v>
@@ -10717,13 +10783,13 @@
         <v>46129</v>
       </c>
       <c r="Q30" s="60" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="R30" s="60" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="S30" s="60" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="T30" s="46" t="s">
         <v>146</v>
@@ -10815,13 +10881,13 @@
         <v>46134</v>
       </c>
       <c r="Q31" s="60" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="R31" s="60" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="S31" s="60" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="T31" s="46" t="s">
         <v>146</v>
@@ -10863,7 +10929,7 @@
         <v>339</v>
       </c>
       <c r="AG31" s="57" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="32" spans="2:35" ht="131.4" customHeight="1">
@@ -10913,13 +10979,13 @@
         <v>46135</v>
       </c>
       <c r="Q32" s="60" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="R32" s="60" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="S32" s="60" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="T32" s="46" t="s">
         <v>146</v>
@@ -11011,13 +11077,13 @@
         <v>46140</v>
       </c>
       <c r="Q33" s="60" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="R33" s="60" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="S33" s="60" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="T33" s="46" t="s">
         <v>146</v>
@@ -11038,7 +11104,7 @@
         <v>146</v>
       </c>
       <c r="Z33" s="57" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="AA33" s="57" t="s">
         <v>360</v>
@@ -11109,13 +11175,13 @@
         <v>46162</v>
       </c>
       <c r="Q34" s="60" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="R34" s="60" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="S34" s="60" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="T34" s="46" t="s">
         <v>146</v>
@@ -11127,7 +11193,7 @@
         <v>373</v>
       </c>
       <c r="W34" s="57" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="X34" s="57" t="s">
         <v>374</v>
@@ -11154,10 +11220,10 @@
         <v>375</v>
       </c>
       <c r="AF34" s="57" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="AG34" s="57" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="35" spans="2:33" ht="62.4" customHeight="1">
@@ -11207,13 +11273,13 @@
         <v>46183</v>
       </c>
       <c r="Q35" s="60" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="R35" s="60" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="S35" s="60" t="s">
-        <v>697</v>
+        <v>690</v>
       </c>
       <c r="T35" s="46" t="s">
         <v>146</v>
@@ -11243,7 +11309,7 @@
         <v>390</v>
       </c>
       <c r="AC35" s="57" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="AD35" s="57" t="s">
         <v>392</v>
@@ -11255,7 +11321,7 @@
         <v>394</v>
       </c>
       <c r="AG35" s="57" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="36" spans="2:33" ht="87">
@@ -11305,13 +11371,13 @@
         <v>46184</v>
       </c>
       <c r="Q36" s="60" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="R36" s="60" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="S36" s="60" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="T36" s="46" t="s">
         <v>146</v>
@@ -11323,10 +11389,10 @@
         <v>385</v>
       </c>
       <c r="W36" s="57" t="s">
+        <v>404</v>
+      </c>
+      <c r="X36" s="57" t="s">
         <v>405</v>
-      </c>
-      <c r="X36" s="57" t="s">
-        <v>406</v>
       </c>
       <c r="Y36" s="46" t="s">
         <v>146</v>
@@ -11335,25 +11401,25 @@
         <v>146</v>
       </c>
       <c r="AA36" s="57" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AB36" s="19" t="s">
         <v>396</v>
       </c>
       <c r="AC36" s="57" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="AD36" s="57" t="s">
+        <v>407</v>
+      </c>
+      <c r="AE36" s="57" t="s">
         <v>408</v>
       </c>
-      <c r="AE36" s="57" t="s">
+      <c r="AF36" s="57" t="s">
         <v>409</v>
       </c>
-      <c r="AF36" s="57" t="s">
-        <v>410</v>
-      </c>
       <c r="AG36" s="57" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="37" spans="2:33" ht="101.5">
@@ -11403,28 +11469,28 @@
         <v>46191</v>
       </c>
       <c r="Q37" s="60" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="R37" s="60" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="S37" s="60" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="T37" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U37" s="57" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="V37" s="57" t="s">
+        <v>412</v>
+      </c>
+      <c r="W37" s="57" t="s">
         <v>413</v>
       </c>
-      <c r="W37" s="57" t="s">
+      <c r="X37" s="57" t="s">
         <v>414</v>
-      </c>
-      <c r="X37" s="57" t="s">
-        <v>415</v>
       </c>
       <c r="Y37" s="46" t="s">
         <v>146</v>
@@ -11433,25 +11499,25 @@
         <v>146</v>
       </c>
       <c r="AA37" s="57" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="AB37" s="19" t="s">
         <v>397</v>
       </c>
       <c r="AC37" s="57" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="AD37" s="57" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="AE37" s="57" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="AF37" s="57" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="AG37" s="57" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="38" spans="2:33" ht="84.9" customHeight="1">
@@ -11501,13 +11567,13 @@
         <v>46192</v>
       </c>
       <c r="Q38" s="60" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="R38" s="60" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="S38" s="60" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="T38" s="46" t="s">
         <v>146</v>
@@ -11531,25 +11597,25 @@
         <v>146</v>
       </c>
       <c r="AA38" s="57" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="AB38" s="19" t="s">
         <v>402</v>
       </c>
       <c r="AC38" s="57" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="AD38" s="57" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AE38" s="57" t="s">
         <v>403</v>
       </c>
       <c r="AF38" s="57" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="AG38" s="57" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="39" spans="2:33" ht="78.900000000000006" customHeight="1">
@@ -11599,28 +11665,28 @@
         <v>46205</v>
       </c>
       <c r="Q39" s="60" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="R39" s="60" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="S39" s="60" t="s">
-        <v>699</v>
+        <v>692</v>
       </c>
       <c r="T39" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U39" s="57" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="V39" s="57" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="W39" s="57" t="s">
+        <v>421</v>
+      </c>
+      <c r="X39" s="57" t="s">
         <v>422</v>
-      </c>
-      <c r="X39" s="57" t="s">
-        <v>423</v>
       </c>
       <c r="Y39" s="46" t="s">
         <v>146</v>
@@ -11629,25 +11695,25 @@
         <v>146</v>
       </c>
       <c r="AA39" s="57" t="s">
+        <v>435</v>
+      </c>
+      <c r="AB39" s="19" t="s">
+        <v>416</v>
+      </c>
+      <c r="AC39" s="57" t="s">
+        <v>498</v>
+      </c>
+      <c r="AD39" s="57" t="s">
+        <v>438</v>
+      </c>
+      <c r="AE39" s="57" t="s">
         <v>436</v>
       </c>
-      <c r="AB39" s="19" t="s">
-        <v>417</v>
-      </c>
-      <c r="AC39" s="57" t="s">
-        <v>501</v>
-      </c>
-      <c r="AD39" s="57" t="s">
-        <v>439</v>
-      </c>
-      <c r="AE39" s="57" t="s">
-        <v>437</v>
-      </c>
       <c r="AF39" s="57" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="AG39" s="57" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="40" spans="2:33" ht="101.5">
@@ -11697,55 +11763,55 @@
         <v>46205</v>
       </c>
       <c r="Q40" s="60" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="R40" s="60" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="S40" s="60" t="s">
-        <v>698</v>
+        <v>691</v>
       </c>
       <c r="T40" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U40" s="57" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="V40" s="57" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="W40" s="57" t="s">
+        <v>425</v>
+      </c>
+      <c r="X40" s="57" t="s">
         <v>426</v>
-      </c>
-      <c r="X40" s="57" t="s">
-        <v>427</v>
       </c>
       <c r="Y40" s="46" t="s">
         <v>146</v>
       </c>
       <c r="Z40" s="57" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="AA40" s="57" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="AB40" s="19" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AC40" s="57" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="AD40" s="57" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="AE40" s="57" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="AF40" s="57" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="AG40" s="57" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="41" spans="2:33" ht="69.650000000000006" customHeight="1">
@@ -11795,55 +11861,55 @@
         <v>46205</v>
       </c>
       <c r="Q41" s="60" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="R41" s="60" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="S41" s="60" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="T41" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U41" s="57" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="V41" s="57" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="W41" s="57" t="s">
+        <v>423</v>
+      </c>
+      <c r="X41" s="57" t="s">
         <v>424</v>
-      </c>
-      <c r="X41" s="57" t="s">
-        <v>425</v>
       </c>
       <c r="Y41" s="46" t="s">
         <v>146</v>
       </c>
       <c r="Z41" s="57" t="s">
+        <v>433</v>
+      </c>
+      <c r="AA41" s="57" t="s">
+        <v>437</v>
+      </c>
+      <c r="AB41" s="19" t="s">
+        <v>420</v>
+      </c>
+      <c r="AC41" s="57" t="s">
+        <v>511</v>
+      </c>
+      <c r="AD41" s="57" t="s">
+        <v>439</v>
+      </c>
+      <c r="AE41" s="57" t="s">
         <v>434</v>
       </c>
-      <c r="AA41" s="57" t="s">
-        <v>438</v>
-      </c>
-      <c r="AB41" s="19" t="s">
-        <v>421</v>
-      </c>
-      <c r="AC41" s="57" t="s">
-        <v>514</v>
-      </c>
-      <c r="AD41" s="57" t="s">
-        <v>440</v>
-      </c>
-      <c r="AE41" s="57" t="s">
-        <v>435</v>
-      </c>
       <c r="AF41" s="57" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="AG41" s="57" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="42" spans="2:33" ht="87">
@@ -11893,55 +11959,55 @@
         <v>46218</v>
       </c>
       <c r="Q42" s="60" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="R42" s="60" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="S42" s="60" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="T42" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U42" s="57" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="V42" s="57" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="W42" s="57" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="X42" s="57" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="Y42" s="46" t="s">
         <v>146</v>
       </c>
       <c r="Z42" s="57" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="AA42" s="57" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="AB42" s="19" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="AC42" s="57" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="AD42" s="57" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="AE42" s="57" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="AF42" s="57" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="AG42" s="57" t="s">
-        <v>669</v>
+        <v>662</v>
       </c>
     </row>
     <row r="43" spans="2:33" ht="87">
@@ -11991,55 +12057,55 @@
         <v>46218</v>
       </c>
       <c r="Q43" s="60" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="R43" s="60" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="S43" s="60" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="T43" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U43" s="57" t="s">
+        <v>462</v>
+      </c>
+      <c r="V43" s="60" t="s">
+        <v>451</v>
+      </c>
+      <c r="W43" s="57" t="s">
+        <v>464</v>
+      </c>
+      <c r="X43" s="57" t="s">
         <v>465</v>
-      </c>
-      <c r="V43" s="60" t="s">
-        <v>453</v>
-      </c>
-      <c r="W43" s="57" t="s">
-        <v>467</v>
-      </c>
-      <c r="X43" s="57" t="s">
-        <v>468</v>
       </c>
       <c r="Y43" s="46" t="s">
         <v>146</v>
       </c>
       <c r="Z43" s="57" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="AA43" s="57" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="AB43" s="19" t="s">
+        <v>472</v>
+      </c>
+      <c r="AC43" s="57" t="s">
+        <v>513</v>
+      </c>
+      <c r="AD43" s="57" t="s">
+        <v>485</v>
+      </c>
+      <c r="AE43" s="57" t="s">
         <v>475</v>
       </c>
-      <c r="AC43" s="57" t="s">
-        <v>516</v>
-      </c>
-      <c r="AD43" s="57" t="s">
-        <v>488</v>
-      </c>
-      <c r="AE43" s="57" t="s">
-        <v>478</v>
-      </c>
       <c r="AF43" s="57" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="AG43" s="57" t="s">
-        <v>670</v>
+        <v>663</v>
       </c>
     </row>
     <row r="44" spans="2:33" ht="87">
@@ -12089,28 +12155,28 @@
         <v>46240</v>
       </c>
       <c r="Q44" s="60" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="R44" s="60" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="S44" s="52" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="T44" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U44" s="57" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="V44" s="60" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="W44" s="57" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="X44" s="57" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="Y44" s="46" t="s">
         <v>146</v>
@@ -12119,25 +12185,25 @@
         <v>146</v>
       </c>
       <c r="AA44" s="57" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="AB44" s="19" t="s">
+        <v>500</v>
+      </c>
+      <c r="AC44" s="57" t="s">
+        <v>734</v>
+      </c>
+      <c r="AD44" s="57" t="s">
+        <v>510</v>
+      </c>
+      <c r="AE44" s="57" t="s">
         <v>503</v>
       </c>
-      <c r="AC44" s="57" t="s">
-        <v>751</v>
-      </c>
-      <c r="AD44" s="57" t="s">
-        <v>513</v>
-      </c>
-      <c r="AE44" s="57" t="s">
-        <v>506</v>
-      </c>
       <c r="AF44" s="59" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="AG44" s="57" t="s">
-        <v>671</v>
+        <v>664</v>
       </c>
     </row>
     <row r="45" spans="2:33" ht="72.5">
@@ -12187,28 +12253,28 @@
         <v>46240</v>
       </c>
       <c r="Q45" s="60" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="R45" s="60" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="S45" s="52" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="T45" s="46" t="s">
         <v>146</v>
       </c>
       <c r="U45" s="57" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="V45" s="60" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="W45" s="57" t="s">
+        <v>506</v>
+      </c>
+      <c r="X45" s="57" t="s">
         <v>509</v>
-      </c>
-      <c r="X45" s="57" t="s">
-        <v>512</v>
       </c>
       <c r="Y45" s="46" t="s">
         <v>146</v>
@@ -12217,25 +12283,25 @@
         <v>146</v>
       </c>
       <c r="AA45" s="57" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="AB45" s="19" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="AC45" s="57" t="s">
-        <v>752</v>
+        <v>735</v>
       </c>
       <c r="AD45" s="57" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="AE45" s="57" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="AF45" s="59" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="AG45" s="57" t="s">
-        <v>675</v>
+        <v>668</v>
       </c>
     </row>
     <row r="46" spans="2:33" ht="87">
@@ -12285,26 +12351,26 @@
         <v>46262</v>
       </c>
       <c r="Q46" s="60" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="R46" s="60" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="S46" s="60" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="T46" s="52"/>
       <c r="U46" s="57" t="s">
+        <v>516</v>
+      </c>
+      <c r="V46" s="60" t="s">
+        <v>517</v>
+      </c>
+      <c r="W46" s="57" t="s">
+        <v>518</v>
+      </c>
+      <c r="X46" s="57" t="s">
         <v>519</v>
-      </c>
-      <c r="V46" s="60" t="s">
-        <v>520</v>
-      </c>
-      <c r="W46" s="57" t="s">
-        <v>521</v>
-      </c>
-      <c r="X46" s="57" t="s">
-        <v>522</v>
       </c>
       <c r="Y46" s="46" t="s">
         <v>146</v>
@@ -12313,25 +12379,25 @@
         <v>146</v>
       </c>
       <c r="AA46" s="57" t="s">
+        <v>520</v>
+      </c>
+      <c r="AB46" s="19" t="s">
+        <v>515</v>
+      </c>
+      <c r="AC46" s="57" t="s">
+        <v>736</v>
+      </c>
+      <c r="AD46" s="57" t="s">
+        <v>521</v>
+      </c>
+      <c r="AE46" s="57" t="s">
+        <v>522</v>
+      </c>
+      <c r="AF46" s="59" t="s">
         <v>523</v>
       </c>
-      <c r="AB46" s="19" t="s">
-        <v>518</v>
-      </c>
-      <c r="AC46" s="57" t="s">
-        <v>753</v>
-      </c>
-      <c r="AD46" s="57" t="s">
-        <v>524</v>
-      </c>
-      <c r="AE46" s="57" t="s">
-        <v>525</v>
-      </c>
-      <c r="AF46" s="59" t="s">
-        <v>526</v>
-      </c>
       <c r="AG46" s="57" t="s">
-        <v>672</v>
+        <v>665</v>
       </c>
     </row>
     <row r="47" spans="2:33" ht="116">
@@ -12381,56 +12447,56 @@
         <v>46275</v>
       </c>
       <c r="Q47" s="60" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="R47" s="60" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="S47" s="60" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="T47" s="56"/>
       <c r="U47" s="57" t="s">
+        <v>638</v>
+      </c>
+      <c r="V47" s="60" t="s">
+        <v>639</v>
+      </c>
+      <c r="W47" s="57" t="s">
+        <v>640</v>
+      </c>
+      <c r="X47" s="57" t="s">
         <v>641</v>
-      </c>
-      <c r="V47" s="60" t="s">
-        <v>642</v>
-      </c>
-      <c r="W47" s="57" t="s">
-        <v>643</v>
-      </c>
-      <c r="X47" s="57" t="s">
-        <v>644</v>
       </c>
       <c r="Y47" s="46" t="s">
         <v>146</v>
       </c>
       <c r="Z47" s="57" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="AA47" s="57" t="s">
-        <v>754</v>
+        <v>737</v>
       </c>
       <c r="AB47" s="19" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="AC47" s="45" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="AD47" s="57" t="s">
-        <v>677</v>
+        <v>670</v>
       </c>
       <c r="AE47" s="57" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="AF47" s="59" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="AG47" s="57" t="s">
-        <v>668</v>
+        <v>661</v>
       </c>
     </row>
-    <row r="48" spans="2:33" ht="72.5">
+    <row r="48" spans="2:33" ht="87">
       <c r="B48" s="16">
         <v>86568</v>
       </c>
@@ -12444,7 +12510,7 @@
         <v>7</v>
       </c>
       <c r="F48" s="25" t="s">
-        <v>750</v>
+        <v>733</v>
       </c>
       <c r="G48" s="23" t="s">
         <v>80</v>
@@ -12477,26 +12543,26 @@
         <v>46286</v>
       </c>
       <c r="Q48" s="60" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="R48" s="60" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="S48" s="60" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="T48" s="56"/>
       <c r="U48" s="57" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
       <c r="V48" s="60" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="W48" s="57" t="s">
-        <v>667</v>
+        <v>660</v>
       </c>
       <c r="X48" s="57" t="s">
-        <v>666</v>
+        <v>659</v>
       </c>
       <c r="Y48" s="46" t="s">
         <v>146</v>
@@ -12504,29 +12570,29 @@
       <c r="Z48" s="46" t="s">
         <v>146</v>
       </c>
-      <c r="AA48" s="59" t="s">
-        <v>648</v>
+      <c r="AA48" s="57" t="s">
+        <v>762</v>
       </c>
       <c r="AB48" s="19" t="s">
+        <v>645</v>
+      </c>
+      <c r="AC48" s="45" t="s">
+        <v>646</v>
+      </c>
+      <c r="AD48" s="57" t="s">
+        <v>763</v>
+      </c>
+      <c r="AE48" s="57" t="s">
         <v>649</v>
       </c>
-      <c r="AC48" s="45" t="s">
+      <c r="AF48" s="59" t="s">
         <v>650</v>
       </c>
-      <c r="AD48" s="59" t="s">
-        <v>651</v>
-      </c>
-      <c r="AE48" s="57" t="s">
-        <v>654</v>
-      </c>
-      <c r="AF48" s="59" t="s">
-        <v>655</v>
-      </c>
       <c r="AG48" s="57" t="s">
-        <v>673</v>
+        <v>666</v>
       </c>
     </row>
-    <row r="49" spans="2:33" ht="72.5">
+    <row r="49" spans="2:33" ht="87">
       <c r="B49" s="16">
         <v>86568</v>
       </c>
@@ -12573,26 +12639,26 @@
         <v>46286</v>
       </c>
       <c r="Q49" s="60" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="R49" s="60" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="S49" s="60" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="T49" s="56"/>
       <c r="U49" s="60" t="s">
-        <v>660</v>
+        <v>653</v>
       </c>
       <c r="V49" s="60" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="W49" s="60" t="s">
-        <v>662</v>
+        <v>655</v>
       </c>
       <c r="X49" s="60" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="Y49" s="63" t="s">
         <v>146</v>
@@ -12600,29 +12666,29 @@
       <c r="Z49" s="63" t="s">
         <v>146</v>
       </c>
-      <c r="AA49" s="64" t="s">
-        <v>656</v>
+      <c r="AA49" s="60" t="s">
+        <v>764</v>
       </c>
       <c r="AB49" s="28" t="s">
+        <v>651</v>
+      </c>
+      <c r="AC49" s="52" t="s">
+        <v>652</v>
+      </c>
+      <c r="AD49" s="70" t="s">
+        <v>768</v>
+      </c>
+      <c r="AE49" s="60" t="s">
         <v>657</v>
       </c>
-      <c r="AC49" s="52" t="s">
+      <c r="AF49" s="64" t="s">
         <v>658</v>
       </c>
-      <c r="AD49" s="64" t="s">
-        <v>659</v>
-      </c>
-      <c r="AE49" s="60" t="s">
-        <v>664</v>
-      </c>
-      <c r="AF49" s="64" t="s">
-        <v>665</v>
-      </c>
       <c r="AG49" s="60" t="s">
-        <v>674</v>
+        <v>667</v>
       </c>
     </row>
-    <row r="50" spans="2:33" ht="48.75" customHeight="1">
+    <row r="50" spans="2:33" ht="72.5">
       <c r="B50" s="16">
         <v>86573</v>
       </c>
@@ -12668,57 +12734,57 @@
       <c r="P50" s="47">
         <v>46296</v>
       </c>
-      <c r="Q50" s="71" t="s">
-        <v>749</v>
-      </c>
-      <c r="R50" s="71" t="s">
-        <v>748</v>
-      </c>
-      <c r="S50" s="71" t="s">
-        <v>747</v>
+      <c r="Q50" s="57" t="s">
+        <v>732</v>
+      </c>
+      <c r="R50" s="57" t="s">
+        <v>731</v>
+      </c>
+      <c r="S50" s="57" t="s">
+        <v>730</v>
       </c>
       <c r="T50" s="65"/>
-      <c r="U50" s="71" t="s">
-        <v>721</v>
-      </c>
-      <c r="V50" s="71" t="s">
-        <v>720</v>
-      </c>
-      <c r="W50" s="66" t="s">
-        <v>712</v>
-      </c>
-      <c r="X50" s="66" t="s">
-        <v>713</v>
-      </c>
-      <c r="Y50" s="67" t="s">
+      <c r="U50" s="57" t="s">
+        <v>710</v>
+      </c>
+      <c r="V50" s="57" t="s">
+        <v>709</v>
+      </c>
+      <c r="W50" s="71" t="s">
+        <v>752</v>
+      </c>
+      <c r="X50" s="57" t="s">
+        <v>753</v>
+      </c>
+      <c r="Y50" s="72" t="s">
         <v>146</v>
       </c>
-      <c r="Z50" s="67" t="s">
+      <c r="Z50" s="72" t="s">
         <v>146</v>
       </c>
-      <c r="AA50" s="66" t="s">
-        <v>714</v>
-      </c>
-      <c r="AB50" s="45" t="s">
-        <v>715</v>
+      <c r="AA50" s="57" t="s">
+        <v>765</v>
+      </c>
+      <c r="AB50" s="19" t="s">
+        <v>705</v>
       </c>
       <c r="AC50" s="45" t="s">
-        <v>716</v>
-      </c>
-      <c r="AD50" s="66" t="s">
-        <v>717</v>
-      </c>
-      <c r="AE50" s="66" t="s">
-        <v>718</v>
-      </c>
-      <c r="AF50" s="66" t="s">
-        <v>719</v>
-      </c>
-      <c r="AG50" s="66" t="s">
-        <v>719</v>
+        <v>706</v>
+      </c>
+      <c r="AD50" s="70" t="s">
+        <v>707</v>
+      </c>
+      <c r="AE50" s="57" t="s">
+        <v>754</v>
+      </c>
+      <c r="AF50" s="59" t="s">
+        <v>755</v>
+      </c>
+      <c r="AG50" s="70" t="s">
+        <v>708</v>
       </c>
     </row>
-    <row r="51" spans="2:33" ht="72.5">
+    <row r="51" spans="2:33" ht="58">
       <c r="B51" s="16">
         <v>44090</v>
       </c>
@@ -12770,50 +12836,50 @@
       <c r="R51" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="S51" s="70" t="s">
-        <v>745</v>
+      <c r="S51" s="57" t="s">
+        <v>729</v>
       </c>
       <c r="T51" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="U51" s="70" t="s">
-        <v>743</v>
-      </c>
-      <c r="V51" s="70" t="s">
-        <v>742</v>
-      </c>
-      <c r="W51" s="66" t="s">
-        <v>734</v>
-      </c>
-      <c r="X51" s="66" t="s">
-        <v>735</v>
-      </c>
-      <c r="Y51" s="67" t="s">
+      <c r="U51" s="57" t="s">
+        <v>727</v>
+      </c>
+      <c r="V51" s="57" t="s">
+        <v>726</v>
+      </c>
+      <c r="W51" s="57" t="s">
+        <v>757</v>
+      </c>
+      <c r="X51" s="57" t="s">
+        <v>771</v>
+      </c>
+      <c r="Y51" s="74" t="s">
+        <v>756</v>
+      </c>
+      <c r="Z51" s="46" t="s">
         <v>146</v>
       </c>
-      <c r="Z51" s="67" t="s">
-        <v>146</v>
-      </c>
-      <c r="AA51" s="66" t="s">
-        <v>736</v>
+      <c r="AA51" s="70" t="s">
+        <v>720</v>
       </c>
       <c r="AB51" s="45" t="s">
-        <v>737</v>
+        <v>721</v>
       </c>
       <c r="AC51" s="45" t="s">
-        <v>738</v>
-      </c>
-      <c r="AD51" s="66" t="s">
-        <v>739</v>
-      </c>
-      <c r="AE51" s="66" t="s">
-        <v>740</v>
-      </c>
-      <c r="AF51" s="66" t="s">
-        <v>741</v>
-      </c>
-      <c r="AG51" s="66" t="s">
-        <v>741</v>
+        <v>722</v>
+      </c>
+      <c r="AD51" s="70" t="s">
+        <v>723</v>
+      </c>
+      <c r="AE51" s="70" t="s">
+        <v>724</v>
+      </c>
+      <c r="AF51" s="59" t="s">
+        <v>772</v>
+      </c>
+      <c r="AG51" s="70" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="52" spans="2:33" ht="72.5">
@@ -12841,7 +12907,9 @@
       <c r="I52" s="3">
         <v>46303</v>
       </c>
-      <c r="J52" s="3"/>
+      <c r="J52" s="3">
+        <v>46310</v>
+      </c>
       <c r="K52" s="3">
         <v>46301</v>
       </c>
@@ -12851,75 +12919,85 @@
       <c r="M52" s="3">
         <v>46304</v>
       </c>
-      <c r="N52" s="18"/>
-      <c r="O52" s="18"/>
-      <c r="P52" s="18"/>
-      <c r="Q52" s="72" t="s">
-        <v>722</v>
-      </c>
-      <c r="R52" s="72" t="s">
-        <v>723</v>
-      </c>
-      <c r="S52" s="70" t="s">
-        <v>746</v>
+      <c r="N52" s="3">
+        <v>46310</v>
+      </c>
+      <c r="O52" s="3">
+        <v>46310</v>
+      </c>
+      <c r="P52" s="47">
+        <v>46310</v>
+      </c>
+      <c r="Q52" s="60" t="s">
+        <v>711</v>
+      </c>
+      <c r="R52" s="60" t="s">
+        <v>712</v>
+      </c>
+      <c r="S52" s="73" t="s">
+        <v>769</v>
       </c>
       <c r="T52" s="56"/>
-      <c r="U52" s="70" t="s">
-        <v>728</v>
-      </c>
-      <c r="V52" s="66" t="s">
-        <v>727</v>
-      </c>
-      <c r="W52" s="66" t="s">
-        <v>724</v>
-      </c>
-      <c r="X52" s="66" t="s">
-        <v>725</v>
-      </c>
-      <c r="Y52" s="67" t="s">
+      <c r="U52" s="57" t="s">
+        <v>714</v>
+      </c>
+      <c r="V52" s="57" t="s">
+        <v>770</v>
+      </c>
+      <c r="W52" s="57" t="s">
+        <v>766</v>
+      </c>
+      <c r="X52" s="57" t="s">
+        <v>767</v>
+      </c>
+      <c r="Y52" s="72" t="s">
         <v>146</v>
       </c>
-      <c r="Z52" s="67"/>
-      <c r="AA52" s="66" t="s">
-        <v>726</v>
+      <c r="Z52" s="72" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA52" s="70" t="s">
+        <v>713</v>
       </c>
       <c r="AB52" s="45" t="s">
-        <v>729</v>
+        <v>715</v>
       </c>
       <c r="AC52" s="45" t="s">
-        <v>730</v>
-      </c>
-      <c r="AD52" s="66" t="s">
-        <v>731</v>
-      </c>
-      <c r="AE52" s="66" t="s">
-        <v>732</v>
-      </c>
-      <c r="AF52" s="66" t="s">
-        <v>733</v>
-      </c>
-      <c r="AG52" s="66" t="s">
-        <v>733</v>
+        <v>716</v>
+      </c>
+      <c r="AD52" s="70" t="s">
+        <v>717</v>
+      </c>
+      <c r="AE52" s="70" t="s">
+        <v>718</v>
+      </c>
+      <c r="AF52" s="70" t="s">
+        <v>719</v>
+      </c>
+      <c r="AG52" s="70" t="s">
+        <v>719</v>
       </c>
     </row>
-    <row r="53" spans="2:33" ht="42.75" customHeight="1">
+    <row r="53" spans="2:33" ht="58">
       <c r="B53" s="16">
-        <v>94001</v>
+        <v>5659</v>
       </c>
       <c r="C53" s="16">
-        <v>58</v>
-      </c>
-      <c r="D53" s="55"/>
-      <c r="E53" s="55">
-        <v>14</v>
-      </c>
-      <c r="F53" s="21" t="s">
-        <v>110</v>
+        <v>34</v>
+      </c>
+      <c r="D53" s="55">
+        <v>43</v>
+      </c>
+      <c r="E53" s="16"/>
+      <c r="F53" s="23" t="s">
+        <v>98</v>
       </c>
       <c r="G53" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="H53" s="17"/>
+        <v>49</v>
+      </c>
+      <c r="H53" s="3">
+        <v>46281</v>
+      </c>
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
       <c r="K53" s="18"/>
@@ -12928,15 +13006,33 @@
       <c r="N53" s="18"/>
       <c r="O53" s="18"/>
       <c r="P53" s="18"/>
-      <c r="Q53" s="18"/>
-      <c r="R53" s="18"/>
-      <c r="S53" s="18"/>
-      <c r="T53" s="18"/>
-      <c r="U53" s="18"/>
-      <c r="V53" s="18"/>
-      <c r="W53" s="19"/>
-      <c r="X53" s="24"/>
-      <c r="Y53" s="24"/>
+      <c r="Q53" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="R53" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="S53" s="75" t="s">
+        <v>728</v>
+      </c>
+      <c r="T53" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="U53" s="57" t="s">
+        <v>758</v>
+      </c>
+      <c r="V53" s="57" t="s">
+        <v>760</v>
+      </c>
+      <c r="W53" s="57" t="s">
+        <v>761</v>
+      </c>
+      <c r="X53" s="57" t="s">
+        <v>759</v>
+      </c>
+      <c r="Y53" s="46" t="s">
+        <v>146</v>
+      </c>
       <c r="Z53" s="32"/>
       <c r="AA53" s="32"/>
       <c r="AB53" s="32"/>
@@ -12946,19 +13042,19 @@
       <c r="AF53" s="32"/>
       <c r="AG53" s="32"/>
     </row>
-    <row r="54" spans="2:33" ht="42.75" customHeight="1">
+    <row r="54" spans="2:33" ht="43.5">
       <c r="B54" s="16">
         <v>94001</v>
       </c>
       <c r="C54" s="16">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D54" s="55"/>
       <c r="E54" s="55">
-        <v>8</v>
-      </c>
-      <c r="F54" s="22" t="s">
-        <v>89</v>
+        <v>14</v>
+      </c>
+      <c r="F54" s="25" t="s">
+        <v>110</v>
       </c>
       <c r="G54" s="23" t="s">
         <v>90</v>
@@ -12977,10 +13073,12 @@
       <c r="S54" s="18"/>
       <c r="T54" s="18"/>
       <c r="U54" s="18"/>
-      <c r="V54" s="18"/>
+      <c r="V54" s="70" t="s">
+        <v>777</v>
+      </c>
       <c r="W54" s="19"/>
-      <c r="X54" s="19"/>
-      <c r="Y54" s="19"/>
+      <c r="X54" s="24"/>
+      <c r="Y54" s="24"/>
       <c r="Z54" s="32"/>
       <c r="AA54" s="32"/>
       <c r="AB54" s="32"/>
@@ -12990,19 +13088,19 @@
       <c r="AF54" s="32"/>
       <c r="AG54" s="32"/>
     </row>
-    <row r="55" spans="2:33" ht="42.75" customHeight="1">
+    <row r="55" spans="2:33" ht="58">
       <c r="B55" s="16">
         <v>94001</v>
       </c>
       <c r="C55" s="16">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D55" s="55"/>
       <c r="E55" s="55">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F55" s="22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G55" s="23" t="s">
         <v>90</v>
@@ -13021,7 +13119,9 @@
       <c r="S55" s="18"/>
       <c r="T55" s="18"/>
       <c r="U55" s="18"/>
-      <c r="V55" s="18"/>
+      <c r="V55" s="70" t="s">
+        <v>778</v>
+      </c>
       <c r="W55" s="19"/>
       <c r="X55" s="19"/>
       <c r="Y55" s="19"/>
@@ -13034,20 +13134,22 @@
       <c r="AF55" s="32"/>
       <c r="AG55" s="32"/>
     </row>
-    <row r="56" spans="2:33" ht="42.75" customHeight="1">
+    <row r="56" spans="2:33" ht="58">
       <c r="B56" s="16">
-        <v>13650</v>
+        <v>94001</v>
       </c>
       <c r="C56" s="16">
-        <v>8</v>
-      </c>
-      <c r="D56" s="27"/>
-      <c r="E56" s="16"/>
+        <v>56</v>
+      </c>
+      <c r="D56" s="55"/>
+      <c r="E56" s="55">
+        <v>10</v>
+      </c>
       <c r="F56" s="22" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="G56" s="23" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="H56" s="17"/>
       <c r="I56" s="18"/>
@@ -13058,47 +13160,37 @@
       <c r="N56" s="18"/>
       <c r="O56" s="18"/>
       <c r="P56" s="18"/>
-      <c r="Q56" s="28" t="s">
-        <v>628</v>
-      </c>
-      <c r="R56" s="28" t="s">
-        <v>629</v>
-      </c>
+      <c r="Q56" s="18"/>
+      <c r="R56" s="18"/>
       <c r="S56" s="18"/>
       <c r="T56" s="18"/>
-      <c r="U56" s="28"/>
-      <c r="V56" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="W56" s="19" t="s">
-        <v>456</v>
-      </c>
-      <c r="X56" s="19" t="s">
-        <v>469</v>
-      </c>
+      <c r="U56" s="18"/>
+      <c r="V56" s="70" t="s">
+        <v>779</v>
+      </c>
+      <c r="W56" s="19"/>
+      <c r="X56" s="19"/>
       <c r="Y56" s="19"/>
       <c r="Z56" s="32"/>
       <c r="AA56" s="32"/>
       <c r="AB56" s="32"/>
       <c r="AC56" s="32"/>
       <c r="AD56" s="32"/>
-      <c r="AE56" s="32" t="s">
-        <v>404</v>
-      </c>
+      <c r="AE56" s="32"/>
       <c r="AF56" s="32"/>
       <c r="AG56" s="32"/>
     </row>
-    <row r="57" spans="2:33" ht="42.75" customHeight="1">
+    <row r="57" spans="2:33" ht="58">
       <c r="B57" s="16">
-        <v>13468</v>
+        <v>13650</v>
       </c>
       <c r="C57" s="16">
-        <v>7</v>
-      </c>
-      <c r="D57" s="16"/>
+        <v>8</v>
+      </c>
+      <c r="D57" s="27"/>
       <c r="E57" s="16"/>
       <c r="F57" s="23" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="G57" s="23" t="s">
         <v>18</v>
@@ -13112,38 +13204,72 @@
       <c r="N57" s="18"/>
       <c r="O57" s="18"/>
       <c r="P57" s="18"/>
-      <c r="Q57" s="18"/>
-      <c r="R57" s="18"/>
-      <c r="S57" s="18"/>
-      <c r="T57" s="18"/>
-      <c r="U57" s="18"/>
-      <c r="V57" s="18"/>
-      <c r="W57" s="19"/>
-      <c r="X57" s="19"/>
-      <c r="Y57" s="19"/>
-      <c r="Z57" s="32"/>
-      <c r="AA57" s="32"/>
-      <c r="AB57" s="32"/>
-      <c r="AC57" s="32"/>
-      <c r="AD57" s="32"/>
-      <c r="AE57" s="32"/>
-      <c r="AF57" s="32"/>
-      <c r="AG57" s="32"/>
+      <c r="Q57" s="60" t="s">
+        <v>625</v>
+      </c>
+      <c r="R57" s="60" t="s">
+        <v>626</v>
+      </c>
+      <c r="S57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="T57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="U57" s="60" t="s">
+        <v>774</v>
+      </c>
+      <c r="V57" s="60" t="s">
+        <v>775</v>
+      </c>
+      <c r="W57" s="57" t="s">
+        <v>776</v>
+      </c>
+      <c r="X57" s="57" t="s">
+        <v>466</v>
+      </c>
+      <c r="Y57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="Z57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AA57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AB57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AC57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AD57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AE57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AF57" s="18" t="s">
+        <v>773</v>
+      </c>
+      <c r="AG57" s="18" t="s">
+        <v>773</v>
+      </c>
     </row>
     <row r="58" spans="2:33" ht="42.75" customHeight="1">
       <c r="B58" s="16">
-        <v>68081</v>
+        <v>13468</v>
       </c>
       <c r="C58" s="16">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="D58" s="16"/>
       <c r="E58" s="16"/>
       <c r="F58" s="23" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G58" s="23" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H58" s="17"/>
       <c r="I58" s="18"/>
@@ -13174,18 +13300,18 @@
     </row>
     <row r="59" spans="2:33" ht="42.75" customHeight="1">
       <c r="B59" s="16">
-        <v>13074</v>
+        <v>68081</v>
       </c>
       <c r="C59" s="16">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="D59" s="16"/>
       <c r="E59" s="16"/>
       <c r="F59" s="23" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G59" s="23" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H59" s="17"/>
       <c r="I59" s="18"/>
@@ -13202,7 +13328,7 @@
       <c r="T59" s="18"/>
       <c r="U59" s="18"/>
       <c r="V59" s="18"/>
-      <c r="W59" s="20"/>
+      <c r="W59" s="19"/>
       <c r="X59" s="19"/>
       <c r="Y59" s="19"/>
       <c r="Z59" s="32"/>
@@ -13216,15 +13342,15 @@
     </row>
     <row r="60" spans="2:33" ht="42.75" customHeight="1">
       <c r="B60" s="16">
-        <v>13160</v>
+        <v>13074</v>
       </c>
       <c r="C60" s="16">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="D60" s="16"/>
       <c r="E60" s="16"/>
       <c r="F60" s="22" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G60" s="23" t="s">
         <v>18</v>
@@ -13244,7 +13370,7 @@
       <c r="T60" s="18"/>
       <c r="U60" s="18"/>
       <c r="V60" s="18"/>
-      <c r="W60" s="19"/>
+      <c r="W60" s="20"/>
       <c r="X60" s="19"/>
       <c r="Y60" s="19"/>
       <c r="Z60" s="32"/>
@@ -13258,20 +13384,20 @@
     </row>
     <row r="61" spans="2:33" ht="48.75" customHeight="1">
       <c r="B61" s="16">
-        <v>13042</v>
+        <v>13160</v>
       </c>
       <c r="C61" s="16">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D61" s="16"/>
       <c r="E61" s="16"/>
-      <c r="F61" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="G61" s="21" t="s">
+      <c r="F61" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G61" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="H61" s="36"/>
+      <c r="H61" s="17"/>
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
       <c r="K61" s="18"/>
@@ -13300,15 +13426,15 @@
     </row>
     <row r="62" spans="2:33" ht="42.75" customHeight="1">
       <c r="B62" s="16">
-        <v>13430</v>
+        <v>13042</v>
       </c>
       <c r="C62" s="16">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="16"/>
       <c r="F62" s="25" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G62" s="21" t="s">
         <v>18</v>
@@ -13342,20 +13468,20 @@
     </row>
     <row r="63" spans="2:33" ht="42.75" customHeight="1">
       <c r="B63" s="16">
-        <v>23068</v>
+        <v>13430</v>
       </c>
       <c r="C63" s="16">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="D63" s="16"/>
       <c r="E63" s="16"/>
-      <c r="F63" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="G63" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="H63" s="17"/>
+      <c r="F63" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="G63" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="H63" s="36"/>
       <c r="I63" s="18"/>
       <c r="J63" s="18"/>
       <c r="K63" s="18"/>
@@ -13384,20 +13510,20 @@
     </row>
     <row r="64" spans="2:33" ht="47.25" customHeight="1">
       <c r="B64" s="16">
-        <v>13580</v>
+        <v>23068</v>
       </c>
       <c r="C64" s="16">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="D64" s="16"/>
       <c r="E64" s="16"/>
-      <c r="F64" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="G64" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="H64" s="36"/>
+      <c r="F64" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="G64" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="H64" s="17"/>
       <c r="I64" s="18"/>
       <c r="J64" s="18"/>
       <c r="K64" s="18"/>
@@ -13412,7 +13538,7 @@
       <c r="T64" s="18"/>
       <c r="U64" s="18"/>
       <c r="V64" s="18"/>
-      <c r="W64" s="20"/>
+      <c r="W64" s="19"/>
       <c r="X64" s="19"/>
       <c r="Y64" s="19"/>
       <c r="Z64" s="32"/>
@@ -13426,20 +13552,20 @@
     </row>
     <row r="65" spans="2:33" ht="46.5" customHeight="1">
       <c r="B65" s="16">
-        <v>68573</v>
+        <v>13580</v>
       </c>
       <c r="C65" s="16">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D65" s="16"/>
       <c r="E65" s="16"/>
-      <c r="F65" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G65" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="H65" s="17"/>
+      <c r="F65" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="G65" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="H65" s="36"/>
       <c r="I65" s="18"/>
       <c r="J65" s="18"/>
       <c r="K65" s="18"/>
@@ -13468,18 +13594,18 @@
     </row>
     <row r="66" spans="2:33" ht="48" customHeight="1">
       <c r="B66" s="23">
-        <v>13549</v>
+        <v>68573</v>
       </c>
       <c r="C66" s="22">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D66" s="22"/>
       <c r="E66" s="22"/>
       <c r="F66" s="22" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H66" s="23"/>
       <c r="I66" s="20"/>
@@ -13509,19 +13635,19 @@
       <c r="AG66" s="32"/>
     </row>
     <row r="67" spans="2:33" ht="47.25" customHeight="1">
-      <c r="B67" s="27">
-        <v>73770</v>
-      </c>
-      <c r="C67" s="27">
-        <v>61</v>
-      </c>
-      <c r="D67" s="27"/>
-      <c r="E67" s="27"/>
+      <c r="B67" s="16">
+        <v>13549</v>
+      </c>
+      <c r="C67" s="16">
+        <v>20</v>
+      </c>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
       <c r="F67" s="22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G67" s="23" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="H67" s="17"/>
       <c r="I67" s="18"/>
@@ -13538,7 +13664,7 @@
       <c r="T67" s="18"/>
       <c r="U67" s="18"/>
       <c r="V67" s="18"/>
-      <c r="W67" s="19"/>
+      <c r="W67" s="20"/>
       <c r="X67" s="19"/>
       <c r="Y67" s="19"/>
       <c r="Z67" s="32"/>
@@ -13552,18 +13678,18 @@
     </row>
     <row r="68" spans="2:33" ht="45" customHeight="1">
       <c r="B68" s="27">
-        <v>19780</v>
+        <v>73770</v>
       </c>
       <c r="C68" s="27">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D68" s="27"/>
       <c r="E68" s="27"/>
-      <c r="F68" s="21" t="s">
-        <v>68</v>
+      <c r="F68" s="23" t="s">
+        <v>61</v>
       </c>
       <c r="G68" s="23" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="H68" s="17"/>
       <c r="I68" s="18"/>
@@ -13593,19 +13719,19 @@
       <c r="AG68" s="32"/>
     </row>
     <row r="69" spans="2:33" ht="46.5" customHeight="1">
-      <c r="B69" s="16">
-        <v>50568</v>
-      </c>
-      <c r="C69" s="16">
-        <v>73</v>
-      </c>
-      <c r="D69" s="16"/>
-      <c r="E69" s="16"/>
-      <c r="F69" s="23" t="s">
-        <v>70</v>
+      <c r="B69" s="27">
+        <v>19780</v>
+      </c>
+      <c r="C69" s="27">
+        <v>79</v>
+      </c>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="21" t="s">
+        <v>68</v>
       </c>
       <c r="G69" s="23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H69" s="17"/>
       <c r="I69" s="18"/>
@@ -13636,18 +13762,18 @@
     </row>
     <row r="70" spans="2:33" ht="52.5" customHeight="1">
       <c r="B70" s="16">
-        <v>76126</v>
+        <v>50568</v>
       </c>
       <c r="C70" s="16">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="D70" s="16"/>
       <c r="E70" s="16"/>
       <c r="F70" s="23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G70" s="23" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H70" s="17"/>
       <c r="I70" s="18"/>
@@ -13678,18 +13804,18 @@
     </row>
     <row r="71" spans="2:33" ht="42.75" customHeight="1">
       <c r="B71" s="23">
-        <v>15047</v>
+        <v>76126</v>
       </c>
       <c r="C71" s="23">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D71" s="23"/>
       <c r="E71" s="23"/>
       <c r="F71" s="23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G71" s="23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H71" s="17"/>
       <c r="I71" s="18"/>
@@ -13720,18 +13846,18 @@
     </row>
     <row r="72" spans="2:33" ht="42.75" customHeight="1">
       <c r="B72" s="16">
-        <v>41885</v>
+        <v>15047</v>
       </c>
       <c r="C72" s="16">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D72" s="16"/>
       <c r="E72" s="16"/>
       <c r="F72" s="23" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="G72" s="23" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H72" s="17"/>
       <c r="I72" s="18"/>
@@ -13762,18 +13888,18 @@
     </row>
     <row r="73" spans="2:33" ht="40.5" customHeight="1">
       <c r="B73" s="16">
-        <v>15572</v>
+        <v>41885</v>
       </c>
       <c r="C73" s="16">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="D73" s="16"/>
       <c r="E73" s="16"/>
       <c r="F73" s="23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G73" s="23" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H73" s="17"/>
       <c r="I73" s="18"/>
@@ -13804,18 +13930,18 @@
     </row>
     <row r="74" spans="2:33" ht="45" customHeight="1">
       <c r="B74" s="16">
-        <v>81065</v>
+        <v>15572</v>
       </c>
       <c r="C74" s="16">
-        <v>86</v>
+        <v>46</v>
       </c>
       <c r="D74" s="16"/>
       <c r="E74" s="16"/>
       <c r="F74" s="23" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="G74" s="23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H74" s="17"/>
       <c r="I74" s="18"/>
@@ -13844,20 +13970,20 @@
       <c r="AF74" s="32"/>
       <c r="AG74" s="32"/>
     </row>
-    <row r="75" spans="2:33">
+    <row r="75" spans="2:33" ht="41.5" customHeight="1">
       <c r="B75" s="16">
-        <v>94343</v>
+        <v>81065</v>
       </c>
       <c r="C75" s="16">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="D75" s="16"/>
       <c r="E75" s="16"/>
       <c r="F75" s="17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G75" s="17" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="H75" s="17"/>
       <c r="I75" s="18"/>
@@ -13888,18 +14014,18 @@
     </row>
     <row r="76" spans="2:33" ht="48" customHeight="1">
       <c r="B76" s="16">
-        <v>81591</v>
+        <v>94343</v>
       </c>
       <c r="C76" s="16">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="D76" s="16"/>
       <c r="E76" s="16"/>
       <c r="F76" s="23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G76" s="23" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="H76" s="17"/>
       <c r="I76" s="18"/>
@@ -13930,18 +14056,18 @@
     </row>
     <row r="77" spans="2:33" ht="48" customHeight="1">
       <c r="B77" s="16">
-        <v>19318</v>
+        <v>81591</v>
       </c>
       <c r="C77" s="16">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="D77" s="16"/>
       <c r="E77" s="16"/>
       <c r="F77" s="23" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G77" s="23" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="H77" s="23"/>
       <c r="I77" s="20"/>
@@ -13958,7 +14084,7 @@
       <c r="T77" s="20"/>
       <c r="U77" s="20"/>
       <c r="V77" s="20"/>
-      <c r="W77" s="20"/>
+      <c r="W77" s="19"/>
       <c r="X77" s="19"/>
       <c r="Y77" s="19"/>
       <c r="Z77" s="32"/>
@@ -13972,18 +14098,18 @@
     </row>
     <row r="78" spans="2:33" ht="48" customHeight="1">
       <c r="B78" s="16">
-        <v>5659</v>
+        <v>19318</v>
       </c>
       <c r="C78" s="16">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="D78" s="16"/>
       <c r="E78" s="16"/>
       <c r="F78" s="23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G78" s="23" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="H78" s="23"/>
       <c r="I78" s="20"/>
@@ -13994,21 +14120,13 @@
       <c r="N78" s="20"/>
       <c r="O78" s="20"/>
       <c r="P78" s="20"/>
-      <c r="Q78" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="R78" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="S78" s="66" t="s">
-        <v>744</v>
-      </c>
-      <c r="T78" s="20" t="s">
-        <v>146</v>
-      </c>
+      <c r="Q78" s="20"/>
+      <c r="R78" s="20"/>
+      <c r="S78" s="20"/>
+      <c r="T78" s="20"/>
       <c r="U78" s="20"/>
       <c r="V78" s="20"/>
-      <c r="W78" s="19"/>
+      <c r="W78" s="20"/>
       <c r="X78" s="19"/>
       <c r="Y78" s="19"/>
       <c r="Z78" s="32"/>
@@ -14147,7 +14265,7 @@
       <c r="AG81" s="32"/>
     </row>
     <row r="82" spans="2:33" ht="36.75" customHeight="1">
-      <c r="B82" s="69">
+      <c r="B82" s="67">
         <v>68092</v>
       </c>
       <c r="C82" s="16">
@@ -14324,7 +14442,7 @@
       <c r="D86" s="16"/>
       <c r="E86" s="16"/>
       <c r="F86" s="23" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
       <c r="G86" s="23" t="s">
         <v>16</v>
@@ -14404,7 +14522,7 @@
       <c r="D88" s="23"/>
       <c r="E88" s="23"/>
       <c r="F88" s="23" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="G88" s="23" t="s">
         <v>44</v>
@@ -14444,7 +14562,7 @@
       <c r="D89" s="23"/>
       <c r="E89" s="23"/>
       <c r="F89" s="23" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
       <c r="G89" s="23" t="s">
         <v>67</v>
@@ -14484,7 +14602,7 @@
       <c r="D90" s="23"/>
       <c r="E90" s="23"/>
       <c r="F90" s="23" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
       <c r="G90" s="23" t="s">
         <v>18</v>
@@ -14524,7 +14642,7 @@
       <c r="D91" s="23"/>
       <c r="E91" s="23"/>
       <c r="F91" s="23" t="s">
-        <v>704</v>
+        <v>697</v>
       </c>
       <c r="G91" s="23" t="s">
         <v>47</v>
@@ -14564,7 +14682,7 @@
       <c r="D92" s="23"/>
       <c r="E92" s="23"/>
       <c r="F92" s="23" t="s">
-        <v>705</v>
+        <v>698</v>
       </c>
       <c r="G92" s="23" t="s">
         <v>44</v>
@@ -14604,7 +14722,7 @@
       <c r="D93" s="23"/>
       <c r="E93" s="23"/>
       <c r="F93" s="23" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
       <c r="G93" s="23" t="s">
         <v>16</v>
@@ -14644,7 +14762,7 @@
       <c r="D94" s="23"/>
       <c r="E94" s="23"/>
       <c r="F94" s="23" t="s">
-        <v>707</v>
+        <v>700</v>
       </c>
       <c r="G94" s="23" t="s">
         <v>18</v>
@@ -14684,7 +14802,7 @@
       <c r="D95" s="23"/>
       <c r="E95" s="23"/>
       <c r="F95" s="23" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
       <c r="G95" s="23" t="s">
         <v>41</v>
@@ -14724,7 +14842,7 @@
       <c r="D96" s="23"/>
       <c r="E96" s="23"/>
       <c r="F96" s="23" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="G96" s="23" t="s">
         <v>35</v>
@@ -14764,7 +14882,7 @@
       <c r="D97" s="23"/>
       <c r="E97" s="23"/>
       <c r="F97" s="23" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
       <c r="G97" s="23" t="s">
         <v>49</v>
@@ -14804,7 +14922,7 @@
       <c r="D98" s="23"/>
       <c r="E98" s="23"/>
       <c r="F98" s="23" t="s">
-        <v>711</v>
+        <v>704</v>
       </c>
       <c r="G98" s="23" t="s">
         <v>77</v>
@@ -15332,7 +15450,7 @@
     <hyperlink ref="Q48" r:id="rId491" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/00_Documentaci%C3%B3nInicio/01_Polizas/Cumplimiento?d=w7b292d32b56b4034975df199ccf45d34&amp;csf=1&amp;web=1&amp;e=cAseis" xr:uid="{218AD224-D6E2-4C1B-BB6B-63F1D304A212}"/>
     <hyperlink ref="R48" r:id="rId492" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/00_Documentaci%C3%B3nInicio/01_Polizas/RCE?d=w6a7bb9c9570545379b41f359d98c1854&amp;csf=1&amp;web=1&amp;e=i6Dqu6" xr:uid="{BE9572F3-BCF3-4961-B237-3FBA9DDCEFB5}"/>
     <hyperlink ref="S48" r:id="rId493" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/00_Documentaci%C3%B3nInicio/02_ActaInicio?d=w690dc6479434441991e1117c77b0a487&amp;csf=1&amp;web=1&amp;e=uRng9V" xr:uid="{92B1F437-5B0A-475D-8E85-35D5B34171A0}"/>
-    <hyperlink ref="AA48" r:id="rId494" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/03_SeguimientoCampo/01_BitacoraObra?d=wb16889c06ccb48b49171ec781b791b4e&amp;csf=1&amp;web=1&amp;e=CIwEMe" xr:uid="{1C38C854-313B-4640-B83E-5E47EE0FA487}"/>
+    <hyperlink ref="AA48" r:id="rId494" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86568%5FPuerto%20As%C3%ADs%5FBrisasHongKong%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F03%5FSeguimientoCampo%2F01%5FBitacoraObra&amp;p=true&amp;share=cgrAiWixy2y0SJFx7HgbeRtOEgUCaeL%5Fao%5FuEuq5gTqTldyymw" xr:uid="{1C38C854-313B-4640-B83E-5E47EE0FA487}"/>
     <hyperlink ref="U48" r:id="rId495" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/01_Socializaci%C3%B3nInicio/00_Cronograma?d=wbed4f6bebad54c61aaefe771861e9542&amp;csf=1&amp;web=1&amp;e=FbX05H" xr:uid="{8E14FCCA-D970-4E7D-9820-AC8372C8F32A}"/>
     <hyperlink ref="V48" r:id="rId496" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/01_Socializaci%C3%B3nInicio/01_Municipio/01_ReunionPreparacionInstalacion?d=wcdd779c07ee2465ea3658f98980d1d4f&amp;csf=1&amp;web=1&amp;e=N8JPzc" xr:uid="{4C9008FE-3FEB-4E56-8E65-A24329E83BE4}"/>
     <hyperlink ref="W48" r:id="rId497" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_BrisasHongKong (Putumayo)/04_Instalaci%C3%B3n/01_Socializaci%C3%B3nInicio/01_Municipio/02_ReunionInicioActividades?d=w199e6e225b5e4541bfda7e99813e7be8&amp;csf=1&amp;web=1&amp;e=9KKi2U" xr:uid="{675EB14F-1457-401A-8C7B-FAB6E49F5FB1}"/>
@@ -15349,32 +15467,53 @@
     <hyperlink ref="W49" r:id="rId508" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/01_Socializaci%C3%B3nInicio/01_Municipio/02_ReunionInicioActividades?d=w26359ba185a34aed8c9ea6a7004c16f7&amp;csf=1&amp;web=1&amp;e=3m2kT6" xr:uid="{A88CDF7F-EC0B-4F0E-A1F0-9FE00C04217D}"/>
     <hyperlink ref="X49" r:id="rId509" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/01_Socializaci%C3%B3nInicio/02_Comunidad?d=w9acbdf63c19d4f04979c86e75b9badb4&amp;csf=1&amp;web=1&amp;e=jJpOio" xr:uid="{C833A1B7-2BD5-4737-AD80-430AF449D217}"/>
     <hyperlink ref="AA49" r:id="rId510" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/03_SeguimientoCampo/01_BitacoraObra?d=w694424346d8742239409533437c3e12f&amp;csf=1&amp;web=1&amp;e=lRMkxR" xr:uid="{F22E6762-3E45-4CEA-96AC-B78802730FBA}"/>
-    <hyperlink ref="AD49" r:id="rId511" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/03_SeguimientoCampo/02_SeguimientoArmado?d=wf600f7c7804f46408ecce4af8d16cc0a&amp;csf=1&amp;web=1&amp;e=bvYjtL" xr:uid="{FDBDC138-D6D4-430D-BD14-866BC93423DE}"/>
-    <hyperlink ref="AE49" r:id="rId512" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/04_Capacitaci%C3%B3n?d=wd1ac432366874abf9ff2806e55ce3888&amp;csf=1&amp;web=1&amp;e=hwmU6c" xr:uid="{5F3B6958-1B21-495B-8078-DB8A56194A20}"/>
-    <hyperlink ref="AF49" r:id="rId513" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/05_Entrega?d=w628871493fb54059bb133467d20bff30&amp;csf=1&amp;web=1&amp;e=lrXWd7" xr:uid="{70BB30F1-EBF6-4BE5-8D38-F15A804519B7}"/>
-    <hyperlink ref="AG49" r:id="rId514" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/05_Entrega?d=w628871493fb54059bb133467d20bff30&amp;csf=1&amp;web=1&amp;e=lrXWd7" xr:uid="{7C84CF5F-0FE8-4C9E-9DE4-F3E9E7F2BA07}"/>
-    <hyperlink ref="AC44" r:id="rId515" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/73483_Natagaima_R_Velu(Tolima)/04_Instalaci%C3%B3n/03_SeguimientoCampo/03_CertificacionesCalidadMateriales/01_Anclajes/02_Interventoria?d=w4033375332ce4826bf4b1e5da0a9a79d&amp;csf=1&amp;web=1&amp;e=ODkbXw" xr:uid="{C3B39160-0095-4263-BFE2-BE3D31758D80}"/>
-    <hyperlink ref="AC45" r:id="rId516" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/73563_Prado (Tolima)/04_Instalaci%C3%B3n/03_SeguimientoCampo/03_CertificacionesCalidadMateriales/01_Anclajes/02_Interventoria?d=w3347d05ef6b44c27a3d077bca303b7ed&amp;csf=1&amp;web=1&amp;e=gLRGG2" xr:uid="{91FDC411-A167-4A2F-9792-E62D7CC9E94A}"/>
-    <hyperlink ref="AC46" r:id="rId517" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/23417_Lorica (C%C3%B3rdoba)/04_Instalaci%C3%B3n/03_SeguimientoCampo/03_CertificacionesCalidadMateriales/01_Anclajes/02_Interventoria?d=wba8b7031fa0a4bd194ff257fefcab016&amp;csf=1&amp;web=1&amp;e=Bfx2Zy" xr:uid="{62524E6A-8C87-4D60-B2B8-AD351DB4C5BD}"/>
-    <hyperlink ref="Q50" r:id="rId518" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FCumplimiento&amp;p=true&amp;share=cgqo6q1rWuB2TqRVkivno11%2DEgUCEIbahvKs%2DffzTYxReJS%2DgQ" xr:uid="{4E26F620-756D-43FE-ADF2-84E257494386}"/>
-    <hyperlink ref="R50" r:id="rId519" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FRCE&amp;p=true&amp;share=cgryvCjj6S0wS4nEucHv%2D%2DjxEgUCSwf%2DbPjy6auFlyVcWg4OWg" xr:uid="{64FDC9D5-69DD-43F7-81B1-FDBEEE5A25CB}"/>
-    <hyperlink ref="S50" r:id="rId520" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F02%5FActaInicio&amp;p=true&amp;share=cgpClkpz4PIYSLC3sDebXKqJEgUCoWywQV1ClWB%2Dtxdy4bXrrA" xr:uid="{AA5403A9-0266-4CE3-9F1B-6FD77605A5AD}"/>
-    <hyperlink ref="U50" r:id="rId521" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F02%5FActaInicio&amp;p=true&amp;share=cgpClkpz4PIYSLC3sDebXKqJEgUCoWywQV1ClWB%2Dtxdy4bXrrA" xr:uid="{2F268A2A-31E9-4BF3-B2B5-01E8FC0C95B7}"/>
-    <hyperlink ref="V50" r:id="rId522" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparacionInstalacion&amp;p=true&amp;share=cgp4z1nO%2DL5JR7%2DoW0gJ6tTzEgUCP65a4mXIP7rmwIK0V60B8A" xr:uid="{CE540CB6-7973-47B5-8FB9-3BBF7FDE0110}"/>
-    <hyperlink ref="Q52" r:id="rId523" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FCumplimiento&amp;p=true&amp;share=cgoGjCCdqXInQYvRAYIGTa1PEgUC8gHCDvWyM6fkg4IIe%2Dso2A" xr:uid="{9E4D1120-6474-40E2-85CB-6E5ED76AE713}"/>
-    <hyperlink ref="R52" r:id="rId524" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FRCE&amp;p=true&amp;share=cgrBUNWwoV5kRJZJGbJmWofjEgUCOH1PA5498z3UkloRBU9Ipw" xr:uid="{87320C00-3E75-46F5-9128-0646168B7E51}"/>
-    <hyperlink ref="S52" r:id="rId525" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F02%5FActaInicio&amp;p=true&amp;share=cgrO4cXG8cdjRZWEicUd0ByXEgUCwwdzsoVqhpIIt%2DEvWYVp4Q" xr:uid="{A080E757-11DF-4CCE-A76F-4442905F5F30}"/>
-    <hyperlink ref="U52" r:id="rId526" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F00%5FCronograma&amp;p=true&amp;share=cgq0%2DL6CpDN7R4Mgwm%5FO4kYzEgUC1bIsHo4Lmka2rIJPgdcubg" xr:uid="{4E1CF9F2-8940-40E1-84C8-C038860ABAFF}"/>
-    <hyperlink ref="S51" r:id="rId527" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio&amp;p=true&amp;share=cgpd%2D7yA2CFlR5L82YPMa%5FWuEgUCZ6qINBaoOc%5FcCv8XnJKt8w" xr:uid="{DAB910C4-FFEF-4F6C-A4E3-53C9585DDADE}"/>
-    <hyperlink ref="U51" r:id="rId528" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F00%5FCronograma&amp;p=true&amp;share=cgruNkHPLKjQTbjz2LfXa5AcEgUC8usjHzzBpwqByHKSBWehCg" xr:uid="{DFB6EDDB-63B0-4F0D-8D7B-43D661B416D6}"/>
-    <hyperlink ref="V51" r:id="rId529" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparacionInstalacion&amp;p=true&amp;share=cgozv78WgR%5FbT4OD6q7j7aSkEgUCoPx1rwlqS4ei7N58sQS8Qg" xr:uid="{9597AD7C-227B-4C00-9D60-95B81B5C2130}"/>
-    <hyperlink ref="W27" r:id="rId530" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F17495%5FNorcasia%20%28Caldas%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgo8REuqZEzKQZPwcLGy1Q5YEgUCiIBLt8ATAw2h7MExz2oaXQ" xr:uid="{6482661C-C640-4D77-9AC7-528559496004}"/>
+    <hyperlink ref="AE49" r:id="rId511" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/04_Capacitaci%C3%B3n?d=wd1ac432366874abf9ff2806e55ce3888&amp;csf=1&amp;web=1&amp;e=hwmU6c" xr:uid="{5F3B6958-1B21-495B-8078-DB8A56194A20}"/>
+    <hyperlink ref="AF49" r:id="rId512" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/05_Entrega?d=w628871493fb54059bb133467d20bff30&amp;csf=1&amp;web=1&amp;e=lrXWd7" xr:uid="{70BB30F1-EBF6-4BE5-8D38-F15A804519B7}"/>
+    <hyperlink ref="AG49" r:id="rId513" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/86568_Puerto As%C3%ADs_PuertoVega (Putumayo)/04_Instalaci%C3%B3n/05_Entrega?d=w628871493fb54059bb133467d20bff30&amp;csf=1&amp;web=1&amp;e=lrXWd7" xr:uid="{7C84CF5F-0FE8-4C9E-9DE4-F3E9E7F2BA07}"/>
+    <hyperlink ref="AC44" r:id="rId514" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/73483_Natagaima_R_Velu(Tolima)/04_Instalaci%C3%B3n/03_SeguimientoCampo/03_CertificacionesCalidadMateriales/01_Anclajes/02_Interventoria?d=w4033375332ce4826bf4b1e5da0a9a79d&amp;csf=1&amp;web=1&amp;e=ODkbXw" xr:uid="{C3B39160-0095-4263-BFE2-BE3D31758D80}"/>
+    <hyperlink ref="AC45" r:id="rId515" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/73563_Prado (Tolima)/04_Instalaci%C3%B3n/03_SeguimientoCampo/03_CertificacionesCalidadMateriales/01_Anclajes/02_Interventoria?d=w3347d05ef6b44c27a3d077bca303b7ed&amp;csf=1&amp;web=1&amp;e=gLRGG2" xr:uid="{91FDC411-A167-4A2F-9792-E62D7CC9E94A}"/>
+    <hyperlink ref="AC46" r:id="rId516" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Documentos T%C3%A9cnicos/Documentos por sitio/23417_Lorica (C%C3%B3rdoba)/04_Instalaci%C3%B3n/03_SeguimientoCampo/03_CertificacionesCalidadMateriales/01_Anclajes/02_Interventoria?d=wba8b7031fa0a4bd194ff257fefcab016&amp;csf=1&amp;web=1&amp;e=Bfx2Zy" xr:uid="{62524E6A-8C87-4D60-B2B8-AD351DB4C5BD}"/>
+    <hyperlink ref="Q50" r:id="rId517" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FCumplimiento&amp;p=true&amp;share=cgqo6q1rWuB2TqRVkivno11%2DEgUCEIbahvKs%2DffzTYxReJS%2DgQ" xr:uid="{4E26F620-756D-43FE-ADF2-84E257494386}"/>
+    <hyperlink ref="R50" r:id="rId518" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FRCE&amp;p=true&amp;share=cgryvCjj6S0wS4nEucHv%2D%2DjxEgUCSwf%2DbPjy6auFlyVcWg4OWg" xr:uid="{64FDC9D5-69DD-43F7-81B1-FDBEEE5A25CB}"/>
+    <hyperlink ref="S50" r:id="rId519" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F02%5FActaInicio&amp;p=true&amp;share=cgpClkpz4PIYSLC3sDebXKqJEgUCoWywQV1ClWB%2Dtxdy4bXrrA" xr:uid="{AA5403A9-0266-4CE3-9F1B-6FD77605A5AD}"/>
+    <hyperlink ref="U50" r:id="rId520" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F02%5FActaInicio&amp;p=true&amp;share=cgpClkpz4PIYSLC3sDebXKqJEgUCoWywQV1ClWB%2Dtxdy4bXrrA" xr:uid="{2F268A2A-31E9-4BF3-B2B5-01E8FC0C95B7}"/>
+    <hyperlink ref="V50" r:id="rId521" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparacionInstalacion&amp;p=true&amp;share=cgp4z1nO%2DL5JR7%2DoW0gJ6tTzEgUCP65a4mXIP7rmwIK0V60B8A" xr:uid="{CE540CB6-7973-47B5-8FB9-3BBF7FDE0110}"/>
+    <hyperlink ref="Q52" r:id="rId522" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FCumplimiento&amp;p=true&amp;share=cgoGjCCdqXInQYvRAYIGTa1PEgUC8gHCDvWyM6fkg4IIe%2Dso2A" xr:uid="{9E4D1120-6474-40E2-85CB-6E5ED76AE713}"/>
+    <hyperlink ref="R52" r:id="rId523" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FPolizas%2FRCE&amp;p=true&amp;share=cgrBUNWwoV5kRJZJGbJmWofjEgUCOH1PA5498z3UkloRBU9Ipw" xr:uid="{87320C00-3E75-46F5-9128-0646168B7E51}"/>
+    <hyperlink ref="U52" r:id="rId524" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F00%5FCronograma&amp;p=true&amp;share=cgq0%2DL6CpDN7R4Mgwm%5FO4kYzEgUC1bIsHo4Lmka2rIJPgdcubg" xr:uid="{4E1CF9F2-8940-40E1-84C8-C038860ABAFF}"/>
+    <hyperlink ref="S51" r:id="rId525" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio&amp;p=true&amp;share=cgpd%2D7yA2CFlR5L82YPMa%5FWuEgUCZ6qINBaoOc%5FcCv8XnJKt8w" xr:uid="{DAB910C4-FFEF-4F6C-A4E3-53C9585DDADE}"/>
+    <hyperlink ref="U51" r:id="rId526" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F00%5FCronograma&amp;p=true&amp;share=cgruNkHPLKjQTbjz2LfXa5AcEgUC8usjHzzBpwqByHKSBWehCg" xr:uid="{DFB6EDDB-63B0-4F0D-8D7B-43D661B416D6}"/>
+    <hyperlink ref="V51" r:id="rId527" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparacionInstalacion&amp;p=true&amp;share=cgozv78WgR%5FbT4OD6q7j7aSkEgUCoPx1rwlqS4ei7N58sQS8Qg" xr:uid="{9597AD7C-227B-4C00-9D60-95B81B5C2130}"/>
+    <hyperlink ref="W27" r:id="rId528" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F17495%5FNorcasia%20%28Caldas%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgo8REuqZEzKQZPwcLGy1Q5YEgUCiIBLt8ATAw2h7MExz2oaXQ" xr:uid="{6482661C-C640-4D77-9AC7-528559496004}"/>
+    <hyperlink ref="U53" r:id="rId529" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5659%5FSan%20Juan%20de%20Urab%C3%A1%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F00%5FCronograma&amp;p=true&amp;share=cgr3rr3jctsMQ5whgDFQFTJ%5FEgUCZOqXKcpFnbE2zPgmerPNfA" xr:uid="{43F75065-8A88-405B-9D3E-59790D4BB3EA}"/>
+    <hyperlink ref="W50" r:id="rId530" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgpNUz8wqybtTKIeQw4FSCLhEgUCbZ3k6iWm6hAVsJcrjNoogA" xr:uid="{15281189-74FA-45DA-89DC-F5963B48D53A}"/>
+    <hyperlink ref="X50" r:id="rId531" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F02%5FComunidad&amp;p=true&amp;share=cgruSkHGXmOvQJXDG75qlfBCEgUCcIRdoULqPDfLnMOALv0KYw" xr:uid="{0F63EE5E-75E3-44F0-BD96-B670D6BBF10E}"/>
+    <hyperlink ref="AA50" r:id="rId532" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F03%5FSeguimientoCampo%2F01%5FBitacoraObra&amp;p=true&amp;share=cgpFEBjdINIkQaYckatJRByXEgUCyLHxInYm1%2DW6KMBBNJDiUw" xr:uid="{F7B28774-D182-4C92-BC69-412F1F85B6A4}"/>
+    <hyperlink ref="AE50" r:id="rId533" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F04%5FCapacitaci%C3%B3n&amp;p=true&amp;share=cgrIPzRS9gBCSoNaCZF4UKxfEgUC8U9lu47QzShFdCg%5FuCXZow" xr:uid="{1D4F80FB-3BC4-417A-A85E-EF2032BA1D9F}"/>
+    <hyperlink ref="AF50" r:id="rId534" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F86573%5FPuerto%20Legu%C3%ADzamo%20%28Putumayo%29%2F04%5FInstalaci%C3%B3n%2F05%5FEntrega&amp;p=true&amp;share=cgqdLX4yWDRJS4Td8SfnLzD3EgUCPsiGt9%5F7OLu0JiipFias1g" xr:uid="{4D7B24AC-ED0A-40DF-A704-FD333A83A15F}"/>
+    <hyperlink ref="Y51" r:id="rId535" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F02%5FAutorizacionesPermisos%2F01%5FEspacioP%C3%BAblico&amp;p=true&amp;share=cgpPDLD3ZWd8R5xWSNM36hfLEgUC4fH2XadV8Xb6fZFhXjWruA" xr:uid="{D0DB07EE-75DB-41E3-83D1-2CD30D06D2C7}"/>
+    <hyperlink ref="V52" r:id="rId536" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparacionInstalacion&amp;p=true&amp;share=cgraE%5Fxi7h5ET7A9W989tAgnEgUCaBIEyvm3kRjU9z7B%5FsD8cQ" xr:uid="{B44ADC5A-5BF2-4380-9A7B-BC8986043522}"/>
+    <hyperlink ref="W52" r:id="rId537" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgrKp7UbhLQURocRWP%2DE9DyrEgUCgGrt6GUTR2hlop8R9nuUdw" xr:uid="{E5C2D81D-030B-41DA-B334-E97E8CF0C9F9}"/>
+    <hyperlink ref="X52" r:id="rId538" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5895%5FZaragoza%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F02%5FComunidad&amp;p=true&amp;share=cgqQy0%2D8AqL4RL%2DhWwEo76NHEgUCXp1%2DyYzkC8yOye47smbnFQ" xr:uid="{95D60D29-3F27-49C9-9AF5-3009F7B34FF9}"/>
+    <hyperlink ref="W51" r:id="rId539" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgqbt9cCcXhVTo0S75euiOYlEgUCLbUZH%5FyGy48Ryj6OwoDiNA" xr:uid="{B6681603-5282-47E7-BD0A-3D884A607272}"/>
+    <hyperlink ref="X51" r:id="rId540" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F02%5FComunidad&amp;p=true&amp;share=cgpZXOF4QutxT4GKjrz5m0VPEgUCgxk%2Ds6Q5JAOY8sgZQK%5Fvrw" xr:uid="{4FDEF4EA-C6F1-4D04-96E3-B21A4D573799}"/>
+    <hyperlink ref="AF51" r:id="rId541" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F44090%5FDibulla%20%28La%20Guajira%29%2F04%5FInstalaci%C3%B3n%2F05%5FEntrega&amp;p=true&amp;share=cgqqpgyUChEPRI%5FwdSVn4M1REgUC9kuuniR%2DQVsZTJABXMiYFQ" xr:uid="{3316D0F5-E18A-437D-BB13-3988319013BD}"/>
+    <hyperlink ref="S53" r:id="rId542" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5659%5FSan%20Juan%20de%20Urab%C3%A1%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio&amp;p=true&amp;share=cgoo%2D3NAqNnpS5hpVqoRzK8AEgUCozUBOc23iy88egXwjMZV%2DA" xr:uid="{CDE1C90F-C104-492B-9AC0-6FE646204719}"/>
+    <hyperlink ref="V53" r:id="rId543" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5659%5FSan%20Juan%20de%20Urab%C3%A1%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparacionInstalacion&amp;p=true&amp;share=cgoUGRxzT0TzRb9ZLf6ERnHcEgUCBUn2GXWIIRjPjfcZhTUjhg" xr:uid="{D4D7ECDB-C83E-44F6-8E08-639FCBBCCACC}"/>
+    <hyperlink ref="W53" r:id="rId544" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5659%5FSan%20Juan%20de%20Urab%C3%A1%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgrQzVJgK8iKSbJJKJ%2DXk5YBEgUC%5FK%2DUCS%5F0t9TtxvNB4jDT1w" xr:uid="{71897C99-EFA7-4D6A-8BF3-386A0ED06C5D}"/>
+    <hyperlink ref="X53" r:id="rId545" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F5659%5FSan%20Juan%20de%20Urab%C3%A1%20%28Antioquia%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F02%5FComunidad&amp;p=true&amp;share=cgoXwWDnRnKnR6G8YTAlxK59EgUCNdOJ64DdSjVe%2DSPd%2DLi%2Dqg" xr:uid="{418E3976-F6CD-4199-8CE7-16805913303D}"/>
+    <hyperlink ref="Q57" r:id="rId546" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F13650%5FSan%20Fernando%20%28Bol%C3%ADvar%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FP%C3%B3lizas%2FCumplimiento&amp;p=true&amp;share=cgp2fXt8FXSYSZTf0dHp6xPnEgUCO%5F%2DhQnzlcionHnnM%2DlZueg" xr:uid="{8FD609A0-CFB0-4758-8F26-BBCA4B947069}"/>
+    <hyperlink ref="R57" r:id="rId547" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F13650%5FSan%20Fernando%20%28Bol%C3%ADvar%29%2F04%5FInstalaci%C3%B3n%2F00%5FDocumentaci%C3%B3nInicio%2F01%5FP%C3%B3lizas%2FRCE&amp;p=true&amp;share=cgo%5F6hWexO2HQrnqkWezbsJkEgUCrP88PMudIegfFNxs%5FmOeVw" xr:uid="{268160EC-90AC-4F03-A1B4-80431E0D330B}"/>
+    <hyperlink ref="U57" r:id="rId548" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F13650%5FSan%20Fernando%20%28Bol%C3%ADvar%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F00%5FCronograma&amp;p=true&amp;share=cgofNlZSLzL7SpAMVsg8cmJgEgUCe8%2DSX4E8Whz66OloZgHH0A" xr:uid="{D4E2A688-F17F-43BC-9C16-1ADDDCE6E917}"/>
+    <hyperlink ref="V57" r:id="rId549" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F13650%5FSan%20Fernando%20%28Bol%C3%ADvar%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F01%5FReunionPreparaci%C3%B3nInstalaci%C3%B3n&amp;p=true&amp;share=cgq4OZtsot90RLS0ySM9N6VqEgUCEy7X7v3JstMHE9DQD6SP7w" xr:uid="{FF9743EB-8079-4B48-B306-82E7133A1F51}"/>
+    <hyperlink ref="W57" r:id="rId550" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F13650%5FSan%20Fernando%20%28Bol%C3%ADvar%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F01%5FMunicipio%2F02%5FReunionInicioActividades&amp;p=true&amp;share=cgrmgCJXo72eRofGzCqSslvOEgUC3T%2DDsggxaCF0NCe6C4BtkA" xr:uid="{05D7CC14-82D8-479D-B27B-B0917810876D}"/>
+    <hyperlink ref="X57" r:id="rId551" display="https://mailuis.sharepoint.com/:f:/r/sites/INTERVENTORIA/Documentos compartidos/Forms/AllItems.aspx?id=%2Fsites%2FINTERVENTORIA%2FDocumentos%20compartidos%2FDocumentos%20T%C3%A9cnicos%2FDocumentos%20por%20sitio%2F13650%5FSan%20Fernando%20%28Bol%C3%ADvar%29%2F04%5FInstalaci%C3%B3n%2F01%5FSocializaci%C3%B3nInicio%2F02%5FComunidad&amp;p=true&amp;share=cgrVGZS8SA5dQaTyfiwbgYH9EgUCK%2Dkbs6u2zqSFYUrUUdt6Sg" xr:uid="{D8119C67-1AE4-42B6-8AA6-281A8E5CF723}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId531"/>
-  <drawing r:id="rId532"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId552"/>
+  <drawing r:id="rId553"/>
   <tableParts count="1">
-    <tablePart r:id="rId533"/>
+    <tablePart r:id="rId554"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>